<commit_message>
corregido lo de las marcas y patrones, y la carga sin fecha de examen
corregido lo de las marcas y patrones, y la carga sin fecha de examen
</commit_message>
<xml_diff>
--- a/evaluaciones-frontend/src/assets/formato_banco_preguntas_asig_EF_1P.xlsx
+++ b/evaluaciones-frontend/src/assets/formato_banco_preguntas_asig_EF_1P.xlsx
@@ -25,6 +25,7 @@
     <x:definedName name="TIPOS_OPCION_G">VALIDACIONES!$Q$1:$Q$5</x:definedName>
     <x:definedName name="TIPOS_OPCION_H">VALIDACIONES!$R$1:$R$3</x:definedName>
   </x:definedNames>
+  <x:calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </x:workbook>
 </file>
 
@@ -2632,7 +2633,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L2" s="343" t="str">
-        <x:f>IF(TRIM($A2)="","",IF(COUNTIF($Q2:$AJ2,"?*")=0,"OK","Falta revisar: "&amp;$Q2&amp;$R2&amp;$S2&amp;$T2&amp;$U2&amp;$V2&amp;$W2&amp;$X2&amp;$Y2&amp;$Z2&amp;$AA2&amp;$AB2&amp;$AC2&amp;$AD2&amp;$AE2&amp;$AF2&amp;$AG2&amp;$AH2&amp;$AI2&amp;$AJ2))</x:f>
+        <x:f>IF(TRIM($A2)="","",IF(OR($A2="Selección de la mejor respuesta",$A2="SELECCION_MEJOR_RESPUESTA",$A2="Subítem de caso o problema",$A2="SUBITEM_CASO"),IF(TRIM($C2)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D2:$H2&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I2)&lt;&gt;"",OR(LEFT(TRIM($I2),1)="A",LEFT(TRIM($I2),1)="B",LEFT(TRIM($I2),1)="C",LEFT(TRIM($I2),1)="D",LEFT(TRIM($I2),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A2)="","",IF(COUNTIF($Q2:$AJ2,"?*")=0,"OK","Falta revisar: "&amp;$Q2&amp;$R2&amp;$S2&amp;$T2&amp;$U2&amp;$V2&amp;$W2&amp;$X2&amp;$Y2&amp;$Z2&amp;$AA2&amp;$AB2&amp;$AC2&amp;$AD2&amp;$AE2&amp;$AF2&amp;$AG2&amp;$AH2&amp;$AI2&amp;$AJ2))))</x:f>
       </x:c>
       <x:c r="M2" s="341"/>
       <x:c r="N2"/>
@@ -2688,7 +2689,7 @@
         <x:f>IF(AND($A2="Verdadero o Falso Complejas",TRIM($I2)&lt;&gt;"",NOT(OR(LEFT(TRIM($I2),1)="A",LEFT(TRIM($I2),1)="B",LEFT(TRIM($I2),1)="C",LEFT(TRIM($I2),1)="D",LEFT(TRIM($I2),1)="E"))),IF(COUNTIF($Q2:$AE2,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG2" t="str">
-        <x:f>IF(AND(OR($A2="Selección de la mejor respuesta",$A2="Subítem de caso o problema"),COUNTIF($D2:$H2,"?*")&lt;5),IF(COUNTIF($Q2:$AF2,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A2="Selección de la mejor respuesta",$A2="Subítem de caso o problema"),COUNTA($D2:$H2)&lt;5),IF(COUNTIF($Q2:$AF2,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH2" t="str">
         <x:f>IF(AND(OR($A2="Selección de la mejor respuesta",$A2="Subítem de caso o problema"),TRIM($I2)&lt;&gt;"",NOT(OR(LEFT(TRIM($I2),1)="A",LEFT(TRIM($I2),1)="B",LEFT(TRIM($I2),1)="C",LEFT(TRIM($I2),1)="D",LEFT(TRIM($I2),1)="E"))),IF(COUNTIF($Q2:$AG2,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -2749,7 +2750,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L3" s="343" t="str">
-        <x:f>IF(TRIM($A3)="","",IF(COUNTIF($Q3:$AJ3,"?*")=0,"OK","Falta revisar: "&amp;$Q3&amp;$R3&amp;$S3&amp;$T3&amp;$U3&amp;$V3&amp;$W3&amp;$X3&amp;$Y3&amp;$Z3&amp;$AA3&amp;$AB3&amp;$AC3&amp;$AD3&amp;$AE3&amp;$AF3&amp;$AG3&amp;$AH3&amp;$AI3&amp;$AJ3))</x:f>
+        <x:f>IF(TRIM($A3)="","",IF(OR($A3="Selección de la mejor respuesta",$A3="SELECCION_MEJOR_RESPUESTA",$A3="Subítem de caso o problema",$A3="SUBITEM_CASO"),IF(TRIM($C3)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D3:$H3&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I3)&lt;&gt;"",OR(LEFT(TRIM($I3),1)="A",LEFT(TRIM($I3),1)="B",LEFT(TRIM($I3),1)="C",LEFT(TRIM($I3),1)="D",LEFT(TRIM($I3),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A3)="","",IF(COUNTIF($Q3:$AJ3,"?*")=0,"OK","Falta revisar: "&amp;$Q3&amp;$R3&amp;$S3&amp;$T3&amp;$U3&amp;$V3&amp;$W3&amp;$X3&amp;$Y3&amp;$Z3&amp;$AA3&amp;$AB3&amp;$AC3&amp;$AD3&amp;$AE3&amp;$AF3&amp;$AG3&amp;$AH3&amp;$AI3&amp;$AJ3))))</x:f>
       </x:c>
       <x:c r="M3" s="341"/>
       <x:c r="N3"/>
@@ -2805,7 +2806,7 @@
         <x:f>IF(AND($A3="Verdadero o Falso Complejas",TRIM($I3)&lt;&gt;"",NOT(OR(LEFT(TRIM($I3),1)="A",LEFT(TRIM($I3),1)="B",LEFT(TRIM($I3),1)="C",LEFT(TRIM($I3),1)="D",LEFT(TRIM($I3),1)="E"))),IF(COUNTIF($Q3:$AE3,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG3" t="str">
-        <x:f>IF(AND(OR($A3="Selección de la mejor respuesta",$A3="Subítem de caso o problema"),COUNTIF($D3:$H3,"?*")&lt;5),IF(COUNTIF($Q3:$AF3,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A3="Selección de la mejor respuesta",$A3="Subítem de caso o problema"),COUNTA($D3:$H3)&lt;5),IF(COUNTIF($Q3:$AF3,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH3" t="str">
         <x:f>IF(AND(OR($A3="Selección de la mejor respuesta",$A3="Subítem de caso o problema"),TRIM($I3)&lt;&gt;"",NOT(OR(LEFT(TRIM($I3),1)="A",LEFT(TRIM($I3),1)="B",LEFT(TRIM($I3),1)="C",LEFT(TRIM($I3),1)="D",LEFT(TRIM($I3),1)="E"))),IF(COUNTIF($Q3:$AG3,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -2866,7 +2867,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L4" s="343" t="str">
-        <x:f>IF(TRIM($A4)="","",IF(COUNTIF($Q4:$AJ4,"?*")=0,"OK","Falta revisar: "&amp;$Q4&amp;$R4&amp;$S4&amp;$T4&amp;$U4&amp;$V4&amp;$W4&amp;$X4&amp;$Y4&amp;$Z4&amp;$AA4&amp;$AB4&amp;$AC4&amp;$AD4&amp;$AE4&amp;$AF4&amp;$AG4&amp;$AH4&amp;$AI4&amp;$AJ4))</x:f>
+        <x:f>IF(TRIM($A4)="","",IF(OR($A4="Selección de la mejor respuesta",$A4="SELECCION_MEJOR_RESPUESTA",$A4="Subítem de caso o problema",$A4="SUBITEM_CASO"),IF(TRIM($C4)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D4:$H4&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I4)&lt;&gt;"",OR(LEFT(TRIM($I4),1)="A",LEFT(TRIM($I4),1)="B",LEFT(TRIM($I4),1)="C",LEFT(TRIM($I4),1)="D",LEFT(TRIM($I4),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A4)="","",IF(COUNTIF($Q4:$AJ4,"?*")=0,"OK","Falta revisar: "&amp;$Q4&amp;$R4&amp;$S4&amp;$T4&amp;$U4&amp;$V4&amp;$W4&amp;$X4&amp;$Y4&amp;$Z4&amp;$AA4&amp;$AB4&amp;$AC4&amp;$AD4&amp;$AE4&amp;$AF4&amp;$AG4&amp;$AH4&amp;$AI4&amp;$AJ4))))</x:f>
       </x:c>
       <x:c r="M4" s="341"/>
       <x:c r="N4"/>
@@ -2922,7 +2923,7 @@
         <x:f>IF(AND($A4="Verdadero o Falso Complejas",TRIM($I4)&lt;&gt;"",NOT(OR(LEFT(TRIM($I4),1)="A",LEFT(TRIM($I4),1)="B",LEFT(TRIM($I4),1)="C",LEFT(TRIM($I4),1)="D",LEFT(TRIM($I4),1)="E"))),IF(COUNTIF($Q4:$AE4,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG4" t="str">
-        <x:f>IF(AND(OR($A4="Selección de la mejor respuesta",$A4="Subítem de caso o problema"),COUNTIF($D4:$H4,"?*")&lt;5),IF(COUNTIF($Q4:$AF4,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A4="Selección de la mejor respuesta",$A4="Subítem de caso o problema"),COUNTA($D4:$H4)&lt;5),IF(COUNTIF($Q4:$AF4,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH4" t="str">
         <x:f>IF(AND(OR($A4="Selección de la mejor respuesta",$A4="Subítem de caso o problema"),TRIM($I4)&lt;&gt;"",NOT(OR(LEFT(TRIM($I4),1)="A",LEFT(TRIM($I4),1)="B",LEFT(TRIM($I4),1)="C",LEFT(TRIM($I4),1)="D",LEFT(TRIM($I4),1)="E"))),IF(COUNTIF($Q4:$AG4,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -2983,7 +2984,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L5" s="343" t="str">
-        <x:f>IF(TRIM($A5)="","",IF(COUNTIF($Q5:$AJ5,"?*")=0,"OK","Falta revisar: "&amp;$Q5&amp;$R5&amp;$S5&amp;$T5&amp;$U5&amp;$V5&amp;$W5&amp;$X5&amp;$Y5&amp;$Z5&amp;$AA5&amp;$AB5&amp;$AC5&amp;$AD5&amp;$AE5&amp;$AF5&amp;$AG5&amp;$AH5&amp;$AI5&amp;$AJ5))</x:f>
+        <x:f>IF(TRIM($A5)="","",IF(OR($A5="Selección de la mejor respuesta",$A5="SELECCION_MEJOR_RESPUESTA",$A5="Subítem de caso o problema",$A5="SUBITEM_CASO"),IF(TRIM($C5)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D5:$H5&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I5)&lt;&gt;"",OR(LEFT(TRIM($I5),1)="A",LEFT(TRIM($I5),1)="B",LEFT(TRIM($I5),1)="C",LEFT(TRIM($I5),1)="D",LEFT(TRIM($I5),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A5)="","",IF(COUNTIF($Q5:$AJ5,"?*")=0,"OK","Falta revisar: "&amp;$Q5&amp;$R5&amp;$S5&amp;$T5&amp;$U5&amp;$V5&amp;$W5&amp;$X5&amp;$Y5&amp;$Z5&amp;$AA5&amp;$AB5&amp;$AC5&amp;$AD5&amp;$AE5&amp;$AF5&amp;$AG5&amp;$AH5&amp;$AI5&amp;$AJ5))))</x:f>
       </x:c>
       <x:c r="M5" s="341"/>
       <x:c r="N5"/>
@@ -3039,7 +3040,7 @@
         <x:f>IF(AND($A5="Verdadero o Falso Complejas",TRIM($I5)&lt;&gt;"",NOT(OR(LEFT(TRIM($I5),1)="A",LEFT(TRIM($I5),1)="B",LEFT(TRIM($I5),1)="C",LEFT(TRIM($I5),1)="D",LEFT(TRIM($I5),1)="E"))),IF(COUNTIF($Q5:$AE5,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG5" t="str">
-        <x:f>IF(AND(OR($A5="Selección de la mejor respuesta",$A5="Subítem de caso o problema"),COUNTIF($D5:$H5,"?*")&lt;5),IF(COUNTIF($Q5:$AF5,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A5="Selección de la mejor respuesta",$A5="Subítem de caso o problema"),COUNTA($D5:$H5)&lt;5),IF(COUNTIF($Q5:$AF5,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH5" t="str">
         <x:f>IF(AND(OR($A5="Selección de la mejor respuesta",$A5="Subítem de caso o problema"),TRIM($I5)&lt;&gt;"",NOT(OR(LEFT(TRIM($I5),1)="A",LEFT(TRIM($I5),1)="B",LEFT(TRIM($I5),1)="C",LEFT(TRIM($I5),1)="D",LEFT(TRIM($I5),1)="E"))),IF(COUNTIF($Q5:$AG5,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3100,7 +3101,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L6" s="343" t="str">
-        <x:f>IF(TRIM($A6)="","",IF(COUNTIF($Q6:$AJ6,"?*")=0,"OK","Falta revisar: "&amp;$Q6&amp;$R6&amp;$S6&amp;$T6&amp;$U6&amp;$V6&amp;$W6&amp;$X6&amp;$Y6&amp;$Z6&amp;$AA6&amp;$AB6&amp;$AC6&amp;$AD6&amp;$AE6&amp;$AF6&amp;$AG6&amp;$AH6&amp;$AI6&amp;$AJ6))</x:f>
+        <x:f>IF(TRIM($A6)="","",IF(OR($A6="Selección de la mejor respuesta",$A6="SELECCION_MEJOR_RESPUESTA",$A6="Subítem de caso o problema",$A6="SUBITEM_CASO"),IF(TRIM($C6)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D6:$H6&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I6)&lt;&gt;"",OR(LEFT(TRIM($I6),1)="A",LEFT(TRIM($I6),1)="B",LEFT(TRIM($I6),1)="C",LEFT(TRIM($I6),1)="D",LEFT(TRIM($I6),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A6)="","",IF(COUNTIF($Q6:$AJ6,"?*")=0,"OK","Falta revisar: "&amp;$Q6&amp;$R6&amp;$S6&amp;$T6&amp;$U6&amp;$V6&amp;$W6&amp;$X6&amp;$Y6&amp;$Z6&amp;$AA6&amp;$AB6&amp;$AC6&amp;$AD6&amp;$AE6&amp;$AF6&amp;$AG6&amp;$AH6&amp;$AI6&amp;$AJ6))))</x:f>
       </x:c>
       <x:c r="M6" s="341"/>
       <x:c r="N6"/>
@@ -3156,7 +3157,7 @@
         <x:f>IF(AND($A6="Verdadero o Falso Complejas",TRIM($I6)&lt;&gt;"",NOT(OR(LEFT(TRIM($I6),1)="A",LEFT(TRIM($I6),1)="B",LEFT(TRIM($I6),1)="C",LEFT(TRIM($I6),1)="D",LEFT(TRIM($I6),1)="E"))),IF(COUNTIF($Q6:$AE6,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG6" t="str">
-        <x:f>IF(AND(OR($A6="Selección de la mejor respuesta",$A6="Subítem de caso o problema"),COUNTIF($D6:$H6,"?*")&lt;5),IF(COUNTIF($Q6:$AF6,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A6="Selección de la mejor respuesta",$A6="Subítem de caso o problema"),COUNTA($D6:$H6)&lt;5),IF(COUNTIF($Q6:$AF6,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH6" t="str">
         <x:f>IF(AND(OR($A6="Selección de la mejor respuesta",$A6="Subítem de caso o problema"),TRIM($I6)&lt;&gt;"",NOT(OR(LEFT(TRIM($I6),1)="A",LEFT(TRIM($I6),1)="B",LEFT(TRIM($I6),1)="C",LEFT(TRIM($I6),1)="D",LEFT(TRIM($I6),1)="E"))),IF(COUNTIF($Q6:$AG6,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3215,7 +3216,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L7" s="343" t="str">
-        <x:f>IF(TRIM($A7)="","",IF(COUNTIF($Q7:$AJ7,"?*")=0,"OK","Falta revisar: "&amp;$Q7&amp;$R7&amp;$S7&amp;$T7&amp;$U7&amp;$V7&amp;$W7&amp;$X7&amp;$Y7&amp;$Z7&amp;$AA7&amp;$AB7&amp;$AC7&amp;$AD7&amp;$AE7&amp;$AF7&amp;$AG7&amp;$AH7&amp;$AI7&amp;$AJ7))</x:f>
+        <x:f>IF(TRIM($A7)="","",IF(OR($A7="Selección de la mejor respuesta",$A7="SELECCION_MEJOR_RESPUESTA",$A7="Subítem de caso o problema",$A7="SUBITEM_CASO"),IF(TRIM($C7)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D7:$H7&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I7)&lt;&gt;"",OR(LEFT(TRIM($I7),1)="A",LEFT(TRIM($I7),1)="B",LEFT(TRIM($I7),1)="C",LEFT(TRIM($I7),1)="D",LEFT(TRIM($I7),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A7)="","",IF(COUNTIF($Q7:$AJ7,"?*")=0,"OK","Falta revisar: "&amp;$Q7&amp;$R7&amp;$S7&amp;$T7&amp;$U7&amp;$V7&amp;$W7&amp;$X7&amp;$Y7&amp;$Z7&amp;$AA7&amp;$AB7&amp;$AC7&amp;$AD7&amp;$AE7&amp;$AF7&amp;$AG7&amp;$AH7&amp;$AI7&amp;$AJ7))))</x:f>
       </x:c>
       <x:c r="M7" s="341"/>
       <x:c r="N7"/>
@@ -3271,7 +3272,7 @@
         <x:f>IF(AND($A7="Verdadero o Falso Complejas",TRIM($I7)&lt;&gt;"",NOT(OR(LEFT(TRIM($I7),1)="A",LEFT(TRIM($I7),1)="B",LEFT(TRIM($I7),1)="C",LEFT(TRIM($I7),1)="D",LEFT(TRIM($I7),1)="E"))),IF(COUNTIF($Q7:$AE7,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG7" t="str">
-        <x:f>IF(AND(OR($A7="Selección de la mejor respuesta",$A7="Subítem de caso o problema"),COUNTIF($D7:$H7,"?*")&lt;5),IF(COUNTIF($Q7:$AF7,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A7="Selección de la mejor respuesta",$A7="Subítem de caso o problema"),COUNTA($D7:$H7)&lt;5),IF(COUNTIF($Q7:$AF7,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH7" t="str">
         <x:f>IF(AND(OR($A7="Selección de la mejor respuesta",$A7="Subítem de caso o problema"),TRIM($I7)&lt;&gt;"",NOT(OR(LEFT(TRIM($I7),1)="A",LEFT(TRIM($I7),1)="B",LEFT(TRIM($I7),1)="C",LEFT(TRIM($I7),1)="D",LEFT(TRIM($I7),1)="E"))),IF(COUNTIF($Q7:$AG7,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3322,7 +3323,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L8" s="343" t="str">
-        <x:f>IF(TRIM($A8)="","",IF(COUNTIF($Q8:$AJ8,"?*")=0,"OK","Falta revisar: "&amp;$Q8&amp;$R8&amp;$S8&amp;$T8&amp;$U8&amp;$V8&amp;$W8&amp;$X8&amp;$Y8&amp;$Z8&amp;$AA8&amp;$AB8&amp;$AC8&amp;$AD8&amp;$AE8&amp;$AF8&amp;$AG8&amp;$AH8&amp;$AI8&amp;$AJ8))</x:f>
+        <x:f>IF(TRIM($A8)="","",IF(OR($A8="Selección de la mejor respuesta",$A8="SELECCION_MEJOR_RESPUESTA",$A8="Subítem de caso o problema",$A8="SUBITEM_CASO"),IF(TRIM($C8)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D8:$H8&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I8)&lt;&gt;"",OR(LEFT(TRIM($I8),1)="A",LEFT(TRIM($I8),1)="B",LEFT(TRIM($I8),1)="C",LEFT(TRIM($I8),1)="D",LEFT(TRIM($I8),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A8)="","",IF(COUNTIF($Q8:$AJ8,"?*")=0,"OK","Falta revisar: "&amp;$Q8&amp;$R8&amp;$S8&amp;$T8&amp;$U8&amp;$V8&amp;$W8&amp;$X8&amp;$Y8&amp;$Z8&amp;$AA8&amp;$AB8&amp;$AC8&amp;$AD8&amp;$AE8&amp;$AF8&amp;$AG8&amp;$AH8&amp;$AI8&amp;$AJ8))))</x:f>
       </x:c>
       <x:c r="M8" s="341"/>
       <x:c r="N8"/>
@@ -3378,7 +3379,7 @@
         <x:f>IF(AND($A8="Verdadero o Falso Complejas",TRIM($I8)&lt;&gt;"",NOT(OR(LEFT(TRIM($I8),1)="A",LEFT(TRIM($I8),1)="B",LEFT(TRIM($I8),1)="C",LEFT(TRIM($I8),1)="D",LEFT(TRIM($I8),1)="E"))),IF(COUNTIF($Q8:$AE8,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG8" t="str">
-        <x:f>IF(AND(OR($A8="Selección de la mejor respuesta",$A8="Subítem de caso o problema"),COUNTIF($D8:$H8,"?*")&lt;5),IF(COUNTIF($Q8:$AF8,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A8="Selección de la mejor respuesta",$A8="Subítem de caso o problema"),COUNTA($D8:$H8)&lt;5),IF(COUNTIF($Q8:$AF8,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH8" t="str">
         <x:f>IF(AND(OR($A8="Selección de la mejor respuesta",$A8="Subítem de caso o problema"),TRIM($I8)&lt;&gt;"",NOT(OR(LEFT(TRIM($I8),1)="A",LEFT(TRIM($I8),1)="B",LEFT(TRIM($I8),1)="C",LEFT(TRIM($I8),1)="D",LEFT(TRIM($I8),1)="E"))),IF(COUNTIF($Q8:$AG8,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3429,7 +3430,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L9" s="343" t="str">
-        <x:f>IF(TRIM($A9)="","",IF(COUNTIF($Q9:$AJ9,"?*")=0,"OK","Falta revisar: "&amp;$Q9&amp;$R9&amp;$S9&amp;$T9&amp;$U9&amp;$V9&amp;$W9&amp;$X9&amp;$Y9&amp;$Z9&amp;$AA9&amp;$AB9&amp;$AC9&amp;$AD9&amp;$AE9&amp;$AF9&amp;$AG9&amp;$AH9&amp;$AI9&amp;$AJ9))</x:f>
+        <x:f>IF(TRIM($A9)="","",IF(OR($A9="Selección de la mejor respuesta",$A9="SELECCION_MEJOR_RESPUESTA",$A9="Subítem de caso o problema",$A9="SUBITEM_CASO"),IF(TRIM($C9)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D9:$H9&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I9)&lt;&gt;"",OR(LEFT(TRIM($I9),1)="A",LEFT(TRIM($I9),1)="B",LEFT(TRIM($I9),1)="C",LEFT(TRIM($I9),1)="D",LEFT(TRIM($I9),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A9)="","",IF(COUNTIF($Q9:$AJ9,"?*")=0,"OK","Falta revisar: "&amp;$Q9&amp;$R9&amp;$S9&amp;$T9&amp;$U9&amp;$V9&amp;$W9&amp;$X9&amp;$Y9&amp;$Z9&amp;$AA9&amp;$AB9&amp;$AC9&amp;$AD9&amp;$AE9&amp;$AF9&amp;$AG9&amp;$AH9&amp;$AI9&amp;$AJ9))))</x:f>
       </x:c>
       <x:c r="M9" s="341"/>
       <x:c r="N9"/>
@@ -3485,7 +3486,7 @@
         <x:f>IF(AND($A9="Verdadero o Falso Complejas",TRIM($I9)&lt;&gt;"",NOT(OR(LEFT(TRIM($I9),1)="A",LEFT(TRIM($I9),1)="B",LEFT(TRIM($I9),1)="C",LEFT(TRIM($I9),1)="D",LEFT(TRIM($I9),1)="E"))),IF(COUNTIF($Q9:$AE9,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG9" t="str">
-        <x:f>IF(AND(OR($A9="Selección de la mejor respuesta",$A9="Subítem de caso o problema"),COUNTIF($D9:$H9,"?*")&lt;5),IF(COUNTIF($Q9:$AF9,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A9="Selección de la mejor respuesta",$A9="Subítem de caso o problema"),COUNTA($D9:$H9)&lt;5),IF(COUNTIF($Q9:$AF9,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH9" t="str">
         <x:f>IF(AND(OR($A9="Selección de la mejor respuesta",$A9="Subítem de caso o problema"),TRIM($I9)&lt;&gt;"",NOT(OR(LEFT(TRIM($I9),1)="A",LEFT(TRIM($I9),1)="B",LEFT(TRIM($I9),1)="C",LEFT(TRIM($I9),1)="D",LEFT(TRIM($I9),1)="E"))),IF(COUNTIF($Q9:$AG9,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3536,7 +3537,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L10" s="343" t="str">
-        <x:f>IF(TRIM($A10)="","",IF(COUNTIF($Q10:$AJ10,"?*")=0,"OK","Falta revisar: "&amp;$Q10&amp;$R10&amp;$S10&amp;$T10&amp;$U10&amp;$V10&amp;$W10&amp;$X10&amp;$Y10&amp;$Z10&amp;$AA10&amp;$AB10&amp;$AC10&amp;$AD10&amp;$AE10&amp;$AF10&amp;$AG10&amp;$AH10&amp;$AI10&amp;$AJ10))</x:f>
+        <x:f>IF(TRIM($A10)="","",IF(OR($A10="Selección de la mejor respuesta",$A10="SELECCION_MEJOR_RESPUESTA",$A10="Subítem de caso o problema",$A10="SUBITEM_CASO"),IF(TRIM($C10)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D10:$H10&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I10)&lt;&gt;"",OR(LEFT(TRIM($I10),1)="A",LEFT(TRIM($I10),1)="B",LEFT(TRIM($I10),1)="C",LEFT(TRIM($I10),1)="D",LEFT(TRIM($I10),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A10)="","",IF(COUNTIF($Q10:$AJ10,"?*")=0,"OK","Falta revisar: "&amp;$Q10&amp;$R10&amp;$S10&amp;$T10&amp;$U10&amp;$V10&amp;$W10&amp;$X10&amp;$Y10&amp;$Z10&amp;$AA10&amp;$AB10&amp;$AC10&amp;$AD10&amp;$AE10&amp;$AF10&amp;$AG10&amp;$AH10&amp;$AI10&amp;$AJ10))))</x:f>
       </x:c>
       <x:c r="M10" s="341"/>
       <x:c r="N10"/>
@@ -3592,7 +3593,7 @@
         <x:f>IF(AND($A10="Verdadero o Falso Complejas",TRIM($I10)&lt;&gt;"",NOT(OR(LEFT(TRIM($I10),1)="A",LEFT(TRIM($I10),1)="B",LEFT(TRIM($I10),1)="C",LEFT(TRIM($I10),1)="D",LEFT(TRIM($I10),1)="E"))),IF(COUNTIF($Q10:$AE10,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG10" t="str">
-        <x:f>IF(AND(OR($A10="Selección de la mejor respuesta",$A10="Subítem de caso o problema"),COUNTIF($D10:$H10,"?*")&lt;5),IF(COUNTIF($Q10:$AF10,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A10="Selección de la mejor respuesta",$A10="Subítem de caso o problema"),COUNTA($D10:$H10)&lt;5),IF(COUNTIF($Q10:$AF10,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH10" t="str">
         <x:f>IF(AND(OR($A10="Selección de la mejor respuesta",$A10="Subítem de caso o problema"),TRIM($I10)&lt;&gt;"",NOT(OR(LEFT(TRIM($I10),1)="A",LEFT(TRIM($I10),1)="B",LEFT(TRIM($I10),1)="C",LEFT(TRIM($I10),1)="D",LEFT(TRIM($I10),1)="E"))),IF(COUNTIF($Q10:$AG10,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3643,7 +3644,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L11" s="343" t="str">
-        <x:f>IF(TRIM($A11)="","",IF(COUNTIF($Q11:$AJ11,"?*")=0,"OK","Falta revisar: "&amp;$Q11&amp;$R11&amp;$S11&amp;$T11&amp;$U11&amp;$V11&amp;$W11&amp;$X11&amp;$Y11&amp;$Z11&amp;$AA11&amp;$AB11&amp;$AC11&amp;$AD11&amp;$AE11&amp;$AF11&amp;$AG11&amp;$AH11&amp;$AI11&amp;$AJ11))</x:f>
+        <x:f>IF(TRIM($A11)="","",IF(OR($A11="Selección de la mejor respuesta",$A11="SELECCION_MEJOR_RESPUESTA",$A11="Subítem de caso o problema",$A11="SUBITEM_CASO"),IF(TRIM($C11)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D11:$H11&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I11)&lt;&gt;"",OR(LEFT(TRIM($I11),1)="A",LEFT(TRIM($I11),1)="B",LEFT(TRIM($I11),1)="C",LEFT(TRIM($I11),1)="D",LEFT(TRIM($I11),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A11)="","",IF(COUNTIF($Q11:$AJ11,"?*")=0,"OK","Falta revisar: "&amp;$Q11&amp;$R11&amp;$S11&amp;$T11&amp;$U11&amp;$V11&amp;$W11&amp;$X11&amp;$Y11&amp;$Z11&amp;$AA11&amp;$AB11&amp;$AC11&amp;$AD11&amp;$AE11&amp;$AF11&amp;$AG11&amp;$AH11&amp;$AI11&amp;$AJ11))))</x:f>
       </x:c>
       <x:c r="M11" s="341"/>
       <x:c r="N11"/>
@@ -3699,7 +3700,7 @@
         <x:f>IF(AND($A11="Verdadero o Falso Complejas",TRIM($I11)&lt;&gt;"",NOT(OR(LEFT(TRIM($I11),1)="A",LEFT(TRIM($I11),1)="B",LEFT(TRIM($I11),1)="C",LEFT(TRIM($I11),1)="D",LEFT(TRIM($I11),1)="E"))),IF(COUNTIF($Q11:$AE11,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG11" t="str">
-        <x:f>IF(AND(OR($A11="Selección de la mejor respuesta",$A11="Subítem de caso o problema"),COUNTIF($D11:$H11,"?*")&lt;5),IF(COUNTIF($Q11:$AF11,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A11="Selección de la mejor respuesta",$A11="Subítem de caso o problema"),COUNTA($D11:$H11)&lt;5),IF(COUNTIF($Q11:$AF11,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH11" t="str">
         <x:f>IF(AND(OR($A11="Selección de la mejor respuesta",$A11="Subítem de caso o problema"),TRIM($I11)&lt;&gt;"",NOT(OR(LEFT(TRIM($I11),1)="A",LEFT(TRIM($I11),1)="B",LEFT(TRIM($I11),1)="C",LEFT(TRIM($I11),1)="D",LEFT(TRIM($I11),1)="E"))),IF(COUNTIF($Q11:$AG11,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3750,7 +3751,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L12" s="343" t="str">
-        <x:f>IF(TRIM($A12)="","",IF(COUNTIF($Q12:$AJ12,"?*")=0,"OK","Falta revisar: "&amp;$Q12&amp;$R12&amp;$S12&amp;$T12&amp;$U12&amp;$V12&amp;$W12&amp;$X12&amp;$Y12&amp;$Z12&amp;$AA12&amp;$AB12&amp;$AC12&amp;$AD12&amp;$AE12&amp;$AF12&amp;$AG12&amp;$AH12&amp;$AI12&amp;$AJ12))</x:f>
+        <x:f>IF(TRIM($A12)="","",IF(OR($A12="Selección de la mejor respuesta",$A12="SELECCION_MEJOR_RESPUESTA",$A12="Subítem de caso o problema",$A12="SUBITEM_CASO"),IF(TRIM($C12)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D12:$H12&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I12)&lt;&gt;"",OR(LEFT(TRIM($I12),1)="A",LEFT(TRIM($I12),1)="B",LEFT(TRIM($I12),1)="C",LEFT(TRIM($I12),1)="D",LEFT(TRIM($I12),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A12)="","",IF(COUNTIF($Q12:$AJ12,"?*")=0,"OK","Falta revisar: "&amp;$Q12&amp;$R12&amp;$S12&amp;$T12&amp;$U12&amp;$V12&amp;$W12&amp;$X12&amp;$Y12&amp;$Z12&amp;$AA12&amp;$AB12&amp;$AC12&amp;$AD12&amp;$AE12&amp;$AF12&amp;$AG12&amp;$AH12&amp;$AI12&amp;$AJ12))))</x:f>
       </x:c>
       <x:c r="M12" s="341"/>
       <x:c r="N12"/>
@@ -3806,7 +3807,7 @@
         <x:f>IF(AND($A12="Verdadero o Falso Complejas",TRIM($I12)&lt;&gt;"",NOT(OR(LEFT(TRIM($I12),1)="A",LEFT(TRIM($I12),1)="B",LEFT(TRIM($I12),1)="C",LEFT(TRIM($I12),1)="D",LEFT(TRIM($I12),1)="E"))),IF(COUNTIF($Q12:$AE12,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG12" t="str">
-        <x:f>IF(AND(OR($A12="Selección de la mejor respuesta",$A12="Subítem de caso o problema"),COUNTIF($D12:$H12,"?*")&lt;5),IF(COUNTIF($Q12:$AF12,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A12="Selección de la mejor respuesta",$A12="Subítem de caso o problema"),COUNTA($D12:$H12)&lt;5),IF(COUNTIF($Q12:$AF12,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH12" t="str">
         <x:f>IF(AND(OR($A12="Selección de la mejor respuesta",$A12="Subítem de caso o problema"),TRIM($I12)&lt;&gt;"",NOT(OR(LEFT(TRIM($I12),1)="A",LEFT(TRIM($I12),1)="B",LEFT(TRIM($I12),1)="C",LEFT(TRIM($I12),1)="D",LEFT(TRIM($I12),1)="E"))),IF(COUNTIF($Q12:$AG12,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3857,7 +3858,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L13" s="343" t="str">
-        <x:f>IF(TRIM($A13)="","",IF(COUNTIF($Q13:$AJ13,"?*")=0,"OK","Falta revisar: "&amp;$Q13&amp;$R13&amp;$S13&amp;$T13&amp;$U13&amp;$V13&amp;$W13&amp;$X13&amp;$Y13&amp;$Z13&amp;$AA13&amp;$AB13&amp;$AC13&amp;$AD13&amp;$AE13&amp;$AF13&amp;$AG13&amp;$AH13&amp;$AI13&amp;$AJ13))</x:f>
+        <x:f>IF(TRIM($A13)="","",IF(OR($A13="Selección de la mejor respuesta",$A13="SELECCION_MEJOR_RESPUESTA",$A13="Subítem de caso o problema",$A13="SUBITEM_CASO"),IF(TRIM($C13)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D13:$H13&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I13)&lt;&gt;"",OR(LEFT(TRIM($I13),1)="A",LEFT(TRIM($I13),1)="B",LEFT(TRIM($I13),1)="C",LEFT(TRIM($I13),1)="D",LEFT(TRIM($I13),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A13)="","",IF(COUNTIF($Q13:$AJ13,"?*")=0,"OK","Falta revisar: "&amp;$Q13&amp;$R13&amp;$S13&amp;$T13&amp;$U13&amp;$V13&amp;$W13&amp;$X13&amp;$Y13&amp;$Z13&amp;$AA13&amp;$AB13&amp;$AC13&amp;$AD13&amp;$AE13&amp;$AF13&amp;$AG13&amp;$AH13&amp;$AI13&amp;$AJ13))))</x:f>
       </x:c>
       <x:c r="M13" s="341"/>
       <x:c r="N13"/>
@@ -3913,7 +3914,7 @@
         <x:f>IF(AND($A13="Verdadero o Falso Complejas",TRIM($I13)&lt;&gt;"",NOT(OR(LEFT(TRIM($I13),1)="A",LEFT(TRIM($I13),1)="B",LEFT(TRIM($I13),1)="C",LEFT(TRIM($I13),1)="D",LEFT(TRIM($I13),1)="E"))),IF(COUNTIF($Q13:$AE13,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG13" t="str">
-        <x:f>IF(AND(OR($A13="Selección de la mejor respuesta",$A13="Subítem de caso o problema"),COUNTIF($D13:$H13,"?*")&lt;5),IF(COUNTIF($Q13:$AF13,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A13="Selección de la mejor respuesta",$A13="Subítem de caso o problema"),COUNTA($D13:$H13)&lt;5),IF(COUNTIF($Q13:$AF13,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH13" t="str">
         <x:f>IF(AND(OR($A13="Selección de la mejor respuesta",$A13="Subítem de caso o problema"),TRIM($I13)&lt;&gt;"",NOT(OR(LEFT(TRIM($I13),1)="A",LEFT(TRIM($I13),1)="B",LEFT(TRIM($I13),1)="C",LEFT(TRIM($I13),1)="D",LEFT(TRIM($I13),1)="E"))),IF(COUNTIF($Q13:$AG13,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -3964,7 +3965,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L14" s="343" t="str">
-        <x:f>IF(TRIM($A14)="","",IF(COUNTIF($Q14:$AJ14,"?*")=0,"OK","Falta revisar: "&amp;$Q14&amp;$R14&amp;$S14&amp;$T14&amp;$U14&amp;$V14&amp;$W14&amp;$X14&amp;$Y14&amp;$Z14&amp;$AA14&amp;$AB14&amp;$AC14&amp;$AD14&amp;$AE14&amp;$AF14&amp;$AG14&amp;$AH14&amp;$AI14&amp;$AJ14))</x:f>
+        <x:f>IF(TRIM($A14)="","",IF(OR($A14="Selección de la mejor respuesta",$A14="SELECCION_MEJOR_RESPUESTA",$A14="Subítem de caso o problema",$A14="SUBITEM_CASO"),IF(TRIM($C14)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D14:$H14&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I14)&lt;&gt;"",OR(LEFT(TRIM($I14),1)="A",LEFT(TRIM($I14),1)="B",LEFT(TRIM($I14),1)="C",LEFT(TRIM($I14),1)="D",LEFT(TRIM($I14),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A14)="","",IF(COUNTIF($Q14:$AJ14,"?*")=0,"OK","Falta revisar: "&amp;$Q14&amp;$R14&amp;$S14&amp;$T14&amp;$U14&amp;$V14&amp;$W14&amp;$X14&amp;$Y14&amp;$Z14&amp;$AA14&amp;$AB14&amp;$AC14&amp;$AD14&amp;$AE14&amp;$AF14&amp;$AG14&amp;$AH14&amp;$AI14&amp;$AJ14))))</x:f>
       </x:c>
       <x:c r="M14" s="341"/>
       <x:c r="N14"/>
@@ -4020,7 +4021,7 @@
         <x:f>IF(AND($A14="Verdadero o Falso Complejas",TRIM($I14)&lt;&gt;"",NOT(OR(LEFT(TRIM($I14),1)="A",LEFT(TRIM($I14),1)="B",LEFT(TRIM($I14),1)="C",LEFT(TRIM($I14),1)="D",LEFT(TRIM($I14),1)="E"))),IF(COUNTIF($Q14:$AE14,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG14" t="str">
-        <x:f>IF(AND(OR($A14="Selección de la mejor respuesta",$A14="Subítem de caso o problema"),COUNTIF($D14:$H14,"?*")&lt;5),IF(COUNTIF($Q14:$AF14,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A14="Selección de la mejor respuesta",$A14="Subítem de caso o problema"),COUNTA($D14:$H14)&lt;5),IF(COUNTIF($Q14:$AF14,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH14" t="str">
         <x:f>IF(AND(OR($A14="Selección de la mejor respuesta",$A14="Subítem de caso o problema"),TRIM($I14)&lt;&gt;"",NOT(OR(LEFT(TRIM($I14),1)="A",LEFT(TRIM($I14),1)="B",LEFT(TRIM($I14),1)="C",LEFT(TRIM($I14),1)="D",LEFT(TRIM($I14),1)="E"))),IF(COUNTIF($Q14:$AG14,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4071,7 +4072,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L15" s="343" t="str">
-        <x:f>IF(TRIM($A15)="","",IF(COUNTIF($Q15:$AJ15,"?*")=0,"OK","Falta revisar: "&amp;$Q15&amp;$R15&amp;$S15&amp;$T15&amp;$U15&amp;$V15&amp;$W15&amp;$X15&amp;$Y15&amp;$Z15&amp;$AA15&amp;$AB15&amp;$AC15&amp;$AD15&amp;$AE15&amp;$AF15&amp;$AG15&amp;$AH15&amp;$AI15&amp;$AJ15))</x:f>
+        <x:f>IF(TRIM($A15)="","",IF(OR($A15="Selección de la mejor respuesta",$A15="SELECCION_MEJOR_RESPUESTA",$A15="Subítem de caso o problema",$A15="SUBITEM_CASO"),IF(TRIM($C15)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D15:$H15&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I15)&lt;&gt;"",OR(LEFT(TRIM($I15),1)="A",LEFT(TRIM($I15),1)="B",LEFT(TRIM($I15),1)="C",LEFT(TRIM($I15),1)="D",LEFT(TRIM($I15),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A15)="","",IF(COUNTIF($Q15:$AJ15,"?*")=0,"OK","Falta revisar: "&amp;$Q15&amp;$R15&amp;$S15&amp;$T15&amp;$U15&amp;$V15&amp;$W15&amp;$X15&amp;$Y15&amp;$Z15&amp;$AA15&amp;$AB15&amp;$AC15&amp;$AD15&amp;$AE15&amp;$AF15&amp;$AG15&amp;$AH15&amp;$AI15&amp;$AJ15))))</x:f>
       </x:c>
       <x:c r="M15" s="341"/>
       <x:c r="N15"/>
@@ -4127,7 +4128,7 @@
         <x:f>IF(AND($A15="Verdadero o Falso Complejas",TRIM($I15)&lt;&gt;"",NOT(OR(LEFT(TRIM($I15),1)="A",LEFT(TRIM($I15),1)="B",LEFT(TRIM($I15),1)="C",LEFT(TRIM($I15),1)="D",LEFT(TRIM($I15),1)="E"))),IF(COUNTIF($Q15:$AE15,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG15" t="str">
-        <x:f>IF(AND(OR($A15="Selección de la mejor respuesta",$A15="Subítem de caso o problema"),COUNTIF($D15:$H15,"?*")&lt;5),IF(COUNTIF($Q15:$AF15,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A15="Selección de la mejor respuesta",$A15="Subítem de caso o problema"),COUNTA($D15:$H15)&lt;5),IF(COUNTIF($Q15:$AF15,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH15" t="str">
         <x:f>IF(AND(OR($A15="Selección de la mejor respuesta",$A15="Subítem de caso o problema"),TRIM($I15)&lt;&gt;"",NOT(OR(LEFT(TRIM($I15),1)="A",LEFT(TRIM($I15),1)="B",LEFT(TRIM($I15),1)="C",LEFT(TRIM($I15),1)="D",LEFT(TRIM($I15),1)="E"))),IF(COUNTIF($Q15:$AG15,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4178,7 +4179,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L16" s="343" t="str">
-        <x:f>IF(TRIM($A16)="","",IF(COUNTIF($Q16:$AJ16,"?*")=0,"OK","Falta revisar: "&amp;$Q16&amp;$R16&amp;$S16&amp;$T16&amp;$U16&amp;$V16&amp;$W16&amp;$X16&amp;$Y16&amp;$Z16&amp;$AA16&amp;$AB16&amp;$AC16&amp;$AD16&amp;$AE16&amp;$AF16&amp;$AG16&amp;$AH16&amp;$AI16&amp;$AJ16))</x:f>
+        <x:f>IF(TRIM($A16)="","",IF(OR($A16="Selección de la mejor respuesta",$A16="SELECCION_MEJOR_RESPUESTA",$A16="Subítem de caso o problema",$A16="SUBITEM_CASO"),IF(TRIM($C16)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D16:$H16&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I16)&lt;&gt;"",OR(LEFT(TRIM($I16),1)="A",LEFT(TRIM($I16),1)="B",LEFT(TRIM($I16),1)="C",LEFT(TRIM($I16),1)="D",LEFT(TRIM($I16),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A16)="","",IF(COUNTIF($Q16:$AJ16,"?*")=0,"OK","Falta revisar: "&amp;$Q16&amp;$R16&amp;$S16&amp;$T16&amp;$U16&amp;$V16&amp;$W16&amp;$X16&amp;$Y16&amp;$Z16&amp;$AA16&amp;$AB16&amp;$AC16&amp;$AD16&amp;$AE16&amp;$AF16&amp;$AG16&amp;$AH16&amp;$AI16&amp;$AJ16))))</x:f>
       </x:c>
       <x:c r="M16" s="341"/>
       <x:c r="N16"/>
@@ -4234,7 +4235,7 @@
         <x:f>IF(AND($A16="Verdadero o Falso Complejas",TRIM($I16)&lt;&gt;"",NOT(OR(LEFT(TRIM($I16),1)="A",LEFT(TRIM($I16),1)="B",LEFT(TRIM($I16),1)="C",LEFT(TRIM($I16),1)="D",LEFT(TRIM($I16),1)="E"))),IF(COUNTIF($Q16:$AE16,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG16" t="str">
-        <x:f>IF(AND(OR($A16="Selección de la mejor respuesta",$A16="Subítem de caso o problema"),COUNTIF($D16:$H16,"?*")&lt;5),IF(COUNTIF($Q16:$AF16,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A16="Selección de la mejor respuesta",$A16="Subítem de caso o problema"),COUNTA($D16:$H16)&lt;5),IF(COUNTIF($Q16:$AF16,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH16" t="str">
         <x:f>IF(AND(OR($A16="Selección de la mejor respuesta",$A16="Subítem de caso o problema"),TRIM($I16)&lt;&gt;"",NOT(OR(LEFT(TRIM($I16),1)="A",LEFT(TRIM($I16),1)="B",LEFT(TRIM($I16),1)="C",LEFT(TRIM($I16),1)="D",LEFT(TRIM($I16),1)="E"))),IF(COUNTIF($Q16:$AG16,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4285,7 +4286,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L17" s="345" t="str">
-        <x:f>IF(TRIM($A17)="","",IF(COUNTIF($Q17:$AJ17,"?*")=0,"OK","Falta revisar: "&amp;$Q17&amp;$R17&amp;$S17&amp;$T17&amp;$U17&amp;$V17&amp;$W17&amp;$X17&amp;$Y17&amp;$Z17&amp;$AA17&amp;$AB17&amp;$AC17&amp;$AD17&amp;$AE17&amp;$AF17&amp;$AG17&amp;$AH17&amp;$AI17&amp;$AJ17))</x:f>
+        <x:f>IF(TRIM($A17)="","",IF(OR($A17="Selección de la mejor respuesta",$A17="SELECCION_MEJOR_RESPUESTA",$A17="Subítem de caso o problema",$A17="SUBITEM_CASO"),IF(TRIM($C17)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D17:$H17&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I17)&lt;&gt;"",OR(LEFT(TRIM($I17),1)="A",LEFT(TRIM($I17),1)="B",LEFT(TRIM($I17),1)="C",LEFT(TRIM($I17),1)="D",LEFT(TRIM($I17),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A17)="","",IF(COUNTIF($Q17:$AJ17,"?*")=0,"OK","Falta revisar: "&amp;$Q17&amp;$R17&amp;$S17&amp;$T17&amp;$U17&amp;$V17&amp;$W17&amp;$X17&amp;$Y17&amp;$Z17&amp;$AA17&amp;$AB17&amp;$AC17&amp;$AD17&amp;$AE17&amp;$AF17&amp;$AG17&amp;$AH17&amp;$AI17&amp;$AJ17))))</x:f>
       </x:c>
       <x:c r="M17" s="341"/>
       <x:c r="N17"/>
@@ -4341,7 +4342,7 @@
         <x:f>IF(AND($A17="Verdadero o Falso Complejas",TRIM($I17)&lt;&gt;"",NOT(OR(LEFT(TRIM($I17),1)="A",LEFT(TRIM($I17),1)="B",LEFT(TRIM($I17),1)="C",LEFT(TRIM($I17),1)="D",LEFT(TRIM($I17),1)="E"))),IF(COUNTIF($Q17:$AE17,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG17" t="str">
-        <x:f>IF(AND(OR($A17="Selección de la mejor respuesta",$A17="Subítem de caso o problema"),COUNTIF($D17:$H17,"?*")&lt;5),IF(COUNTIF($Q17:$AF17,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A17="Selección de la mejor respuesta",$A17="Subítem de caso o problema"),COUNTA($D17:$H17)&lt;5),IF(COUNTIF($Q17:$AF17,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH17" t="str">
         <x:f>IF(AND(OR($A17="Selección de la mejor respuesta",$A17="Subítem de caso o problema"),TRIM($I17)&lt;&gt;"",NOT(OR(LEFT(TRIM($I17),1)="A",LEFT(TRIM($I17),1)="B",LEFT(TRIM($I17),1)="C",LEFT(TRIM($I17),1)="D",LEFT(TRIM($I17),1)="E"))),IF(COUNTIF($Q17:$AG17,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4392,7 +4393,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L18" s="345" t="str">
-        <x:f>IF(TRIM($A18)="","",IF(COUNTIF($Q18:$AJ18,"?*")=0,"OK","Falta revisar: "&amp;$Q18&amp;$R18&amp;$S18&amp;$T18&amp;$U18&amp;$V18&amp;$W18&amp;$X18&amp;$Y18&amp;$Z18&amp;$AA18&amp;$AB18&amp;$AC18&amp;$AD18&amp;$AE18&amp;$AF18&amp;$AG18&amp;$AH18&amp;$AI18&amp;$AJ18))</x:f>
+        <x:f>IF(TRIM($A18)="","",IF(OR($A18="Selección de la mejor respuesta",$A18="SELECCION_MEJOR_RESPUESTA",$A18="Subítem de caso o problema",$A18="SUBITEM_CASO"),IF(TRIM($C18)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D18:$H18&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I18)&lt;&gt;"",OR(LEFT(TRIM($I18),1)="A",LEFT(TRIM($I18),1)="B",LEFT(TRIM($I18),1)="C",LEFT(TRIM($I18),1)="D",LEFT(TRIM($I18),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A18)="","",IF(COUNTIF($Q18:$AJ18,"?*")=0,"OK","Falta revisar: "&amp;$Q18&amp;$R18&amp;$S18&amp;$T18&amp;$U18&amp;$V18&amp;$W18&amp;$X18&amp;$Y18&amp;$Z18&amp;$AA18&amp;$AB18&amp;$AC18&amp;$AD18&amp;$AE18&amp;$AF18&amp;$AG18&amp;$AH18&amp;$AI18&amp;$AJ18))))</x:f>
       </x:c>
       <x:c r="M18" s="341"/>
       <x:c r="N18"/>
@@ -4448,7 +4449,7 @@
         <x:f>IF(AND($A18="Verdadero o Falso Complejas",TRIM($I18)&lt;&gt;"",NOT(OR(LEFT(TRIM($I18),1)="A",LEFT(TRIM($I18),1)="B",LEFT(TRIM($I18),1)="C",LEFT(TRIM($I18),1)="D",LEFT(TRIM($I18),1)="E"))),IF(COUNTIF($Q18:$AE18,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG18" t="str">
-        <x:f>IF(AND(OR($A18="Selección de la mejor respuesta",$A18="Subítem de caso o problema"),COUNTIF($D18:$H18,"?*")&lt;5),IF(COUNTIF($Q18:$AF18,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A18="Selección de la mejor respuesta",$A18="Subítem de caso o problema"),COUNTA($D18:$H18)&lt;5),IF(COUNTIF($Q18:$AF18,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH18" t="str">
         <x:f>IF(AND(OR($A18="Selección de la mejor respuesta",$A18="Subítem de caso o problema"),TRIM($I18)&lt;&gt;"",NOT(OR(LEFT(TRIM($I18),1)="A",LEFT(TRIM($I18),1)="B",LEFT(TRIM($I18),1)="C",LEFT(TRIM($I18),1)="D",LEFT(TRIM($I18),1)="E"))),IF(COUNTIF($Q18:$AG18,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4499,7 +4500,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L19" s="345" t="str">
-        <x:f>IF(TRIM($A19)="","",IF(COUNTIF($Q19:$AJ19,"?*")=0,"OK","Falta revisar: "&amp;$Q19&amp;$R19&amp;$S19&amp;$T19&amp;$U19&amp;$V19&amp;$W19&amp;$X19&amp;$Y19&amp;$Z19&amp;$AA19&amp;$AB19&amp;$AC19&amp;$AD19&amp;$AE19&amp;$AF19&amp;$AG19&amp;$AH19&amp;$AI19&amp;$AJ19))</x:f>
+        <x:f>IF(TRIM($A19)="","",IF(OR($A19="Selección de la mejor respuesta",$A19="SELECCION_MEJOR_RESPUESTA",$A19="Subítem de caso o problema",$A19="SUBITEM_CASO"),IF(TRIM($C19)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D19:$H19&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I19)&lt;&gt;"",OR(LEFT(TRIM($I19),1)="A",LEFT(TRIM($I19),1)="B",LEFT(TRIM($I19),1)="C",LEFT(TRIM($I19),1)="D",LEFT(TRIM($I19),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A19)="","",IF(COUNTIF($Q19:$AJ19,"?*")=0,"OK","Falta revisar: "&amp;$Q19&amp;$R19&amp;$S19&amp;$T19&amp;$U19&amp;$V19&amp;$W19&amp;$X19&amp;$Y19&amp;$Z19&amp;$AA19&amp;$AB19&amp;$AC19&amp;$AD19&amp;$AE19&amp;$AF19&amp;$AG19&amp;$AH19&amp;$AI19&amp;$AJ19))))</x:f>
       </x:c>
       <x:c r="M19" s="341"/>
       <x:c r="N19"/>
@@ -4555,7 +4556,7 @@
         <x:f>IF(AND($A19="Verdadero o Falso Complejas",TRIM($I19)&lt;&gt;"",NOT(OR(LEFT(TRIM($I19),1)="A",LEFT(TRIM($I19),1)="B",LEFT(TRIM($I19),1)="C",LEFT(TRIM($I19),1)="D",LEFT(TRIM($I19),1)="E"))),IF(COUNTIF($Q19:$AE19,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG19" t="str">
-        <x:f>IF(AND(OR($A19="Selección de la mejor respuesta",$A19="Subítem de caso o problema"),COUNTIF($D19:$H19,"?*")&lt;5),IF(COUNTIF($Q19:$AF19,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A19="Selección de la mejor respuesta",$A19="Subítem de caso o problema"),COUNTA($D19:$H19)&lt;5),IF(COUNTIF($Q19:$AF19,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH19" t="str">
         <x:f>IF(AND(OR($A19="Selección de la mejor respuesta",$A19="Subítem de caso o problema"),TRIM($I19)&lt;&gt;"",NOT(OR(LEFT(TRIM($I19),1)="A",LEFT(TRIM($I19),1)="B",LEFT(TRIM($I19),1)="C",LEFT(TRIM($I19),1)="D",LEFT(TRIM($I19),1)="E"))),IF(COUNTIF($Q19:$AG19,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4606,7 +4607,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L20" s="345" t="str">
-        <x:f>IF(TRIM($A20)="","",IF(COUNTIF($Q20:$AJ20,"?*")=0,"OK","Falta revisar: "&amp;$Q20&amp;$R20&amp;$S20&amp;$T20&amp;$U20&amp;$V20&amp;$W20&amp;$X20&amp;$Y20&amp;$Z20&amp;$AA20&amp;$AB20&amp;$AC20&amp;$AD20&amp;$AE20&amp;$AF20&amp;$AG20&amp;$AH20&amp;$AI20&amp;$AJ20))</x:f>
+        <x:f>IF(TRIM($A20)="","",IF(OR($A20="Selección de la mejor respuesta",$A20="SELECCION_MEJOR_RESPUESTA",$A20="Subítem de caso o problema",$A20="SUBITEM_CASO"),IF(TRIM($C20)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D20:$H20&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I20)&lt;&gt;"",OR(LEFT(TRIM($I20),1)="A",LEFT(TRIM($I20),1)="B",LEFT(TRIM($I20),1)="C",LEFT(TRIM($I20),1)="D",LEFT(TRIM($I20),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A20)="","",IF(COUNTIF($Q20:$AJ20,"?*")=0,"OK","Falta revisar: "&amp;$Q20&amp;$R20&amp;$S20&amp;$T20&amp;$U20&amp;$V20&amp;$W20&amp;$X20&amp;$Y20&amp;$Z20&amp;$AA20&amp;$AB20&amp;$AC20&amp;$AD20&amp;$AE20&amp;$AF20&amp;$AG20&amp;$AH20&amp;$AI20&amp;$AJ20))))</x:f>
       </x:c>
       <x:c r="M20" s="341"/>
       <x:c r="N20"/>
@@ -4662,7 +4663,7 @@
         <x:f>IF(AND($A20="Verdadero o Falso Complejas",TRIM($I20)&lt;&gt;"",NOT(OR(LEFT(TRIM($I20),1)="A",LEFT(TRIM($I20),1)="B",LEFT(TRIM($I20),1)="C",LEFT(TRIM($I20),1)="D",LEFT(TRIM($I20),1)="E"))),IF(COUNTIF($Q20:$AE20,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG20" t="str">
-        <x:f>IF(AND(OR($A20="Selección de la mejor respuesta",$A20="Subítem de caso o problema"),COUNTIF($D20:$H20,"?*")&lt;5),IF(COUNTIF($Q20:$AF20,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A20="Selección de la mejor respuesta",$A20="Subítem de caso o problema"),COUNTA($D20:$H20)&lt;5),IF(COUNTIF($Q20:$AF20,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH20" t="str">
         <x:f>IF(AND(OR($A20="Selección de la mejor respuesta",$A20="Subítem de caso o problema"),TRIM($I20)&lt;&gt;"",NOT(OR(LEFT(TRIM($I20),1)="A",LEFT(TRIM($I20),1)="B",LEFT(TRIM($I20),1)="C",LEFT(TRIM($I20),1)="D",LEFT(TRIM($I20),1)="E"))),IF(COUNTIF($Q20:$AG20,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4713,7 +4714,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L21" s="345" t="str">
-        <x:f>IF(TRIM($A21)="","",IF(COUNTIF($Q21:$AJ21,"?*")=0,"OK","Falta revisar: "&amp;$Q21&amp;$R21&amp;$S21&amp;$T21&amp;$U21&amp;$V21&amp;$W21&amp;$X21&amp;$Y21&amp;$Z21&amp;$AA21&amp;$AB21&amp;$AC21&amp;$AD21&amp;$AE21&amp;$AF21&amp;$AG21&amp;$AH21&amp;$AI21&amp;$AJ21))</x:f>
+        <x:f>IF(TRIM($A21)="","",IF(OR($A21="Selección de la mejor respuesta",$A21="SELECCION_MEJOR_RESPUESTA",$A21="Subítem de caso o problema",$A21="SUBITEM_CASO"),IF(TRIM($C21)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D21:$H21&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I21)&lt;&gt;"",OR(LEFT(TRIM($I21),1)="A",LEFT(TRIM($I21),1)="B",LEFT(TRIM($I21),1)="C",LEFT(TRIM($I21),1)="D",LEFT(TRIM($I21),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A21)="","",IF(COUNTIF($Q21:$AJ21,"?*")=0,"OK","Falta revisar: "&amp;$Q21&amp;$R21&amp;$S21&amp;$T21&amp;$U21&amp;$V21&amp;$W21&amp;$X21&amp;$Y21&amp;$Z21&amp;$AA21&amp;$AB21&amp;$AC21&amp;$AD21&amp;$AE21&amp;$AF21&amp;$AG21&amp;$AH21&amp;$AI21&amp;$AJ21))))</x:f>
       </x:c>
       <x:c r="M21" s="341"/>
       <x:c r="N21"/>
@@ -4769,7 +4770,7 @@
         <x:f>IF(AND($A21="Verdadero o Falso Complejas",TRIM($I21)&lt;&gt;"",NOT(OR(LEFT(TRIM($I21),1)="A",LEFT(TRIM($I21),1)="B",LEFT(TRIM($I21),1)="C",LEFT(TRIM($I21),1)="D",LEFT(TRIM($I21),1)="E"))),IF(COUNTIF($Q21:$AE21,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG21" t="str">
-        <x:f>IF(AND(OR($A21="Selección de la mejor respuesta",$A21="Subítem de caso o problema"),COUNTIF($D21:$H21,"?*")&lt;5),IF(COUNTIF($Q21:$AF21,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A21="Selección de la mejor respuesta",$A21="Subítem de caso o problema"),COUNTA($D21:$H21)&lt;5),IF(COUNTIF($Q21:$AF21,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH21" t="str">
         <x:f>IF(AND(OR($A21="Selección de la mejor respuesta",$A21="Subítem de caso o problema"),TRIM($I21)&lt;&gt;"",NOT(OR(LEFT(TRIM($I21),1)="A",LEFT(TRIM($I21),1)="B",LEFT(TRIM($I21),1)="C",LEFT(TRIM($I21),1)="D",LEFT(TRIM($I21),1)="E"))),IF(COUNTIF($Q21:$AG21,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4820,7 +4821,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L22" s="345" t="str">
-        <x:f>IF(TRIM($A22)="","",IF(COUNTIF($Q22:$AJ22,"?*")=0,"OK","Falta revisar: "&amp;$Q22&amp;$R22&amp;$S22&amp;$T22&amp;$U22&amp;$V22&amp;$W22&amp;$X22&amp;$Y22&amp;$Z22&amp;$AA22&amp;$AB22&amp;$AC22&amp;$AD22&amp;$AE22&amp;$AF22&amp;$AG22&amp;$AH22&amp;$AI22&amp;$AJ22))</x:f>
+        <x:f>IF(TRIM($A22)="","",IF(OR($A22="Selección de la mejor respuesta",$A22="SELECCION_MEJOR_RESPUESTA",$A22="Subítem de caso o problema",$A22="SUBITEM_CASO"),IF(TRIM($C22)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D22:$H22&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I22)&lt;&gt;"",OR(LEFT(TRIM($I22),1)="A",LEFT(TRIM($I22),1)="B",LEFT(TRIM($I22),1)="C",LEFT(TRIM($I22),1)="D",LEFT(TRIM($I22),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A22)="","",IF(COUNTIF($Q22:$AJ22,"?*")=0,"OK","Falta revisar: "&amp;$Q22&amp;$R22&amp;$S22&amp;$T22&amp;$U22&amp;$V22&amp;$W22&amp;$X22&amp;$Y22&amp;$Z22&amp;$AA22&amp;$AB22&amp;$AC22&amp;$AD22&amp;$AE22&amp;$AF22&amp;$AG22&amp;$AH22&amp;$AI22&amp;$AJ22))))</x:f>
       </x:c>
       <x:c r="M22" s="341"/>
       <x:c r="N22"/>
@@ -4876,7 +4877,7 @@
         <x:f>IF(AND($A22="Verdadero o Falso Complejas",TRIM($I22)&lt;&gt;"",NOT(OR(LEFT(TRIM($I22),1)="A",LEFT(TRIM($I22),1)="B",LEFT(TRIM($I22),1)="C",LEFT(TRIM($I22),1)="D",LEFT(TRIM($I22),1)="E"))),IF(COUNTIF($Q22:$AE22,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG22" t="str">
-        <x:f>IF(AND(OR($A22="Selección de la mejor respuesta",$A22="Subítem de caso o problema"),COUNTIF($D22:$H22,"?*")&lt;5),IF(COUNTIF($Q22:$AF22,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A22="Selección de la mejor respuesta",$A22="Subítem de caso o problema"),COUNTA($D22:$H22)&lt;5),IF(COUNTIF($Q22:$AF22,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH22" t="str">
         <x:f>IF(AND(OR($A22="Selección de la mejor respuesta",$A22="Subítem de caso o problema"),TRIM($I22)&lt;&gt;"",NOT(OR(LEFT(TRIM($I22),1)="A",LEFT(TRIM($I22),1)="B",LEFT(TRIM($I22),1)="C",LEFT(TRIM($I22),1)="D",LEFT(TRIM($I22),1)="E"))),IF(COUNTIF($Q22:$AG22,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -4927,7 +4928,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L23" s="345" t="str">
-        <x:f>IF(TRIM($A23)="","",IF(COUNTIF($Q23:$AJ23,"?*")=0,"OK","Falta revisar: "&amp;$Q23&amp;$R23&amp;$S23&amp;$T23&amp;$U23&amp;$V23&amp;$W23&amp;$X23&amp;$Y23&amp;$Z23&amp;$AA23&amp;$AB23&amp;$AC23&amp;$AD23&amp;$AE23&amp;$AF23&amp;$AG23&amp;$AH23&amp;$AI23&amp;$AJ23))</x:f>
+        <x:f>IF(TRIM($A23)="","",IF(OR($A23="Selección de la mejor respuesta",$A23="SELECCION_MEJOR_RESPUESTA",$A23="Subítem de caso o problema",$A23="SUBITEM_CASO"),IF(TRIM($C23)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D23:$H23&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I23)&lt;&gt;"",OR(LEFT(TRIM($I23),1)="A",LEFT(TRIM($I23),1)="B",LEFT(TRIM($I23),1)="C",LEFT(TRIM($I23),1)="D",LEFT(TRIM($I23),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A23)="","",IF(COUNTIF($Q23:$AJ23,"?*")=0,"OK","Falta revisar: "&amp;$Q23&amp;$R23&amp;$S23&amp;$T23&amp;$U23&amp;$V23&amp;$W23&amp;$X23&amp;$Y23&amp;$Z23&amp;$AA23&amp;$AB23&amp;$AC23&amp;$AD23&amp;$AE23&amp;$AF23&amp;$AG23&amp;$AH23&amp;$AI23&amp;$AJ23))))</x:f>
       </x:c>
       <x:c r="M23" s="341"/>
       <x:c r="N23"/>
@@ -4983,7 +4984,7 @@
         <x:f>IF(AND($A23="Verdadero o Falso Complejas",TRIM($I23)&lt;&gt;"",NOT(OR(LEFT(TRIM($I23),1)="A",LEFT(TRIM($I23),1)="B",LEFT(TRIM($I23),1)="C",LEFT(TRIM($I23),1)="D",LEFT(TRIM($I23),1)="E"))),IF(COUNTIF($Q23:$AE23,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG23" t="str">
-        <x:f>IF(AND(OR($A23="Selección de la mejor respuesta",$A23="Subítem de caso o problema"),COUNTIF($D23:$H23,"?*")&lt;5),IF(COUNTIF($Q23:$AF23,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A23="Selección de la mejor respuesta",$A23="Subítem de caso o problema"),COUNTA($D23:$H23)&lt;5),IF(COUNTIF($Q23:$AF23,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH23" t="str">
         <x:f>IF(AND(OR($A23="Selección de la mejor respuesta",$A23="Subítem de caso o problema"),TRIM($I23)&lt;&gt;"",NOT(OR(LEFT(TRIM($I23),1)="A",LEFT(TRIM($I23),1)="B",LEFT(TRIM($I23),1)="C",LEFT(TRIM($I23),1)="D",LEFT(TRIM($I23),1)="E"))),IF(COUNTIF($Q23:$AG23,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5034,7 +5035,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L24" s="345" t="str">
-        <x:f>IF(TRIM($A24)="","",IF(COUNTIF($Q24:$AJ24,"?*")=0,"OK","Falta revisar: "&amp;$Q24&amp;$R24&amp;$S24&amp;$T24&amp;$U24&amp;$V24&amp;$W24&amp;$X24&amp;$Y24&amp;$Z24&amp;$AA24&amp;$AB24&amp;$AC24&amp;$AD24&amp;$AE24&amp;$AF24&amp;$AG24&amp;$AH24&amp;$AI24&amp;$AJ24))</x:f>
+        <x:f>IF(TRIM($A24)="","",IF(OR($A24="Selección de la mejor respuesta",$A24="SELECCION_MEJOR_RESPUESTA",$A24="Subítem de caso o problema",$A24="SUBITEM_CASO"),IF(TRIM($C24)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D24:$H24&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I24)&lt;&gt;"",OR(LEFT(TRIM($I24),1)="A",LEFT(TRIM($I24),1)="B",LEFT(TRIM($I24),1)="C",LEFT(TRIM($I24),1)="D",LEFT(TRIM($I24),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A24)="","",IF(COUNTIF($Q24:$AJ24,"?*")=0,"OK","Falta revisar: "&amp;$Q24&amp;$R24&amp;$S24&amp;$T24&amp;$U24&amp;$V24&amp;$W24&amp;$X24&amp;$Y24&amp;$Z24&amp;$AA24&amp;$AB24&amp;$AC24&amp;$AD24&amp;$AE24&amp;$AF24&amp;$AG24&amp;$AH24&amp;$AI24&amp;$AJ24))))</x:f>
       </x:c>
       <x:c r="M24" s="341"/>
       <x:c r="N24"/>
@@ -5090,7 +5091,7 @@
         <x:f>IF(AND($A24="Verdadero o Falso Complejas",TRIM($I24)&lt;&gt;"",NOT(OR(LEFT(TRIM($I24),1)="A",LEFT(TRIM($I24),1)="B",LEFT(TRIM($I24),1)="C",LEFT(TRIM($I24),1)="D",LEFT(TRIM($I24),1)="E"))),IF(COUNTIF($Q24:$AE24,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG24" t="str">
-        <x:f>IF(AND(OR($A24="Selección de la mejor respuesta",$A24="Subítem de caso o problema"),COUNTIF($D24:$H24,"?*")&lt;5),IF(COUNTIF($Q24:$AF24,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A24="Selección de la mejor respuesta",$A24="Subítem de caso o problema"),COUNTA($D24:$H24)&lt;5),IF(COUNTIF($Q24:$AF24,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH24" t="str">
         <x:f>IF(AND(OR($A24="Selección de la mejor respuesta",$A24="Subítem de caso o problema"),TRIM($I24)&lt;&gt;"",NOT(OR(LEFT(TRIM($I24),1)="A",LEFT(TRIM($I24),1)="B",LEFT(TRIM($I24),1)="C",LEFT(TRIM($I24),1)="D",LEFT(TRIM($I24),1)="E"))),IF(COUNTIF($Q24:$AG24,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5141,7 +5142,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L25" s="345" t="str">
-        <x:f>IF(TRIM($A25)="","",IF(COUNTIF($Q25:$AJ25,"?*")=0,"OK","Falta revisar: "&amp;$Q25&amp;$R25&amp;$S25&amp;$T25&amp;$U25&amp;$V25&amp;$W25&amp;$X25&amp;$Y25&amp;$Z25&amp;$AA25&amp;$AB25&amp;$AC25&amp;$AD25&amp;$AE25&amp;$AF25&amp;$AG25&amp;$AH25&amp;$AI25&amp;$AJ25))</x:f>
+        <x:f>IF(TRIM($A25)="","",IF(OR($A25="Selección de la mejor respuesta",$A25="SELECCION_MEJOR_RESPUESTA",$A25="Subítem de caso o problema",$A25="SUBITEM_CASO"),IF(TRIM($C25)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D25:$H25&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I25)&lt;&gt;"",OR(LEFT(TRIM($I25),1)="A",LEFT(TRIM($I25),1)="B",LEFT(TRIM($I25),1)="C",LEFT(TRIM($I25),1)="D",LEFT(TRIM($I25),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A25)="","",IF(COUNTIF($Q25:$AJ25,"?*")=0,"OK","Falta revisar: "&amp;$Q25&amp;$R25&amp;$S25&amp;$T25&amp;$U25&amp;$V25&amp;$W25&amp;$X25&amp;$Y25&amp;$Z25&amp;$AA25&amp;$AB25&amp;$AC25&amp;$AD25&amp;$AE25&amp;$AF25&amp;$AG25&amp;$AH25&amp;$AI25&amp;$AJ25))))</x:f>
       </x:c>
       <x:c r="M25" s="341"/>
       <x:c r="N25"/>
@@ -5197,7 +5198,7 @@
         <x:f>IF(AND($A25="Verdadero o Falso Complejas",TRIM($I25)&lt;&gt;"",NOT(OR(LEFT(TRIM($I25),1)="A",LEFT(TRIM($I25),1)="B",LEFT(TRIM($I25),1)="C",LEFT(TRIM($I25),1)="D",LEFT(TRIM($I25),1)="E"))),IF(COUNTIF($Q25:$AE25,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG25" t="str">
-        <x:f>IF(AND(OR($A25="Selección de la mejor respuesta",$A25="Subítem de caso o problema"),COUNTIF($D25:$H25,"?*")&lt;5),IF(COUNTIF($Q25:$AF25,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A25="Selección de la mejor respuesta",$A25="Subítem de caso o problema"),COUNTA($D25:$H25)&lt;5),IF(COUNTIF($Q25:$AF25,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH25" t="str">
         <x:f>IF(AND(OR($A25="Selección de la mejor respuesta",$A25="Subítem de caso o problema"),TRIM($I25)&lt;&gt;"",NOT(OR(LEFT(TRIM($I25),1)="A",LEFT(TRIM($I25),1)="B",LEFT(TRIM($I25),1)="C",LEFT(TRIM($I25),1)="D",LEFT(TRIM($I25),1)="E"))),IF(COUNTIF($Q25:$AG25,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5248,7 +5249,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L26" s="345" t="str">
-        <x:f>IF(TRIM($A26)="","",IF(COUNTIF($Q26:$AJ26,"?*")=0,"OK","Falta revisar: "&amp;$Q26&amp;$R26&amp;$S26&amp;$T26&amp;$U26&amp;$V26&amp;$W26&amp;$X26&amp;$Y26&amp;$Z26&amp;$AA26&amp;$AB26&amp;$AC26&amp;$AD26&amp;$AE26&amp;$AF26&amp;$AG26&amp;$AH26&amp;$AI26&amp;$AJ26))</x:f>
+        <x:f>IF(TRIM($A26)="","",IF(OR($A26="Selección de la mejor respuesta",$A26="SELECCION_MEJOR_RESPUESTA",$A26="Subítem de caso o problema",$A26="SUBITEM_CASO"),IF(TRIM($C26)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D26:$H26&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I26)&lt;&gt;"",OR(LEFT(TRIM($I26),1)="A",LEFT(TRIM($I26),1)="B",LEFT(TRIM($I26),1)="C",LEFT(TRIM($I26),1)="D",LEFT(TRIM($I26),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A26)="","",IF(COUNTIF($Q26:$AJ26,"?*")=0,"OK","Falta revisar: "&amp;$Q26&amp;$R26&amp;$S26&amp;$T26&amp;$U26&amp;$V26&amp;$W26&amp;$X26&amp;$Y26&amp;$Z26&amp;$AA26&amp;$AB26&amp;$AC26&amp;$AD26&amp;$AE26&amp;$AF26&amp;$AG26&amp;$AH26&amp;$AI26&amp;$AJ26))))</x:f>
       </x:c>
       <x:c r="M26" s="341"/>
       <x:c r="N26"/>
@@ -5304,7 +5305,7 @@
         <x:f>IF(AND($A26="Verdadero o Falso Complejas",TRIM($I26)&lt;&gt;"",NOT(OR(LEFT(TRIM($I26),1)="A",LEFT(TRIM($I26),1)="B",LEFT(TRIM($I26),1)="C",LEFT(TRIM($I26),1)="D",LEFT(TRIM($I26),1)="E"))),IF(COUNTIF($Q26:$AE26,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG26" t="str">
-        <x:f>IF(AND(OR($A26="Selección de la mejor respuesta",$A26="Subítem de caso o problema"),COUNTIF($D26:$H26,"?*")&lt;5),IF(COUNTIF($Q26:$AF26,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A26="Selección de la mejor respuesta",$A26="Subítem de caso o problema"),COUNTA($D26:$H26)&lt;5),IF(COUNTIF($Q26:$AF26,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH26" t="str">
         <x:f>IF(AND(OR($A26="Selección de la mejor respuesta",$A26="Subítem de caso o problema"),TRIM($I26)&lt;&gt;"",NOT(OR(LEFT(TRIM($I26),1)="A",LEFT(TRIM($I26),1)="B",LEFT(TRIM($I26),1)="C",LEFT(TRIM($I26),1)="D",LEFT(TRIM($I26),1)="E"))),IF(COUNTIF($Q26:$AG26,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5355,7 +5356,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L27" s="345" t="str">
-        <x:f>IF(TRIM($A27)="","",IF(COUNTIF($Q27:$AJ27,"?*")=0,"OK","Falta revisar: "&amp;$Q27&amp;$R27&amp;$S27&amp;$T27&amp;$U27&amp;$V27&amp;$W27&amp;$X27&amp;$Y27&amp;$Z27&amp;$AA27&amp;$AB27&amp;$AC27&amp;$AD27&amp;$AE27&amp;$AF27&amp;$AG27&amp;$AH27&amp;$AI27&amp;$AJ27))</x:f>
+        <x:f>IF(TRIM($A27)="","",IF(OR($A27="Selección de la mejor respuesta",$A27="SELECCION_MEJOR_RESPUESTA",$A27="Subítem de caso o problema",$A27="SUBITEM_CASO"),IF(TRIM($C27)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D27:$H27&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I27)&lt;&gt;"",OR(LEFT(TRIM($I27),1)="A",LEFT(TRIM($I27),1)="B",LEFT(TRIM($I27),1)="C",LEFT(TRIM($I27),1)="D",LEFT(TRIM($I27),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A27)="","",IF(COUNTIF($Q27:$AJ27,"?*")=0,"OK","Falta revisar: "&amp;$Q27&amp;$R27&amp;$S27&amp;$T27&amp;$U27&amp;$V27&amp;$W27&amp;$X27&amp;$Y27&amp;$Z27&amp;$AA27&amp;$AB27&amp;$AC27&amp;$AD27&amp;$AE27&amp;$AF27&amp;$AG27&amp;$AH27&amp;$AI27&amp;$AJ27))))</x:f>
       </x:c>
       <x:c r="M27" s="341"/>
       <x:c r="N27"/>
@@ -5411,7 +5412,7 @@
         <x:f>IF(AND($A27="Verdadero o Falso Complejas",TRIM($I27)&lt;&gt;"",NOT(OR(LEFT(TRIM($I27),1)="A",LEFT(TRIM($I27),1)="B",LEFT(TRIM($I27),1)="C",LEFT(TRIM($I27),1)="D",LEFT(TRIM($I27),1)="E"))),IF(COUNTIF($Q27:$AE27,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG27" t="str">
-        <x:f>IF(AND(OR($A27="Selección de la mejor respuesta",$A27="Subítem de caso o problema"),COUNTIF($D27:$H27,"?*")&lt;5),IF(COUNTIF($Q27:$AF27,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A27="Selección de la mejor respuesta",$A27="Subítem de caso o problema"),COUNTA($D27:$H27)&lt;5),IF(COUNTIF($Q27:$AF27,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH27" t="str">
         <x:f>IF(AND(OR($A27="Selección de la mejor respuesta",$A27="Subítem de caso o problema"),TRIM($I27)&lt;&gt;"",NOT(OR(LEFT(TRIM($I27),1)="A",LEFT(TRIM($I27),1)="B",LEFT(TRIM($I27),1)="C",LEFT(TRIM($I27),1)="D",LEFT(TRIM($I27),1)="E"))),IF(COUNTIF($Q27:$AG27,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5462,7 +5463,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L28" s="345" t="str">
-        <x:f>IF(TRIM($A28)="","",IF(COUNTIF($Q28:$AJ28,"?*")=0,"OK","Falta revisar: "&amp;$Q28&amp;$R28&amp;$S28&amp;$T28&amp;$U28&amp;$V28&amp;$W28&amp;$X28&amp;$Y28&amp;$Z28&amp;$AA28&amp;$AB28&amp;$AC28&amp;$AD28&amp;$AE28&amp;$AF28&amp;$AG28&amp;$AH28&amp;$AI28&amp;$AJ28))</x:f>
+        <x:f>IF(TRIM($A28)="","",IF(OR($A28="Selección de la mejor respuesta",$A28="SELECCION_MEJOR_RESPUESTA",$A28="Subítem de caso o problema",$A28="SUBITEM_CASO"),IF(TRIM($C28)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D28:$H28&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I28)&lt;&gt;"",OR(LEFT(TRIM($I28),1)="A",LEFT(TRIM($I28),1)="B",LEFT(TRIM($I28),1)="C",LEFT(TRIM($I28),1)="D",LEFT(TRIM($I28),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A28)="","",IF(COUNTIF($Q28:$AJ28,"?*")=0,"OK","Falta revisar: "&amp;$Q28&amp;$R28&amp;$S28&amp;$T28&amp;$U28&amp;$V28&amp;$W28&amp;$X28&amp;$Y28&amp;$Z28&amp;$AA28&amp;$AB28&amp;$AC28&amp;$AD28&amp;$AE28&amp;$AF28&amp;$AG28&amp;$AH28&amp;$AI28&amp;$AJ28))))</x:f>
       </x:c>
       <x:c r="M28" s="341"/>
       <x:c r="N28"/>
@@ -5518,7 +5519,7 @@
         <x:f>IF(AND($A28="Verdadero o Falso Complejas",TRIM($I28)&lt;&gt;"",NOT(OR(LEFT(TRIM($I28),1)="A",LEFT(TRIM($I28),1)="B",LEFT(TRIM($I28),1)="C",LEFT(TRIM($I28),1)="D",LEFT(TRIM($I28),1)="E"))),IF(COUNTIF($Q28:$AE28,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG28" t="str">
-        <x:f>IF(AND(OR($A28="Selección de la mejor respuesta",$A28="Subítem de caso o problema"),COUNTIF($D28:$H28,"?*")&lt;5),IF(COUNTIF($Q28:$AF28,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A28="Selección de la mejor respuesta",$A28="Subítem de caso o problema"),COUNTA($D28:$H28)&lt;5),IF(COUNTIF($Q28:$AF28,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH28" t="str">
         <x:f>IF(AND(OR($A28="Selección de la mejor respuesta",$A28="Subítem de caso o problema"),TRIM($I28)&lt;&gt;"",NOT(OR(LEFT(TRIM($I28),1)="A",LEFT(TRIM($I28),1)="B",LEFT(TRIM($I28),1)="C",LEFT(TRIM($I28),1)="D",LEFT(TRIM($I28),1)="E"))),IF(COUNTIF($Q28:$AG28,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5569,7 +5570,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L29" s="345" t="str">
-        <x:f>IF(TRIM($A29)="","",IF(COUNTIF($Q29:$AJ29,"?*")=0,"OK","Falta revisar: "&amp;$Q29&amp;$R29&amp;$S29&amp;$T29&amp;$U29&amp;$V29&amp;$W29&amp;$X29&amp;$Y29&amp;$Z29&amp;$AA29&amp;$AB29&amp;$AC29&amp;$AD29&amp;$AE29&amp;$AF29&amp;$AG29&amp;$AH29&amp;$AI29&amp;$AJ29))</x:f>
+        <x:f>IF(TRIM($A29)="","",IF(OR($A29="Selección de la mejor respuesta",$A29="SELECCION_MEJOR_RESPUESTA",$A29="Subítem de caso o problema",$A29="SUBITEM_CASO"),IF(TRIM($C29)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D29:$H29&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I29)&lt;&gt;"",OR(LEFT(TRIM($I29),1)="A",LEFT(TRIM($I29),1)="B",LEFT(TRIM($I29),1)="C",LEFT(TRIM($I29),1)="D",LEFT(TRIM($I29),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A29)="","",IF(COUNTIF($Q29:$AJ29,"?*")=0,"OK","Falta revisar: "&amp;$Q29&amp;$R29&amp;$S29&amp;$T29&amp;$U29&amp;$V29&amp;$W29&amp;$X29&amp;$Y29&amp;$Z29&amp;$AA29&amp;$AB29&amp;$AC29&amp;$AD29&amp;$AE29&amp;$AF29&amp;$AG29&amp;$AH29&amp;$AI29&amp;$AJ29))))</x:f>
       </x:c>
       <x:c r="M29" s="341"/>
       <x:c r="N29"/>
@@ -5625,7 +5626,7 @@
         <x:f>IF(AND($A29="Verdadero o Falso Complejas",TRIM($I29)&lt;&gt;"",NOT(OR(LEFT(TRIM($I29),1)="A",LEFT(TRIM($I29),1)="B",LEFT(TRIM($I29),1)="C",LEFT(TRIM($I29),1)="D",LEFT(TRIM($I29),1)="E"))),IF(COUNTIF($Q29:$AE29,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG29" t="str">
-        <x:f>IF(AND(OR($A29="Selección de la mejor respuesta",$A29="Subítem de caso o problema"),COUNTIF($D29:$H29,"?*")&lt;5),IF(COUNTIF($Q29:$AF29,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A29="Selección de la mejor respuesta",$A29="Subítem de caso o problema"),COUNTA($D29:$H29)&lt;5),IF(COUNTIF($Q29:$AF29,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH29" t="str">
         <x:f>IF(AND(OR($A29="Selección de la mejor respuesta",$A29="Subítem de caso o problema"),TRIM($I29)&lt;&gt;"",NOT(OR(LEFT(TRIM($I29),1)="A",LEFT(TRIM($I29),1)="B",LEFT(TRIM($I29),1)="C",LEFT(TRIM($I29),1)="D",LEFT(TRIM($I29),1)="E"))),IF(COUNTIF($Q29:$AG29,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5676,7 +5677,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L30" s="345" t="str">
-        <x:f>IF(TRIM($A30)="","",IF(COUNTIF($Q30:$AJ30,"?*")=0,"OK","Falta revisar: "&amp;$Q30&amp;$R30&amp;$S30&amp;$T30&amp;$U30&amp;$V30&amp;$W30&amp;$X30&amp;$Y30&amp;$Z30&amp;$AA30&amp;$AB30&amp;$AC30&amp;$AD30&amp;$AE30&amp;$AF30&amp;$AG30&amp;$AH30&amp;$AI30&amp;$AJ30))</x:f>
+        <x:f>IF(TRIM($A30)="","",IF(OR($A30="Selección de la mejor respuesta",$A30="SELECCION_MEJOR_RESPUESTA",$A30="Subítem de caso o problema",$A30="SUBITEM_CASO"),IF(TRIM($C30)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D30:$H30&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I30)&lt;&gt;"",OR(LEFT(TRIM($I30),1)="A",LEFT(TRIM($I30),1)="B",LEFT(TRIM($I30),1)="C",LEFT(TRIM($I30),1)="D",LEFT(TRIM($I30),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A30)="","",IF(COUNTIF($Q30:$AJ30,"?*")=0,"OK","Falta revisar: "&amp;$Q30&amp;$R30&amp;$S30&amp;$T30&amp;$U30&amp;$V30&amp;$W30&amp;$X30&amp;$Y30&amp;$Z30&amp;$AA30&amp;$AB30&amp;$AC30&amp;$AD30&amp;$AE30&amp;$AF30&amp;$AG30&amp;$AH30&amp;$AI30&amp;$AJ30))))</x:f>
       </x:c>
       <x:c r="M30" s="341"/>
       <x:c r="N30"/>
@@ -5732,7 +5733,7 @@
         <x:f>IF(AND($A30="Verdadero o Falso Complejas",TRIM($I30)&lt;&gt;"",NOT(OR(LEFT(TRIM($I30),1)="A",LEFT(TRIM($I30),1)="B",LEFT(TRIM($I30),1)="C",LEFT(TRIM($I30),1)="D",LEFT(TRIM($I30),1)="E"))),IF(COUNTIF($Q30:$AE30,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG30" t="str">
-        <x:f>IF(AND(OR($A30="Selección de la mejor respuesta",$A30="Subítem de caso o problema"),COUNTIF($D30:$H30,"?*")&lt;5),IF(COUNTIF($Q30:$AF30,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A30="Selección de la mejor respuesta",$A30="Subítem de caso o problema"),COUNTA($D30:$H30)&lt;5),IF(COUNTIF($Q30:$AF30,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH30" t="str">
         <x:f>IF(AND(OR($A30="Selección de la mejor respuesta",$A30="Subítem de caso o problema"),TRIM($I30)&lt;&gt;"",NOT(OR(LEFT(TRIM($I30),1)="A",LEFT(TRIM($I30),1)="B",LEFT(TRIM($I30),1)="C",LEFT(TRIM($I30),1)="D",LEFT(TRIM($I30),1)="E"))),IF(COUNTIF($Q30:$AG30,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5783,7 +5784,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L31" s="345" t="str">
-        <x:f>IF(TRIM($A31)="","",IF(COUNTIF($Q31:$AJ31,"?*")=0,"OK","Falta revisar: "&amp;$Q31&amp;$R31&amp;$S31&amp;$T31&amp;$U31&amp;$V31&amp;$W31&amp;$X31&amp;$Y31&amp;$Z31&amp;$AA31&amp;$AB31&amp;$AC31&amp;$AD31&amp;$AE31&amp;$AF31&amp;$AG31&amp;$AH31&amp;$AI31&amp;$AJ31))</x:f>
+        <x:f>IF(TRIM($A31)="","",IF(OR($A31="Selección de la mejor respuesta",$A31="SELECCION_MEJOR_RESPUESTA",$A31="Subítem de caso o problema",$A31="SUBITEM_CASO"),IF(TRIM($C31)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D31:$H31&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I31)&lt;&gt;"",OR(LEFT(TRIM($I31),1)="A",LEFT(TRIM($I31),1)="B",LEFT(TRIM($I31),1)="C",LEFT(TRIM($I31),1)="D",LEFT(TRIM($I31),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A31)="","",IF(COUNTIF($Q31:$AJ31,"?*")=0,"OK","Falta revisar: "&amp;$Q31&amp;$R31&amp;$S31&amp;$T31&amp;$U31&amp;$V31&amp;$W31&amp;$X31&amp;$Y31&amp;$Z31&amp;$AA31&amp;$AB31&amp;$AC31&amp;$AD31&amp;$AE31&amp;$AF31&amp;$AG31&amp;$AH31&amp;$AI31&amp;$AJ31))))</x:f>
       </x:c>
       <x:c r="M31" s="341"/>
       <x:c r="N31"/>
@@ -5839,7 +5840,7 @@
         <x:f>IF(AND($A31="Verdadero o Falso Complejas",TRIM($I31)&lt;&gt;"",NOT(OR(LEFT(TRIM($I31),1)="A",LEFT(TRIM($I31),1)="B",LEFT(TRIM($I31),1)="C",LEFT(TRIM($I31),1)="D",LEFT(TRIM($I31),1)="E"))),IF(COUNTIF($Q31:$AE31,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG31" t="str">
-        <x:f>IF(AND(OR($A31="Selección de la mejor respuesta",$A31="Subítem de caso o problema"),COUNTIF($D31:$H31,"?*")&lt;5),IF(COUNTIF($Q31:$AF31,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A31="Selección de la mejor respuesta",$A31="Subítem de caso o problema"),COUNTA($D31:$H31)&lt;5),IF(COUNTIF($Q31:$AF31,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH31" t="str">
         <x:f>IF(AND(OR($A31="Selección de la mejor respuesta",$A31="Subítem de caso o problema"),TRIM($I31)&lt;&gt;"",NOT(OR(LEFT(TRIM($I31),1)="A",LEFT(TRIM($I31),1)="B",LEFT(TRIM($I31),1)="C",LEFT(TRIM($I31),1)="D",LEFT(TRIM($I31),1)="E"))),IF(COUNTIF($Q31:$AG31,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5890,7 +5891,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L32" s="345" t="str">
-        <x:f>IF(TRIM($A32)="","",IF(COUNTIF($Q32:$AJ32,"?*")=0,"OK","Falta revisar: "&amp;$Q32&amp;$R32&amp;$S32&amp;$T32&amp;$U32&amp;$V32&amp;$W32&amp;$X32&amp;$Y32&amp;$Z32&amp;$AA32&amp;$AB32&amp;$AC32&amp;$AD32&amp;$AE32&amp;$AF32&amp;$AG32&amp;$AH32&amp;$AI32&amp;$AJ32))</x:f>
+        <x:f>IF(TRIM($A32)="","",IF(OR($A32="Selección de la mejor respuesta",$A32="SELECCION_MEJOR_RESPUESTA",$A32="Subítem de caso o problema",$A32="SUBITEM_CASO"),IF(TRIM($C32)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D32:$H32&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I32)&lt;&gt;"",OR(LEFT(TRIM($I32),1)="A",LEFT(TRIM($I32),1)="B",LEFT(TRIM($I32),1)="C",LEFT(TRIM($I32),1)="D",LEFT(TRIM($I32),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A32)="","",IF(COUNTIF($Q32:$AJ32,"?*")=0,"OK","Falta revisar: "&amp;$Q32&amp;$R32&amp;$S32&amp;$T32&amp;$U32&amp;$V32&amp;$W32&amp;$X32&amp;$Y32&amp;$Z32&amp;$AA32&amp;$AB32&amp;$AC32&amp;$AD32&amp;$AE32&amp;$AF32&amp;$AG32&amp;$AH32&amp;$AI32&amp;$AJ32))))</x:f>
       </x:c>
       <x:c r="M32" s="341"/>
       <x:c r="N32"/>
@@ -5946,7 +5947,7 @@
         <x:f>IF(AND($A32="Verdadero o Falso Complejas",TRIM($I32)&lt;&gt;"",NOT(OR(LEFT(TRIM($I32),1)="A",LEFT(TRIM($I32),1)="B",LEFT(TRIM($I32),1)="C",LEFT(TRIM($I32),1)="D",LEFT(TRIM($I32),1)="E"))),IF(COUNTIF($Q32:$AE32,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG32" t="str">
-        <x:f>IF(AND(OR($A32="Selección de la mejor respuesta",$A32="Subítem de caso o problema"),COUNTIF($D32:$H32,"?*")&lt;5),IF(COUNTIF($Q32:$AF32,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A32="Selección de la mejor respuesta",$A32="Subítem de caso o problema"),COUNTA($D32:$H32)&lt;5),IF(COUNTIF($Q32:$AF32,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH32" t="str">
         <x:f>IF(AND(OR($A32="Selección de la mejor respuesta",$A32="Subítem de caso o problema"),TRIM($I32)&lt;&gt;"",NOT(OR(LEFT(TRIM($I32),1)="A",LEFT(TRIM($I32),1)="B",LEFT(TRIM($I32),1)="C",LEFT(TRIM($I32),1)="D",LEFT(TRIM($I32),1)="E"))),IF(COUNTIF($Q32:$AG32,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -5997,7 +5998,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L33" s="345" t="str">
-        <x:f>IF(TRIM($A33)="","",IF(COUNTIF($Q33:$AJ33,"?*")=0,"OK","Falta revisar: "&amp;$Q33&amp;$R33&amp;$S33&amp;$T33&amp;$U33&amp;$V33&amp;$W33&amp;$X33&amp;$Y33&amp;$Z33&amp;$AA33&amp;$AB33&amp;$AC33&amp;$AD33&amp;$AE33&amp;$AF33&amp;$AG33&amp;$AH33&amp;$AI33&amp;$AJ33))</x:f>
+        <x:f>IF(TRIM($A33)="","",IF(OR($A33="Selección de la mejor respuesta",$A33="SELECCION_MEJOR_RESPUESTA",$A33="Subítem de caso o problema",$A33="SUBITEM_CASO"),IF(TRIM($C33)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D33:$H33&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I33)&lt;&gt;"",OR(LEFT(TRIM($I33),1)="A",LEFT(TRIM($I33),1)="B",LEFT(TRIM($I33),1)="C",LEFT(TRIM($I33),1)="D",LEFT(TRIM($I33),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A33)="","",IF(COUNTIF($Q33:$AJ33,"?*")=0,"OK","Falta revisar: "&amp;$Q33&amp;$R33&amp;$S33&amp;$T33&amp;$U33&amp;$V33&amp;$W33&amp;$X33&amp;$Y33&amp;$Z33&amp;$AA33&amp;$AB33&amp;$AC33&amp;$AD33&amp;$AE33&amp;$AF33&amp;$AG33&amp;$AH33&amp;$AI33&amp;$AJ33))))</x:f>
       </x:c>
       <x:c r="M33" s="341"/>
       <x:c r="N33"/>
@@ -6053,7 +6054,7 @@
         <x:f>IF(AND($A33="Verdadero o Falso Complejas",TRIM($I33)&lt;&gt;"",NOT(OR(LEFT(TRIM($I33),1)="A",LEFT(TRIM($I33),1)="B",LEFT(TRIM($I33),1)="C",LEFT(TRIM($I33),1)="D",LEFT(TRIM($I33),1)="E"))),IF(COUNTIF($Q33:$AE33,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG33" t="str">
-        <x:f>IF(AND(OR($A33="Selección de la mejor respuesta",$A33="Subítem de caso o problema"),COUNTIF($D33:$H33,"?*")&lt;5),IF(COUNTIF($Q33:$AF33,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A33="Selección de la mejor respuesta",$A33="Subítem de caso o problema"),COUNTA($D33:$H33)&lt;5),IF(COUNTIF($Q33:$AF33,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH33" t="str">
         <x:f>IF(AND(OR($A33="Selección de la mejor respuesta",$A33="Subítem de caso o problema"),TRIM($I33)&lt;&gt;"",NOT(OR(LEFT(TRIM($I33),1)="A",LEFT(TRIM($I33),1)="B",LEFT(TRIM($I33),1)="C",LEFT(TRIM($I33),1)="D",LEFT(TRIM($I33),1)="E"))),IF(COUNTIF($Q33:$AG33,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6104,7 +6105,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L34" s="345" t="str">
-        <x:f>IF(TRIM($A34)="","",IF(COUNTIF($Q34:$AJ34,"?*")=0,"OK","Falta revisar: "&amp;$Q34&amp;$R34&amp;$S34&amp;$T34&amp;$U34&amp;$V34&amp;$W34&amp;$X34&amp;$Y34&amp;$Z34&amp;$AA34&amp;$AB34&amp;$AC34&amp;$AD34&amp;$AE34&amp;$AF34&amp;$AG34&amp;$AH34&amp;$AI34&amp;$AJ34))</x:f>
+        <x:f>IF(TRIM($A34)="","",IF(OR($A34="Selección de la mejor respuesta",$A34="SELECCION_MEJOR_RESPUESTA",$A34="Subítem de caso o problema",$A34="SUBITEM_CASO"),IF(TRIM($C34)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D34:$H34&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I34)&lt;&gt;"",OR(LEFT(TRIM($I34),1)="A",LEFT(TRIM($I34),1)="B",LEFT(TRIM($I34),1)="C",LEFT(TRIM($I34),1)="D",LEFT(TRIM($I34),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A34)="","",IF(COUNTIF($Q34:$AJ34,"?*")=0,"OK","Falta revisar: "&amp;$Q34&amp;$R34&amp;$S34&amp;$T34&amp;$U34&amp;$V34&amp;$W34&amp;$X34&amp;$Y34&amp;$Z34&amp;$AA34&amp;$AB34&amp;$AC34&amp;$AD34&amp;$AE34&amp;$AF34&amp;$AG34&amp;$AH34&amp;$AI34&amp;$AJ34))))</x:f>
       </x:c>
       <x:c r="M34" s="341"/>
       <x:c r="N34"/>
@@ -6160,7 +6161,7 @@
         <x:f>IF(AND($A34="Verdadero o Falso Complejas",TRIM($I34)&lt;&gt;"",NOT(OR(LEFT(TRIM($I34),1)="A",LEFT(TRIM($I34),1)="B",LEFT(TRIM($I34),1)="C",LEFT(TRIM($I34),1)="D",LEFT(TRIM($I34),1)="E"))),IF(COUNTIF($Q34:$AE34,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG34" t="str">
-        <x:f>IF(AND(OR($A34="Selección de la mejor respuesta",$A34="Subítem de caso o problema"),COUNTIF($D34:$H34,"?*")&lt;5),IF(COUNTIF($Q34:$AF34,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A34="Selección de la mejor respuesta",$A34="Subítem de caso o problema"),COUNTA($D34:$H34)&lt;5),IF(COUNTIF($Q34:$AF34,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH34" t="str">
         <x:f>IF(AND(OR($A34="Selección de la mejor respuesta",$A34="Subítem de caso o problema"),TRIM($I34)&lt;&gt;"",NOT(OR(LEFT(TRIM($I34),1)="A",LEFT(TRIM($I34),1)="B",LEFT(TRIM($I34),1)="C",LEFT(TRIM($I34),1)="D",LEFT(TRIM($I34),1)="E"))),IF(COUNTIF($Q34:$AG34,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6211,7 +6212,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L35" s="345" t="str">
-        <x:f>IF(TRIM($A35)="","",IF(COUNTIF($Q35:$AJ35,"?*")=0,"OK","Falta revisar: "&amp;$Q35&amp;$R35&amp;$S35&amp;$T35&amp;$U35&amp;$V35&amp;$W35&amp;$X35&amp;$Y35&amp;$Z35&amp;$AA35&amp;$AB35&amp;$AC35&amp;$AD35&amp;$AE35&amp;$AF35&amp;$AG35&amp;$AH35&amp;$AI35&amp;$AJ35))</x:f>
+        <x:f>IF(TRIM($A35)="","",IF(OR($A35="Selección de la mejor respuesta",$A35="SELECCION_MEJOR_RESPUESTA",$A35="Subítem de caso o problema",$A35="SUBITEM_CASO"),IF(TRIM($C35)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D35:$H35&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I35)&lt;&gt;"",OR(LEFT(TRIM($I35),1)="A",LEFT(TRIM($I35),1)="B",LEFT(TRIM($I35),1)="C",LEFT(TRIM($I35),1)="D",LEFT(TRIM($I35),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A35)="","",IF(COUNTIF($Q35:$AJ35,"?*")=0,"OK","Falta revisar: "&amp;$Q35&amp;$R35&amp;$S35&amp;$T35&amp;$U35&amp;$V35&amp;$W35&amp;$X35&amp;$Y35&amp;$Z35&amp;$AA35&amp;$AB35&amp;$AC35&amp;$AD35&amp;$AE35&amp;$AF35&amp;$AG35&amp;$AH35&amp;$AI35&amp;$AJ35))))</x:f>
       </x:c>
       <x:c r="M35" s="341"/>
       <x:c r="N35"/>
@@ -6267,7 +6268,7 @@
         <x:f>IF(AND($A35="Verdadero o Falso Complejas",TRIM($I35)&lt;&gt;"",NOT(OR(LEFT(TRIM($I35),1)="A",LEFT(TRIM($I35),1)="B",LEFT(TRIM($I35),1)="C",LEFT(TRIM($I35),1)="D",LEFT(TRIM($I35),1)="E"))),IF(COUNTIF($Q35:$AE35,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG35" t="str">
-        <x:f>IF(AND(OR($A35="Selección de la mejor respuesta",$A35="Subítem de caso o problema"),COUNTIF($D35:$H35,"?*")&lt;5),IF(COUNTIF($Q35:$AF35,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A35="Selección de la mejor respuesta",$A35="Subítem de caso o problema"),COUNTA($D35:$H35)&lt;5),IF(COUNTIF($Q35:$AF35,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH35" t="str">
         <x:f>IF(AND(OR($A35="Selección de la mejor respuesta",$A35="Subítem de caso o problema"),TRIM($I35)&lt;&gt;"",NOT(OR(LEFT(TRIM($I35),1)="A",LEFT(TRIM($I35),1)="B",LEFT(TRIM($I35),1)="C",LEFT(TRIM($I35),1)="D",LEFT(TRIM($I35),1)="E"))),IF(COUNTIF($Q35:$AG35,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6318,7 +6319,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L36" s="345" t="str">
-        <x:f>IF(TRIM($A36)="","",IF(COUNTIF($Q36:$AJ36,"?*")=0,"OK","Falta revisar: "&amp;$Q36&amp;$R36&amp;$S36&amp;$T36&amp;$U36&amp;$V36&amp;$W36&amp;$X36&amp;$Y36&amp;$Z36&amp;$AA36&amp;$AB36&amp;$AC36&amp;$AD36&amp;$AE36&amp;$AF36&amp;$AG36&amp;$AH36&amp;$AI36&amp;$AJ36))</x:f>
+        <x:f>IF(TRIM($A36)="","",IF(OR($A36="Selección de la mejor respuesta",$A36="SELECCION_MEJOR_RESPUESTA",$A36="Subítem de caso o problema",$A36="SUBITEM_CASO"),IF(TRIM($C36)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D36:$H36&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I36)&lt;&gt;"",OR(LEFT(TRIM($I36),1)="A",LEFT(TRIM($I36),1)="B",LEFT(TRIM($I36),1)="C",LEFT(TRIM($I36),1)="D",LEFT(TRIM($I36),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A36)="","",IF(COUNTIF($Q36:$AJ36,"?*")=0,"OK","Falta revisar: "&amp;$Q36&amp;$R36&amp;$S36&amp;$T36&amp;$U36&amp;$V36&amp;$W36&amp;$X36&amp;$Y36&amp;$Z36&amp;$AA36&amp;$AB36&amp;$AC36&amp;$AD36&amp;$AE36&amp;$AF36&amp;$AG36&amp;$AH36&amp;$AI36&amp;$AJ36))))</x:f>
       </x:c>
       <x:c r="M36" s="341"/>
       <x:c r="N36"/>
@@ -6374,7 +6375,7 @@
         <x:f>IF(AND($A36="Verdadero o Falso Complejas",TRIM($I36)&lt;&gt;"",NOT(OR(LEFT(TRIM($I36),1)="A",LEFT(TRIM($I36),1)="B",LEFT(TRIM($I36),1)="C",LEFT(TRIM($I36),1)="D",LEFT(TRIM($I36),1)="E"))),IF(COUNTIF($Q36:$AE36,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG36" t="str">
-        <x:f>IF(AND(OR($A36="Selección de la mejor respuesta",$A36="Subítem de caso o problema"),COUNTIF($D36:$H36,"?*")&lt;5),IF(COUNTIF($Q36:$AF36,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A36="Selección de la mejor respuesta",$A36="Subítem de caso o problema"),COUNTA($D36:$H36)&lt;5),IF(COUNTIF($Q36:$AF36,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH36" t="str">
         <x:f>IF(AND(OR($A36="Selección de la mejor respuesta",$A36="Subítem de caso o problema"),TRIM($I36)&lt;&gt;"",NOT(OR(LEFT(TRIM($I36),1)="A",LEFT(TRIM($I36),1)="B",LEFT(TRIM($I36),1)="C",LEFT(TRIM($I36),1)="D",LEFT(TRIM($I36),1)="E"))),IF(COUNTIF($Q36:$AG36,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6425,7 +6426,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L37" s="345" t="str">
-        <x:f>IF(TRIM($A37)="","",IF(COUNTIF($Q37:$AJ37,"?*")=0,"OK","Falta revisar: "&amp;$Q37&amp;$R37&amp;$S37&amp;$T37&amp;$U37&amp;$V37&amp;$W37&amp;$X37&amp;$Y37&amp;$Z37&amp;$AA37&amp;$AB37&amp;$AC37&amp;$AD37&amp;$AE37&amp;$AF37&amp;$AG37&amp;$AH37&amp;$AI37&amp;$AJ37))</x:f>
+        <x:f>IF(TRIM($A37)="","",IF(OR($A37="Selección de la mejor respuesta",$A37="SELECCION_MEJOR_RESPUESTA",$A37="Subítem de caso o problema",$A37="SUBITEM_CASO"),IF(TRIM($C37)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D37:$H37&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I37)&lt;&gt;"",OR(LEFT(TRIM($I37),1)="A",LEFT(TRIM($I37),1)="B",LEFT(TRIM($I37),1)="C",LEFT(TRIM($I37),1)="D",LEFT(TRIM($I37),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A37)="","",IF(COUNTIF($Q37:$AJ37,"?*")=0,"OK","Falta revisar: "&amp;$Q37&amp;$R37&amp;$S37&amp;$T37&amp;$U37&amp;$V37&amp;$W37&amp;$X37&amp;$Y37&amp;$Z37&amp;$AA37&amp;$AB37&amp;$AC37&amp;$AD37&amp;$AE37&amp;$AF37&amp;$AG37&amp;$AH37&amp;$AI37&amp;$AJ37))))</x:f>
       </x:c>
       <x:c r="M37" s="341"/>
       <x:c r="N37"/>
@@ -6481,7 +6482,7 @@
         <x:f>IF(AND($A37="Verdadero o Falso Complejas",TRIM($I37)&lt;&gt;"",NOT(OR(LEFT(TRIM($I37),1)="A",LEFT(TRIM($I37),1)="B",LEFT(TRIM($I37),1)="C",LEFT(TRIM($I37),1)="D",LEFT(TRIM($I37),1)="E"))),IF(COUNTIF($Q37:$AE37,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG37" t="str">
-        <x:f>IF(AND(OR($A37="Selección de la mejor respuesta",$A37="Subítem de caso o problema"),COUNTIF($D37:$H37,"?*")&lt;5),IF(COUNTIF($Q37:$AF37,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A37="Selección de la mejor respuesta",$A37="Subítem de caso o problema"),COUNTA($D37:$H37)&lt;5),IF(COUNTIF($Q37:$AF37,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH37" t="str">
         <x:f>IF(AND(OR($A37="Selección de la mejor respuesta",$A37="Subítem de caso o problema"),TRIM($I37)&lt;&gt;"",NOT(OR(LEFT(TRIM($I37),1)="A",LEFT(TRIM($I37),1)="B",LEFT(TRIM($I37),1)="C",LEFT(TRIM($I37),1)="D",LEFT(TRIM($I37),1)="E"))),IF(COUNTIF($Q37:$AG37,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6532,7 +6533,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L38" s="345" t="str">
-        <x:f>IF(TRIM($A38)="","",IF(COUNTIF($Q38:$AJ38,"?*")=0,"OK","Falta revisar: "&amp;$Q38&amp;$R38&amp;$S38&amp;$T38&amp;$U38&amp;$V38&amp;$W38&amp;$X38&amp;$Y38&amp;$Z38&amp;$AA38&amp;$AB38&amp;$AC38&amp;$AD38&amp;$AE38&amp;$AF38&amp;$AG38&amp;$AH38&amp;$AI38&amp;$AJ38))</x:f>
+        <x:f>IF(TRIM($A38)="","",IF(OR($A38="Selección de la mejor respuesta",$A38="SELECCION_MEJOR_RESPUESTA",$A38="Subítem de caso o problema",$A38="SUBITEM_CASO"),IF(TRIM($C38)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D38:$H38&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I38)&lt;&gt;"",OR(LEFT(TRIM($I38),1)="A",LEFT(TRIM($I38),1)="B",LEFT(TRIM($I38),1)="C",LEFT(TRIM($I38),1)="D",LEFT(TRIM($I38),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A38)="","",IF(COUNTIF($Q38:$AJ38,"?*")=0,"OK","Falta revisar: "&amp;$Q38&amp;$R38&amp;$S38&amp;$T38&amp;$U38&amp;$V38&amp;$W38&amp;$X38&amp;$Y38&amp;$Z38&amp;$AA38&amp;$AB38&amp;$AC38&amp;$AD38&amp;$AE38&amp;$AF38&amp;$AG38&amp;$AH38&amp;$AI38&amp;$AJ38))))</x:f>
       </x:c>
       <x:c r="M38" s="341"/>
       <x:c r="N38"/>
@@ -6588,7 +6589,7 @@
         <x:f>IF(AND($A38="Verdadero o Falso Complejas",TRIM($I38)&lt;&gt;"",NOT(OR(LEFT(TRIM($I38),1)="A",LEFT(TRIM($I38),1)="B",LEFT(TRIM($I38),1)="C",LEFT(TRIM($I38),1)="D",LEFT(TRIM($I38),1)="E"))),IF(COUNTIF($Q38:$AE38,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG38" t="str">
-        <x:f>IF(AND(OR($A38="Selección de la mejor respuesta",$A38="Subítem de caso o problema"),COUNTIF($D38:$H38,"?*")&lt;5),IF(COUNTIF($Q38:$AF38,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A38="Selección de la mejor respuesta",$A38="Subítem de caso o problema"),COUNTA($D38:$H38)&lt;5),IF(COUNTIF($Q38:$AF38,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH38" t="str">
         <x:f>IF(AND(OR($A38="Selección de la mejor respuesta",$A38="Subítem de caso o problema"),TRIM($I38)&lt;&gt;"",NOT(OR(LEFT(TRIM($I38),1)="A",LEFT(TRIM($I38),1)="B",LEFT(TRIM($I38),1)="C",LEFT(TRIM($I38),1)="D",LEFT(TRIM($I38),1)="E"))),IF(COUNTIF($Q38:$AG38,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6639,7 +6640,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L39" s="345" t="str">
-        <x:f>IF(TRIM($A39)="","",IF(COUNTIF($Q39:$AJ39,"?*")=0,"OK","Falta revisar: "&amp;$Q39&amp;$R39&amp;$S39&amp;$T39&amp;$U39&amp;$V39&amp;$W39&amp;$X39&amp;$Y39&amp;$Z39&amp;$AA39&amp;$AB39&amp;$AC39&amp;$AD39&amp;$AE39&amp;$AF39&amp;$AG39&amp;$AH39&amp;$AI39&amp;$AJ39))</x:f>
+        <x:f>IF(TRIM($A39)="","",IF(OR($A39="Selección de la mejor respuesta",$A39="SELECCION_MEJOR_RESPUESTA",$A39="Subítem de caso o problema",$A39="SUBITEM_CASO"),IF(TRIM($C39)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D39:$H39&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I39)&lt;&gt;"",OR(LEFT(TRIM($I39),1)="A",LEFT(TRIM($I39),1)="B",LEFT(TRIM($I39),1)="C",LEFT(TRIM($I39),1)="D",LEFT(TRIM($I39),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A39)="","",IF(COUNTIF($Q39:$AJ39,"?*")=0,"OK","Falta revisar: "&amp;$Q39&amp;$R39&amp;$S39&amp;$T39&amp;$U39&amp;$V39&amp;$W39&amp;$X39&amp;$Y39&amp;$Z39&amp;$AA39&amp;$AB39&amp;$AC39&amp;$AD39&amp;$AE39&amp;$AF39&amp;$AG39&amp;$AH39&amp;$AI39&amp;$AJ39))))</x:f>
       </x:c>
       <x:c r="M39" s="341"/>
       <x:c r="N39"/>
@@ -6695,7 +6696,7 @@
         <x:f>IF(AND($A39="Verdadero o Falso Complejas",TRIM($I39)&lt;&gt;"",NOT(OR(LEFT(TRIM($I39),1)="A",LEFT(TRIM($I39),1)="B",LEFT(TRIM($I39),1)="C",LEFT(TRIM($I39),1)="D",LEFT(TRIM($I39),1)="E"))),IF(COUNTIF($Q39:$AE39,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG39" t="str">
-        <x:f>IF(AND(OR($A39="Selección de la mejor respuesta",$A39="Subítem de caso o problema"),COUNTIF($D39:$H39,"?*")&lt;5),IF(COUNTIF($Q39:$AF39,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A39="Selección de la mejor respuesta",$A39="Subítem de caso o problema"),COUNTA($D39:$H39)&lt;5),IF(COUNTIF($Q39:$AF39,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH39" t="str">
         <x:f>IF(AND(OR($A39="Selección de la mejor respuesta",$A39="Subítem de caso o problema"),TRIM($I39)&lt;&gt;"",NOT(OR(LEFT(TRIM($I39),1)="A",LEFT(TRIM($I39),1)="B",LEFT(TRIM($I39),1)="C",LEFT(TRIM($I39),1)="D",LEFT(TRIM($I39),1)="E"))),IF(COUNTIF($Q39:$AG39,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6746,7 +6747,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L40" s="345" t="str">
-        <x:f>IF(TRIM($A40)="","",IF(COUNTIF($Q40:$AJ40,"?*")=0,"OK","Falta revisar: "&amp;$Q40&amp;$R40&amp;$S40&amp;$T40&amp;$U40&amp;$V40&amp;$W40&amp;$X40&amp;$Y40&amp;$Z40&amp;$AA40&amp;$AB40&amp;$AC40&amp;$AD40&amp;$AE40&amp;$AF40&amp;$AG40&amp;$AH40&amp;$AI40&amp;$AJ40))</x:f>
+        <x:f>IF(TRIM($A40)="","",IF(OR($A40="Selección de la mejor respuesta",$A40="SELECCION_MEJOR_RESPUESTA",$A40="Subítem de caso o problema",$A40="SUBITEM_CASO"),IF(TRIM($C40)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D40:$H40&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I40)&lt;&gt;"",OR(LEFT(TRIM($I40),1)="A",LEFT(TRIM($I40),1)="B",LEFT(TRIM($I40),1)="C",LEFT(TRIM($I40),1)="D",LEFT(TRIM($I40),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A40)="","",IF(COUNTIF($Q40:$AJ40,"?*")=0,"OK","Falta revisar: "&amp;$Q40&amp;$R40&amp;$S40&amp;$T40&amp;$U40&amp;$V40&amp;$W40&amp;$X40&amp;$Y40&amp;$Z40&amp;$AA40&amp;$AB40&amp;$AC40&amp;$AD40&amp;$AE40&amp;$AF40&amp;$AG40&amp;$AH40&amp;$AI40&amp;$AJ40))))</x:f>
       </x:c>
       <x:c r="M40" s="341"/>
       <x:c r="N40"/>
@@ -6802,7 +6803,7 @@
         <x:f>IF(AND($A40="Verdadero o Falso Complejas",TRIM($I40)&lt;&gt;"",NOT(OR(LEFT(TRIM($I40),1)="A",LEFT(TRIM($I40),1)="B",LEFT(TRIM($I40),1)="C",LEFT(TRIM($I40),1)="D",LEFT(TRIM($I40),1)="E"))),IF(COUNTIF($Q40:$AE40,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG40" t="str">
-        <x:f>IF(AND(OR($A40="Selección de la mejor respuesta",$A40="Subítem de caso o problema"),COUNTIF($D40:$H40,"?*")&lt;5),IF(COUNTIF($Q40:$AF40,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A40="Selección de la mejor respuesta",$A40="Subítem de caso o problema"),COUNTA($D40:$H40)&lt;5),IF(COUNTIF($Q40:$AF40,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH40" t="str">
         <x:f>IF(AND(OR($A40="Selección de la mejor respuesta",$A40="Subítem de caso o problema"),TRIM($I40)&lt;&gt;"",NOT(OR(LEFT(TRIM($I40),1)="A",LEFT(TRIM($I40),1)="B",LEFT(TRIM($I40),1)="C",LEFT(TRIM($I40),1)="D",LEFT(TRIM($I40),1)="E"))),IF(COUNTIF($Q40:$AG40,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6853,7 +6854,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L41" s="345" t="str">
-        <x:f>IF(TRIM($A41)="","",IF(COUNTIF($Q41:$AJ41,"?*")=0,"OK","Falta revisar: "&amp;$Q41&amp;$R41&amp;$S41&amp;$T41&amp;$U41&amp;$V41&amp;$W41&amp;$X41&amp;$Y41&amp;$Z41&amp;$AA41&amp;$AB41&amp;$AC41&amp;$AD41&amp;$AE41&amp;$AF41&amp;$AG41&amp;$AH41&amp;$AI41&amp;$AJ41))</x:f>
+        <x:f>IF(TRIM($A41)="","",IF(OR($A41="Selección de la mejor respuesta",$A41="SELECCION_MEJOR_RESPUESTA",$A41="Subítem de caso o problema",$A41="SUBITEM_CASO"),IF(TRIM($C41)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D41:$H41&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I41)&lt;&gt;"",OR(LEFT(TRIM($I41),1)="A",LEFT(TRIM($I41),1)="B",LEFT(TRIM($I41),1)="C",LEFT(TRIM($I41),1)="D",LEFT(TRIM($I41),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A41)="","",IF(COUNTIF($Q41:$AJ41,"?*")=0,"OK","Falta revisar: "&amp;$Q41&amp;$R41&amp;$S41&amp;$T41&amp;$U41&amp;$V41&amp;$W41&amp;$X41&amp;$Y41&amp;$Z41&amp;$AA41&amp;$AB41&amp;$AC41&amp;$AD41&amp;$AE41&amp;$AF41&amp;$AG41&amp;$AH41&amp;$AI41&amp;$AJ41))))</x:f>
       </x:c>
       <x:c r="M41" s="341"/>
       <x:c r="N41"/>
@@ -6909,7 +6910,7 @@
         <x:f>IF(AND($A41="Verdadero o Falso Complejas",TRIM($I41)&lt;&gt;"",NOT(OR(LEFT(TRIM($I41),1)="A",LEFT(TRIM($I41),1)="B",LEFT(TRIM($I41),1)="C",LEFT(TRIM($I41),1)="D",LEFT(TRIM($I41),1)="E"))),IF(COUNTIF($Q41:$AE41,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG41" t="str">
-        <x:f>IF(AND(OR($A41="Selección de la mejor respuesta",$A41="Subítem de caso o problema"),COUNTIF($D41:$H41,"?*")&lt;5),IF(COUNTIF($Q41:$AF41,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A41="Selección de la mejor respuesta",$A41="Subítem de caso o problema"),COUNTA($D41:$H41)&lt;5),IF(COUNTIF($Q41:$AF41,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH41" t="str">
         <x:f>IF(AND(OR($A41="Selección de la mejor respuesta",$A41="Subítem de caso o problema"),TRIM($I41)&lt;&gt;"",NOT(OR(LEFT(TRIM($I41),1)="A",LEFT(TRIM($I41),1)="B",LEFT(TRIM($I41),1)="C",LEFT(TRIM($I41),1)="D",LEFT(TRIM($I41),1)="E"))),IF(COUNTIF($Q41:$AG41,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -6960,7 +6961,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L42" s="345" t="str">
-        <x:f>IF(TRIM($A42)="","",IF(COUNTIF($Q42:$AJ42,"?*")=0,"OK","Falta revisar: "&amp;$Q42&amp;$R42&amp;$S42&amp;$T42&amp;$U42&amp;$V42&amp;$W42&amp;$X42&amp;$Y42&amp;$Z42&amp;$AA42&amp;$AB42&amp;$AC42&amp;$AD42&amp;$AE42&amp;$AF42&amp;$AG42&amp;$AH42&amp;$AI42&amp;$AJ42))</x:f>
+        <x:f>IF(TRIM($A42)="","",IF(OR($A42="Selección de la mejor respuesta",$A42="SELECCION_MEJOR_RESPUESTA",$A42="Subítem de caso o problema",$A42="SUBITEM_CASO"),IF(TRIM($C42)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D42:$H42&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I42)&lt;&gt;"",OR(LEFT(TRIM($I42),1)="A",LEFT(TRIM($I42),1)="B",LEFT(TRIM($I42),1)="C",LEFT(TRIM($I42),1)="D",LEFT(TRIM($I42),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A42)="","",IF(COUNTIF($Q42:$AJ42,"?*")=0,"OK","Falta revisar: "&amp;$Q42&amp;$R42&amp;$S42&amp;$T42&amp;$U42&amp;$V42&amp;$W42&amp;$X42&amp;$Y42&amp;$Z42&amp;$AA42&amp;$AB42&amp;$AC42&amp;$AD42&amp;$AE42&amp;$AF42&amp;$AG42&amp;$AH42&amp;$AI42&amp;$AJ42))))</x:f>
       </x:c>
       <x:c r="M42" s="341"/>
       <x:c r="N42"/>
@@ -7016,7 +7017,7 @@
         <x:f>IF(AND($A42="Verdadero o Falso Complejas",TRIM($I42)&lt;&gt;"",NOT(OR(LEFT(TRIM($I42),1)="A",LEFT(TRIM($I42),1)="B",LEFT(TRIM($I42),1)="C",LEFT(TRIM($I42),1)="D",LEFT(TRIM($I42),1)="E"))),IF(COUNTIF($Q42:$AE42,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG42" t="str">
-        <x:f>IF(AND(OR($A42="Selección de la mejor respuesta",$A42="Subítem de caso o problema"),COUNTIF($D42:$H42,"?*")&lt;5),IF(COUNTIF($Q42:$AF42,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A42="Selección de la mejor respuesta",$A42="Subítem de caso o problema"),COUNTA($D42:$H42)&lt;5),IF(COUNTIF($Q42:$AF42,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH42" t="str">
         <x:f>IF(AND(OR($A42="Selección de la mejor respuesta",$A42="Subítem de caso o problema"),TRIM($I42)&lt;&gt;"",NOT(OR(LEFT(TRIM($I42),1)="A",LEFT(TRIM($I42),1)="B",LEFT(TRIM($I42),1)="C",LEFT(TRIM($I42),1)="D",LEFT(TRIM($I42),1)="E"))),IF(COUNTIF($Q42:$AG42,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7067,7 +7068,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L43" s="345" t="str">
-        <x:f>IF(TRIM($A43)="","",IF(COUNTIF($Q43:$AJ43,"?*")=0,"OK","Falta revisar: "&amp;$Q43&amp;$R43&amp;$S43&amp;$T43&amp;$U43&amp;$V43&amp;$W43&amp;$X43&amp;$Y43&amp;$Z43&amp;$AA43&amp;$AB43&amp;$AC43&amp;$AD43&amp;$AE43&amp;$AF43&amp;$AG43&amp;$AH43&amp;$AI43&amp;$AJ43))</x:f>
+        <x:f>IF(TRIM($A43)="","",IF(OR($A43="Selección de la mejor respuesta",$A43="SELECCION_MEJOR_RESPUESTA",$A43="Subítem de caso o problema",$A43="SUBITEM_CASO"),IF(TRIM($C43)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D43:$H43&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I43)&lt;&gt;"",OR(LEFT(TRIM($I43),1)="A",LEFT(TRIM($I43),1)="B",LEFT(TRIM($I43),1)="C",LEFT(TRIM($I43),1)="D",LEFT(TRIM($I43),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A43)="","",IF(COUNTIF($Q43:$AJ43,"?*")=0,"OK","Falta revisar: "&amp;$Q43&amp;$R43&amp;$S43&amp;$T43&amp;$U43&amp;$V43&amp;$W43&amp;$X43&amp;$Y43&amp;$Z43&amp;$AA43&amp;$AB43&amp;$AC43&amp;$AD43&amp;$AE43&amp;$AF43&amp;$AG43&amp;$AH43&amp;$AI43&amp;$AJ43))))</x:f>
       </x:c>
       <x:c r="M43" s="341"/>
       <x:c r="N43"/>
@@ -7123,7 +7124,7 @@
         <x:f>IF(AND($A43="Verdadero o Falso Complejas",TRIM($I43)&lt;&gt;"",NOT(OR(LEFT(TRIM($I43),1)="A",LEFT(TRIM($I43),1)="B",LEFT(TRIM($I43),1)="C",LEFT(TRIM($I43),1)="D",LEFT(TRIM($I43),1)="E"))),IF(COUNTIF($Q43:$AE43,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG43" t="str">
-        <x:f>IF(AND(OR($A43="Selección de la mejor respuesta",$A43="Subítem de caso o problema"),COUNTIF($D43:$H43,"?*")&lt;5),IF(COUNTIF($Q43:$AF43,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A43="Selección de la mejor respuesta",$A43="Subítem de caso o problema"),COUNTA($D43:$H43)&lt;5),IF(COUNTIF($Q43:$AF43,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH43" t="str">
         <x:f>IF(AND(OR($A43="Selección de la mejor respuesta",$A43="Subítem de caso o problema"),TRIM($I43)&lt;&gt;"",NOT(OR(LEFT(TRIM($I43),1)="A",LEFT(TRIM($I43),1)="B",LEFT(TRIM($I43),1)="C",LEFT(TRIM($I43),1)="D",LEFT(TRIM($I43),1)="E"))),IF(COUNTIF($Q43:$AG43,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7174,7 +7175,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L44" s="345" t="str">
-        <x:f>IF(TRIM($A44)="","",IF(COUNTIF($Q44:$AJ44,"?*")=0,"OK","Falta revisar: "&amp;$Q44&amp;$R44&amp;$S44&amp;$T44&amp;$U44&amp;$V44&amp;$W44&amp;$X44&amp;$Y44&amp;$Z44&amp;$AA44&amp;$AB44&amp;$AC44&amp;$AD44&amp;$AE44&amp;$AF44&amp;$AG44&amp;$AH44&amp;$AI44&amp;$AJ44))</x:f>
+        <x:f>IF(TRIM($A44)="","",IF(OR($A44="Selección de la mejor respuesta",$A44="SELECCION_MEJOR_RESPUESTA",$A44="Subítem de caso o problema",$A44="SUBITEM_CASO"),IF(TRIM($C44)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D44:$H44&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I44)&lt;&gt;"",OR(LEFT(TRIM($I44),1)="A",LEFT(TRIM($I44),1)="B",LEFT(TRIM($I44),1)="C",LEFT(TRIM($I44),1)="D",LEFT(TRIM($I44),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A44)="","",IF(COUNTIF($Q44:$AJ44,"?*")=0,"OK","Falta revisar: "&amp;$Q44&amp;$R44&amp;$S44&amp;$T44&amp;$U44&amp;$V44&amp;$W44&amp;$X44&amp;$Y44&amp;$Z44&amp;$AA44&amp;$AB44&amp;$AC44&amp;$AD44&amp;$AE44&amp;$AF44&amp;$AG44&amp;$AH44&amp;$AI44&amp;$AJ44))))</x:f>
       </x:c>
       <x:c r="M44" s="341"/>
       <x:c r="N44"/>
@@ -7230,7 +7231,7 @@
         <x:f>IF(AND($A44="Verdadero o Falso Complejas",TRIM($I44)&lt;&gt;"",NOT(OR(LEFT(TRIM($I44),1)="A",LEFT(TRIM($I44),1)="B",LEFT(TRIM($I44),1)="C",LEFT(TRIM($I44),1)="D",LEFT(TRIM($I44),1)="E"))),IF(COUNTIF($Q44:$AE44,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG44" t="str">
-        <x:f>IF(AND(OR($A44="Selección de la mejor respuesta",$A44="Subítem de caso o problema"),COUNTIF($D44:$H44,"?*")&lt;5),IF(COUNTIF($Q44:$AF44,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A44="Selección de la mejor respuesta",$A44="Subítem de caso o problema"),COUNTA($D44:$H44)&lt;5),IF(COUNTIF($Q44:$AF44,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH44" t="str">
         <x:f>IF(AND(OR($A44="Selección de la mejor respuesta",$A44="Subítem de caso o problema"),TRIM($I44)&lt;&gt;"",NOT(OR(LEFT(TRIM($I44),1)="A",LEFT(TRIM($I44),1)="B",LEFT(TRIM($I44),1)="C",LEFT(TRIM($I44),1)="D",LEFT(TRIM($I44),1)="E"))),IF(COUNTIF($Q44:$AG44,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7281,7 +7282,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L45" s="345" t="str">
-        <x:f>IF(TRIM($A45)="","",IF(COUNTIF($Q45:$AJ45,"?*")=0,"OK","Falta revisar: "&amp;$Q45&amp;$R45&amp;$S45&amp;$T45&amp;$U45&amp;$V45&amp;$W45&amp;$X45&amp;$Y45&amp;$Z45&amp;$AA45&amp;$AB45&amp;$AC45&amp;$AD45&amp;$AE45&amp;$AF45&amp;$AG45&amp;$AH45&amp;$AI45&amp;$AJ45))</x:f>
+        <x:f>IF(TRIM($A45)="","",IF(OR($A45="Selección de la mejor respuesta",$A45="SELECCION_MEJOR_RESPUESTA",$A45="Subítem de caso o problema",$A45="SUBITEM_CASO"),IF(TRIM($C45)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D45:$H45&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I45)&lt;&gt;"",OR(LEFT(TRIM($I45),1)="A",LEFT(TRIM($I45),1)="B",LEFT(TRIM($I45),1)="C",LEFT(TRIM($I45),1)="D",LEFT(TRIM($I45),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A45)="","",IF(COUNTIF($Q45:$AJ45,"?*")=0,"OK","Falta revisar: "&amp;$Q45&amp;$R45&amp;$S45&amp;$T45&amp;$U45&amp;$V45&amp;$W45&amp;$X45&amp;$Y45&amp;$Z45&amp;$AA45&amp;$AB45&amp;$AC45&amp;$AD45&amp;$AE45&amp;$AF45&amp;$AG45&amp;$AH45&amp;$AI45&amp;$AJ45))))</x:f>
       </x:c>
       <x:c r="M45" s="341"/>
       <x:c r="N45"/>
@@ -7337,7 +7338,7 @@
         <x:f>IF(AND($A45="Verdadero o Falso Complejas",TRIM($I45)&lt;&gt;"",NOT(OR(LEFT(TRIM($I45),1)="A",LEFT(TRIM($I45),1)="B",LEFT(TRIM($I45),1)="C",LEFT(TRIM($I45),1)="D",LEFT(TRIM($I45),1)="E"))),IF(COUNTIF($Q45:$AE45,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG45" t="str">
-        <x:f>IF(AND(OR($A45="Selección de la mejor respuesta",$A45="Subítem de caso o problema"),COUNTIF($D45:$H45,"?*")&lt;5),IF(COUNTIF($Q45:$AF45,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A45="Selección de la mejor respuesta",$A45="Subítem de caso o problema"),COUNTA($D45:$H45)&lt;5),IF(COUNTIF($Q45:$AF45,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH45" t="str">
         <x:f>IF(AND(OR($A45="Selección de la mejor respuesta",$A45="Subítem de caso o problema"),TRIM($I45)&lt;&gt;"",NOT(OR(LEFT(TRIM($I45),1)="A",LEFT(TRIM($I45),1)="B",LEFT(TRIM($I45),1)="C",LEFT(TRIM($I45),1)="D",LEFT(TRIM($I45),1)="E"))),IF(COUNTIF($Q45:$AG45,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7388,7 +7389,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L46" s="345" t="str">
-        <x:f>IF(TRIM($A46)="","",IF(COUNTIF($Q46:$AJ46,"?*")=0,"OK","Falta revisar: "&amp;$Q46&amp;$R46&amp;$S46&amp;$T46&amp;$U46&amp;$V46&amp;$W46&amp;$X46&amp;$Y46&amp;$Z46&amp;$AA46&amp;$AB46&amp;$AC46&amp;$AD46&amp;$AE46&amp;$AF46&amp;$AG46&amp;$AH46&amp;$AI46&amp;$AJ46))</x:f>
+        <x:f>IF(TRIM($A46)="","",IF(OR($A46="Selección de la mejor respuesta",$A46="SELECCION_MEJOR_RESPUESTA",$A46="Subítem de caso o problema",$A46="SUBITEM_CASO"),IF(TRIM($C46)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D46:$H46&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I46)&lt;&gt;"",OR(LEFT(TRIM($I46),1)="A",LEFT(TRIM($I46),1)="B",LEFT(TRIM($I46),1)="C",LEFT(TRIM($I46),1)="D",LEFT(TRIM($I46),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A46)="","",IF(COUNTIF($Q46:$AJ46,"?*")=0,"OK","Falta revisar: "&amp;$Q46&amp;$R46&amp;$S46&amp;$T46&amp;$U46&amp;$V46&amp;$W46&amp;$X46&amp;$Y46&amp;$Z46&amp;$AA46&amp;$AB46&amp;$AC46&amp;$AD46&amp;$AE46&amp;$AF46&amp;$AG46&amp;$AH46&amp;$AI46&amp;$AJ46))))</x:f>
       </x:c>
       <x:c r="M46" s="341"/>
       <x:c r="N46"/>
@@ -7444,7 +7445,7 @@
         <x:f>IF(AND($A46="Verdadero o Falso Complejas",TRIM($I46)&lt;&gt;"",NOT(OR(LEFT(TRIM($I46),1)="A",LEFT(TRIM($I46),1)="B",LEFT(TRIM($I46),1)="C",LEFT(TRIM($I46),1)="D",LEFT(TRIM($I46),1)="E"))),IF(COUNTIF($Q46:$AE46,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG46" t="str">
-        <x:f>IF(AND(OR($A46="Selección de la mejor respuesta",$A46="Subítem de caso o problema"),COUNTIF($D46:$H46,"?*")&lt;5),IF(COUNTIF($Q46:$AF46,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A46="Selección de la mejor respuesta",$A46="Subítem de caso o problema"),COUNTA($D46:$H46)&lt;5),IF(COUNTIF($Q46:$AF46,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH46" t="str">
         <x:f>IF(AND(OR($A46="Selección de la mejor respuesta",$A46="Subítem de caso o problema"),TRIM($I46)&lt;&gt;"",NOT(OR(LEFT(TRIM($I46),1)="A",LEFT(TRIM($I46),1)="B",LEFT(TRIM($I46),1)="C",LEFT(TRIM($I46),1)="D",LEFT(TRIM($I46),1)="E"))),IF(COUNTIF($Q46:$AG46,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7495,7 +7496,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L47" s="347" t="str">
-        <x:f>IF(TRIM($A47)="","",IF(COUNTIF($Q47:$AJ47,"?*")=0,"OK","Falta revisar: "&amp;$Q47&amp;$R47&amp;$S47&amp;$T47&amp;$U47&amp;$V47&amp;$W47&amp;$X47&amp;$Y47&amp;$Z47&amp;$AA47&amp;$AB47&amp;$AC47&amp;$AD47&amp;$AE47&amp;$AF47&amp;$AG47&amp;$AH47&amp;$AI47&amp;$AJ47))</x:f>
+        <x:f>IF(TRIM($A47)="","",IF(OR($A47="Selección de la mejor respuesta",$A47="SELECCION_MEJOR_RESPUESTA",$A47="Subítem de caso o problema",$A47="SUBITEM_CASO"),IF(TRIM($C47)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D47:$H47&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I47)&lt;&gt;"",OR(LEFT(TRIM($I47),1)="A",LEFT(TRIM($I47),1)="B",LEFT(TRIM($I47),1)="C",LEFT(TRIM($I47),1)="D",LEFT(TRIM($I47),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A47)="","",IF(COUNTIF($Q47:$AJ47,"?*")=0,"OK","Falta revisar: "&amp;$Q47&amp;$R47&amp;$S47&amp;$T47&amp;$U47&amp;$V47&amp;$W47&amp;$X47&amp;$Y47&amp;$Z47&amp;$AA47&amp;$AB47&amp;$AC47&amp;$AD47&amp;$AE47&amp;$AF47&amp;$AG47&amp;$AH47&amp;$AI47&amp;$AJ47))))</x:f>
       </x:c>
       <x:c r="M47" s="341"/>
       <x:c r="N47"/>
@@ -7551,7 +7552,7 @@
         <x:f>IF(AND($A47="Verdadero o Falso Complejas",TRIM($I47)&lt;&gt;"",NOT(OR(LEFT(TRIM($I47),1)="A",LEFT(TRIM($I47),1)="B",LEFT(TRIM($I47),1)="C",LEFT(TRIM($I47),1)="D",LEFT(TRIM($I47),1)="E"))),IF(COUNTIF($Q47:$AE47,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG47" t="str">
-        <x:f>IF(AND(OR($A47="Selección de la mejor respuesta",$A47="Subítem de caso o problema"),COUNTIF($D47:$H47,"?*")&lt;5),IF(COUNTIF($Q47:$AF47,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A47="Selección de la mejor respuesta",$A47="Subítem de caso o problema"),COUNTA($D47:$H47)&lt;5),IF(COUNTIF($Q47:$AF47,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH47" t="str">
         <x:f>IF(AND(OR($A47="Selección de la mejor respuesta",$A47="Subítem de caso o problema"),TRIM($I47)&lt;&gt;"",NOT(OR(LEFT(TRIM($I47),1)="A",LEFT(TRIM($I47),1)="B",LEFT(TRIM($I47),1)="C",LEFT(TRIM($I47),1)="D",LEFT(TRIM($I47),1)="E"))),IF(COUNTIF($Q47:$AG47,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7602,7 +7603,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L48" s="347" t="str">
-        <x:f>IF(TRIM($A48)="","",IF(COUNTIF($Q48:$AJ48,"?*")=0,"OK","Falta revisar: "&amp;$Q48&amp;$R48&amp;$S48&amp;$T48&amp;$U48&amp;$V48&amp;$W48&amp;$X48&amp;$Y48&amp;$Z48&amp;$AA48&amp;$AB48&amp;$AC48&amp;$AD48&amp;$AE48&amp;$AF48&amp;$AG48&amp;$AH48&amp;$AI48&amp;$AJ48))</x:f>
+        <x:f>IF(TRIM($A48)="","",IF(OR($A48="Selección de la mejor respuesta",$A48="SELECCION_MEJOR_RESPUESTA",$A48="Subítem de caso o problema",$A48="SUBITEM_CASO"),IF(TRIM($C48)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D48:$H48&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I48)&lt;&gt;"",OR(LEFT(TRIM($I48),1)="A",LEFT(TRIM($I48),1)="B",LEFT(TRIM($I48),1)="C",LEFT(TRIM($I48),1)="D",LEFT(TRIM($I48),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A48)="","",IF(COUNTIF($Q48:$AJ48,"?*")=0,"OK","Falta revisar: "&amp;$Q48&amp;$R48&amp;$S48&amp;$T48&amp;$U48&amp;$V48&amp;$W48&amp;$X48&amp;$Y48&amp;$Z48&amp;$AA48&amp;$AB48&amp;$AC48&amp;$AD48&amp;$AE48&amp;$AF48&amp;$AG48&amp;$AH48&amp;$AI48&amp;$AJ48))))</x:f>
       </x:c>
       <x:c r="M48" s="341"/>
       <x:c r="N48"/>
@@ -7658,7 +7659,7 @@
         <x:f>IF(AND($A48="Verdadero o Falso Complejas",TRIM($I48)&lt;&gt;"",NOT(OR(LEFT(TRIM($I48),1)="A",LEFT(TRIM($I48),1)="B",LEFT(TRIM($I48),1)="C",LEFT(TRIM($I48),1)="D",LEFT(TRIM($I48),1)="E"))),IF(COUNTIF($Q48:$AE48,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG48" t="str">
-        <x:f>IF(AND(OR($A48="Selección de la mejor respuesta",$A48="Subítem de caso o problema"),COUNTIF($D48:$H48,"?*")&lt;5),IF(COUNTIF($Q48:$AF48,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A48="Selección de la mejor respuesta",$A48="Subítem de caso o problema"),COUNTA($D48:$H48)&lt;5),IF(COUNTIF($Q48:$AF48,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH48" t="str">
         <x:f>IF(AND(OR($A48="Selección de la mejor respuesta",$A48="Subítem de caso o problema"),TRIM($I48)&lt;&gt;"",NOT(OR(LEFT(TRIM($I48),1)="A",LEFT(TRIM($I48),1)="B",LEFT(TRIM($I48),1)="C",LEFT(TRIM($I48),1)="D",LEFT(TRIM($I48),1)="E"))),IF(COUNTIF($Q48:$AG48,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7709,7 +7710,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L49" s="347" t="str">
-        <x:f>IF(TRIM($A49)="","",IF(COUNTIF($Q49:$AJ49,"?*")=0,"OK","Falta revisar: "&amp;$Q49&amp;$R49&amp;$S49&amp;$T49&amp;$U49&amp;$V49&amp;$W49&amp;$X49&amp;$Y49&amp;$Z49&amp;$AA49&amp;$AB49&amp;$AC49&amp;$AD49&amp;$AE49&amp;$AF49&amp;$AG49&amp;$AH49&amp;$AI49&amp;$AJ49))</x:f>
+        <x:f>IF(TRIM($A49)="","",IF(OR($A49="Selección de la mejor respuesta",$A49="SELECCION_MEJOR_RESPUESTA",$A49="Subítem de caso o problema",$A49="SUBITEM_CASO"),IF(TRIM($C49)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D49:$H49&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I49)&lt;&gt;"",OR(LEFT(TRIM($I49),1)="A",LEFT(TRIM($I49),1)="B",LEFT(TRIM($I49),1)="C",LEFT(TRIM($I49),1)="D",LEFT(TRIM($I49),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A49)="","",IF(COUNTIF($Q49:$AJ49,"?*")=0,"OK","Falta revisar: "&amp;$Q49&amp;$R49&amp;$S49&amp;$T49&amp;$U49&amp;$V49&amp;$W49&amp;$X49&amp;$Y49&amp;$Z49&amp;$AA49&amp;$AB49&amp;$AC49&amp;$AD49&amp;$AE49&amp;$AF49&amp;$AG49&amp;$AH49&amp;$AI49&amp;$AJ49))))</x:f>
       </x:c>
       <x:c r="M49" s="341"/>
       <x:c r="N49"/>
@@ -7765,7 +7766,7 @@
         <x:f>IF(AND($A49="Verdadero o Falso Complejas",TRIM($I49)&lt;&gt;"",NOT(OR(LEFT(TRIM($I49),1)="A",LEFT(TRIM($I49),1)="B",LEFT(TRIM($I49),1)="C",LEFT(TRIM($I49),1)="D",LEFT(TRIM($I49),1)="E"))),IF(COUNTIF($Q49:$AE49,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG49" t="str">
-        <x:f>IF(AND(OR($A49="Selección de la mejor respuesta",$A49="Subítem de caso o problema"),COUNTIF($D49:$H49,"?*")&lt;5),IF(COUNTIF($Q49:$AF49,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A49="Selección de la mejor respuesta",$A49="Subítem de caso o problema"),COUNTA($D49:$H49)&lt;5),IF(COUNTIF($Q49:$AF49,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH49" t="str">
         <x:f>IF(AND(OR($A49="Selección de la mejor respuesta",$A49="Subítem de caso o problema"),TRIM($I49)&lt;&gt;"",NOT(OR(LEFT(TRIM($I49),1)="A",LEFT(TRIM($I49),1)="B",LEFT(TRIM($I49),1)="C",LEFT(TRIM($I49),1)="D",LEFT(TRIM($I49),1)="E"))),IF(COUNTIF($Q49:$AG49,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7816,7 +7817,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L50" s="347" t="str">
-        <x:f>IF(TRIM($A50)="","",IF(COUNTIF($Q50:$AJ50,"?*")=0,"OK","Falta revisar: "&amp;$Q50&amp;$R50&amp;$S50&amp;$T50&amp;$U50&amp;$V50&amp;$W50&amp;$X50&amp;$Y50&amp;$Z50&amp;$AA50&amp;$AB50&amp;$AC50&amp;$AD50&amp;$AE50&amp;$AF50&amp;$AG50&amp;$AH50&amp;$AI50&amp;$AJ50))</x:f>
+        <x:f>IF(TRIM($A50)="","",IF(OR($A50="Selección de la mejor respuesta",$A50="SELECCION_MEJOR_RESPUESTA",$A50="Subítem de caso o problema",$A50="SUBITEM_CASO"),IF(TRIM($C50)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D50:$H50&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I50)&lt;&gt;"",OR(LEFT(TRIM($I50),1)="A",LEFT(TRIM($I50),1)="B",LEFT(TRIM($I50),1)="C",LEFT(TRIM($I50),1)="D",LEFT(TRIM($I50),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A50)="","",IF(COUNTIF($Q50:$AJ50,"?*")=0,"OK","Falta revisar: "&amp;$Q50&amp;$R50&amp;$S50&amp;$T50&amp;$U50&amp;$V50&amp;$W50&amp;$X50&amp;$Y50&amp;$Z50&amp;$AA50&amp;$AB50&amp;$AC50&amp;$AD50&amp;$AE50&amp;$AF50&amp;$AG50&amp;$AH50&amp;$AI50&amp;$AJ50))))</x:f>
       </x:c>
       <x:c r="M50" s="341"/>
       <x:c r="N50"/>
@@ -7872,7 +7873,7 @@
         <x:f>IF(AND($A50="Verdadero o Falso Complejas",TRIM($I50)&lt;&gt;"",NOT(OR(LEFT(TRIM($I50),1)="A",LEFT(TRIM($I50),1)="B",LEFT(TRIM($I50),1)="C",LEFT(TRIM($I50),1)="D",LEFT(TRIM($I50),1)="E"))),IF(COUNTIF($Q50:$AE50,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG50" t="str">
-        <x:f>IF(AND(OR($A50="Selección de la mejor respuesta",$A50="Subítem de caso o problema"),COUNTIF($D50:$H50,"?*")&lt;5),IF(COUNTIF($Q50:$AF50,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A50="Selección de la mejor respuesta",$A50="Subítem de caso o problema"),COUNTA($D50:$H50)&lt;5),IF(COUNTIF($Q50:$AF50,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH50" t="str">
         <x:f>IF(AND(OR($A50="Selección de la mejor respuesta",$A50="Subítem de caso o problema"),TRIM($I50)&lt;&gt;"",NOT(OR(LEFT(TRIM($I50),1)="A",LEFT(TRIM($I50),1)="B",LEFT(TRIM($I50),1)="C",LEFT(TRIM($I50),1)="D",LEFT(TRIM($I50),1)="E"))),IF(COUNTIF($Q50:$AG50,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -7923,7 +7924,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L51" s="347" t="str">
-        <x:f>IF(TRIM($A51)="","",IF(COUNTIF($Q51:$AJ51,"?*")=0,"OK","Falta revisar: "&amp;$Q51&amp;$R51&amp;$S51&amp;$T51&amp;$U51&amp;$V51&amp;$W51&amp;$X51&amp;$Y51&amp;$Z51&amp;$AA51&amp;$AB51&amp;$AC51&amp;$AD51&amp;$AE51&amp;$AF51&amp;$AG51&amp;$AH51&amp;$AI51&amp;$AJ51))</x:f>
+        <x:f>IF(TRIM($A51)="","",IF(OR($A51="Selección de la mejor respuesta",$A51="SELECCION_MEJOR_RESPUESTA",$A51="Subítem de caso o problema",$A51="SUBITEM_CASO"),IF(TRIM($C51)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D51:$H51&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I51)&lt;&gt;"",OR(LEFT(TRIM($I51),1)="A",LEFT(TRIM($I51),1)="B",LEFT(TRIM($I51),1)="C",LEFT(TRIM($I51),1)="D",LEFT(TRIM($I51),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A51)="","",IF(COUNTIF($Q51:$AJ51,"?*")=0,"OK","Falta revisar: "&amp;$Q51&amp;$R51&amp;$S51&amp;$T51&amp;$U51&amp;$V51&amp;$W51&amp;$X51&amp;$Y51&amp;$Z51&amp;$AA51&amp;$AB51&amp;$AC51&amp;$AD51&amp;$AE51&amp;$AF51&amp;$AG51&amp;$AH51&amp;$AI51&amp;$AJ51))))</x:f>
       </x:c>
       <x:c r="M51" s="341"/>
       <x:c r="N51"/>
@@ -7979,7 +7980,7 @@
         <x:f>IF(AND($A51="Verdadero o Falso Complejas",TRIM($I51)&lt;&gt;"",NOT(OR(LEFT(TRIM($I51),1)="A",LEFT(TRIM($I51),1)="B",LEFT(TRIM($I51),1)="C",LEFT(TRIM($I51),1)="D",LEFT(TRIM($I51),1)="E"))),IF(COUNTIF($Q51:$AE51,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG51" t="str">
-        <x:f>IF(AND(OR($A51="Selección de la mejor respuesta",$A51="Subítem de caso o problema"),COUNTIF($D51:$H51,"?*")&lt;5),IF(COUNTIF($Q51:$AF51,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A51="Selección de la mejor respuesta",$A51="Subítem de caso o problema"),COUNTA($D51:$H51)&lt;5),IF(COUNTIF($Q51:$AF51,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH51" t="str">
         <x:f>IF(AND(OR($A51="Selección de la mejor respuesta",$A51="Subítem de caso o problema"),TRIM($I51)&lt;&gt;"",NOT(OR(LEFT(TRIM($I51),1)="A",LEFT(TRIM($I51),1)="B",LEFT(TRIM($I51),1)="C",LEFT(TRIM($I51),1)="D",LEFT(TRIM($I51),1)="E"))),IF(COUNTIF($Q51:$AG51,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8030,7 +8031,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L52" s="347" t="str">
-        <x:f>IF(TRIM($A52)="","",IF(COUNTIF($Q52:$AJ52,"?*")=0,"OK","Falta revisar: "&amp;$Q52&amp;$R52&amp;$S52&amp;$T52&amp;$U52&amp;$V52&amp;$W52&amp;$X52&amp;$Y52&amp;$Z52&amp;$AA52&amp;$AB52&amp;$AC52&amp;$AD52&amp;$AE52&amp;$AF52&amp;$AG52&amp;$AH52&amp;$AI52&amp;$AJ52))</x:f>
+        <x:f>IF(TRIM($A52)="","",IF(OR($A52="Selección de la mejor respuesta",$A52="SELECCION_MEJOR_RESPUESTA",$A52="Subítem de caso o problema",$A52="SUBITEM_CASO"),IF(TRIM($C52)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D52:$H52&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I52)&lt;&gt;"",OR(LEFT(TRIM($I52),1)="A",LEFT(TRIM($I52),1)="B",LEFT(TRIM($I52),1)="C",LEFT(TRIM($I52),1)="D",LEFT(TRIM($I52),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A52)="","",IF(COUNTIF($Q52:$AJ52,"?*")=0,"OK","Falta revisar: "&amp;$Q52&amp;$R52&amp;$S52&amp;$T52&amp;$U52&amp;$V52&amp;$W52&amp;$X52&amp;$Y52&amp;$Z52&amp;$AA52&amp;$AB52&amp;$AC52&amp;$AD52&amp;$AE52&amp;$AF52&amp;$AG52&amp;$AH52&amp;$AI52&amp;$AJ52))))</x:f>
       </x:c>
       <x:c r="M52" s="341"/>
       <x:c r="N52"/>
@@ -8086,7 +8087,7 @@
         <x:f>IF(AND($A52="Verdadero o Falso Complejas",TRIM($I52)&lt;&gt;"",NOT(OR(LEFT(TRIM($I52),1)="A",LEFT(TRIM($I52),1)="B",LEFT(TRIM($I52),1)="C",LEFT(TRIM($I52),1)="D",LEFT(TRIM($I52),1)="E"))),IF(COUNTIF($Q52:$AE52,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG52" t="str">
-        <x:f>IF(AND(OR($A52="Selección de la mejor respuesta",$A52="Subítem de caso o problema"),COUNTIF($D52:$H52,"?*")&lt;5),IF(COUNTIF($Q52:$AF52,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A52="Selección de la mejor respuesta",$A52="Subítem de caso o problema"),COUNTA($D52:$H52)&lt;5),IF(COUNTIF($Q52:$AF52,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH52" t="str">
         <x:f>IF(AND(OR($A52="Selección de la mejor respuesta",$A52="Subítem de caso o problema"),TRIM($I52)&lt;&gt;"",NOT(OR(LEFT(TRIM($I52),1)="A",LEFT(TRIM($I52),1)="B",LEFT(TRIM($I52),1)="C",LEFT(TRIM($I52),1)="D",LEFT(TRIM($I52),1)="E"))),IF(COUNTIF($Q52:$AG52,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8137,7 +8138,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L53" s="347" t="str">
-        <x:f>IF(TRIM($A53)="","",IF(COUNTIF($Q53:$AJ53,"?*")=0,"OK","Falta revisar: "&amp;$Q53&amp;$R53&amp;$S53&amp;$T53&amp;$U53&amp;$V53&amp;$W53&amp;$X53&amp;$Y53&amp;$Z53&amp;$AA53&amp;$AB53&amp;$AC53&amp;$AD53&amp;$AE53&amp;$AF53&amp;$AG53&amp;$AH53&amp;$AI53&amp;$AJ53))</x:f>
+        <x:f>IF(TRIM($A53)="","",IF(OR($A53="Selección de la mejor respuesta",$A53="SELECCION_MEJOR_RESPUESTA",$A53="Subítem de caso o problema",$A53="SUBITEM_CASO"),IF(TRIM($C53)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D53:$H53&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I53)&lt;&gt;"",OR(LEFT(TRIM($I53),1)="A",LEFT(TRIM($I53),1)="B",LEFT(TRIM($I53),1)="C",LEFT(TRIM($I53),1)="D",LEFT(TRIM($I53),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A53)="","",IF(COUNTIF($Q53:$AJ53,"?*")=0,"OK","Falta revisar: "&amp;$Q53&amp;$R53&amp;$S53&amp;$T53&amp;$U53&amp;$V53&amp;$W53&amp;$X53&amp;$Y53&amp;$Z53&amp;$AA53&amp;$AB53&amp;$AC53&amp;$AD53&amp;$AE53&amp;$AF53&amp;$AG53&amp;$AH53&amp;$AI53&amp;$AJ53))))</x:f>
       </x:c>
       <x:c r="M53" s="341"/>
       <x:c r="N53"/>
@@ -8193,7 +8194,7 @@
         <x:f>IF(AND($A53="Verdadero o Falso Complejas",TRIM($I53)&lt;&gt;"",NOT(OR(LEFT(TRIM($I53),1)="A",LEFT(TRIM($I53),1)="B",LEFT(TRIM($I53),1)="C",LEFT(TRIM($I53),1)="D",LEFT(TRIM($I53),1)="E"))),IF(COUNTIF($Q53:$AE53,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG53" t="str">
-        <x:f>IF(AND(OR($A53="Selección de la mejor respuesta",$A53="Subítem de caso o problema"),COUNTIF($D53:$H53,"?*")&lt;5),IF(COUNTIF($Q53:$AF53,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A53="Selección de la mejor respuesta",$A53="Subítem de caso o problema"),COUNTA($D53:$H53)&lt;5),IF(COUNTIF($Q53:$AF53,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH53" t="str">
         <x:f>IF(AND(OR($A53="Selección de la mejor respuesta",$A53="Subítem de caso o problema"),TRIM($I53)&lt;&gt;"",NOT(OR(LEFT(TRIM($I53),1)="A",LEFT(TRIM($I53),1)="B",LEFT(TRIM($I53),1)="C",LEFT(TRIM($I53),1)="D",LEFT(TRIM($I53),1)="E"))),IF(COUNTIF($Q53:$AG53,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8244,7 +8245,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L54" s="347" t="str">
-        <x:f>IF(TRIM($A54)="","",IF(COUNTIF($Q54:$AJ54,"?*")=0,"OK","Falta revisar: "&amp;$Q54&amp;$R54&amp;$S54&amp;$T54&amp;$U54&amp;$V54&amp;$W54&amp;$X54&amp;$Y54&amp;$Z54&amp;$AA54&amp;$AB54&amp;$AC54&amp;$AD54&amp;$AE54&amp;$AF54&amp;$AG54&amp;$AH54&amp;$AI54&amp;$AJ54))</x:f>
+        <x:f>IF(TRIM($A54)="","",IF(OR($A54="Selección de la mejor respuesta",$A54="SELECCION_MEJOR_RESPUESTA",$A54="Subítem de caso o problema",$A54="SUBITEM_CASO"),IF(TRIM($C54)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D54:$H54&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I54)&lt;&gt;"",OR(LEFT(TRIM($I54),1)="A",LEFT(TRIM($I54),1)="B",LEFT(TRIM($I54),1)="C",LEFT(TRIM($I54),1)="D",LEFT(TRIM($I54),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A54)="","",IF(COUNTIF($Q54:$AJ54,"?*")=0,"OK","Falta revisar: "&amp;$Q54&amp;$R54&amp;$S54&amp;$T54&amp;$U54&amp;$V54&amp;$W54&amp;$X54&amp;$Y54&amp;$Z54&amp;$AA54&amp;$AB54&amp;$AC54&amp;$AD54&amp;$AE54&amp;$AF54&amp;$AG54&amp;$AH54&amp;$AI54&amp;$AJ54))))</x:f>
       </x:c>
       <x:c r="M54" s="341"/>
       <x:c r="N54"/>
@@ -8300,7 +8301,7 @@
         <x:f>IF(AND($A54="Verdadero o Falso Complejas",TRIM($I54)&lt;&gt;"",NOT(OR(LEFT(TRIM($I54),1)="A",LEFT(TRIM($I54),1)="B",LEFT(TRIM($I54),1)="C",LEFT(TRIM($I54),1)="D",LEFT(TRIM($I54),1)="E"))),IF(COUNTIF($Q54:$AE54,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG54" t="str">
-        <x:f>IF(AND(OR($A54="Selección de la mejor respuesta",$A54="Subítem de caso o problema"),COUNTIF($D54:$H54,"?*")&lt;5),IF(COUNTIF($Q54:$AF54,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A54="Selección de la mejor respuesta",$A54="Subítem de caso o problema"),COUNTA($D54:$H54)&lt;5),IF(COUNTIF($Q54:$AF54,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH54" t="str">
         <x:f>IF(AND(OR($A54="Selección de la mejor respuesta",$A54="Subítem de caso o problema"),TRIM($I54)&lt;&gt;"",NOT(OR(LEFT(TRIM($I54),1)="A",LEFT(TRIM($I54),1)="B",LEFT(TRIM($I54),1)="C",LEFT(TRIM($I54),1)="D",LEFT(TRIM($I54),1)="E"))),IF(COUNTIF($Q54:$AG54,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8351,7 +8352,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L55" s="347" t="str">
-        <x:f>IF(TRIM($A55)="","",IF(COUNTIF($Q55:$AJ55,"?*")=0,"OK","Falta revisar: "&amp;$Q55&amp;$R55&amp;$S55&amp;$T55&amp;$U55&amp;$V55&amp;$W55&amp;$X55&amp;$Y55&amp;$Z55&amp;$AA55&amp;$AB55&amp;$AC55&amp;$AD55&amp;$AE55&amp;$AF55&amp;$AG55&amp;$AH55&amp;$AI55&amp;$AJ55))</x:f>
+        <x:f>IF(TRIM($A55)="","",IF(OR($A55="Selección de la mejor respuesta",$A55="SELECCION_MEJOR_RESPUESTA",$A55="Subítem de caso o problema",$A55="SUBITEM_CASO"),IF(TRIM($C55)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D55:$H55&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I55)&lt;&gt;"",OR(LEFT(TRIM($I55),1)="A",LEFT(TRIM($I55),1)="B",LEFT(TRIM($I55),1)="C",LEFT(TRIM($I55),1)="D",LEFT(TRIM($I55),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A55)="","",IF(COUNTIF($Q55:$AJ55,"?*")=0,"OK","Falta revisar: "&amp;$Q55&amp;$R55&amp;$S55&amp;$T55&amp;$U55&amp;$V55&amp;$W55&amp;$X55&amp;$Y55&amp;$Z55&amp;$AA55&amp;$AB55&amp;$AC55&amp;$AD55&amp;$AE55&amp;$AF55&amp;$AG55&amp;$AH55&amp;$AI55&amp;$AJ55))))</x:f>
       </x:c>
       <x:c r="M55" s="341"/>
       <x:c r="N55"/>
@@ -8407,7 +8408,7 @@
         <x:f>IF(AND($A55="Verdadero o Falso Complejas",TRIM($I55)&lt;&gt;"",NOT(OR(LEFT(TRIM($I55),1)="A",LEFT(TRIM($I55),1)="B",LEFT(TRIM($I55),1)="C",LEFT(TRIM($I55),1)="D",LEFT(TRIM($I55),1)="E"))),IF(COUNTIF($Q55:$AE55,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG55" t="str">
-        <x:f>IF(AND(OR($A55="Selección de la mejor respuesta",$A55="Subítem de caso o problema"),COUNTIF($D55:$H55,"?*")&lt;5),IF(COUNTIF($Q55:$AF55,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A55="Selección de la mejor respuesta",$A55="Subítem de caso o problema"),COUNTA($D55:$H55)&lt;5),IF(COUNTIF($Q55:$AF55,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH55" t="str">
         <x:f>IF(AND(OR($A55="Selección de la mejor respuesta",$A55="Subítem de caso o problema"),TRIM($I55)&lt;&gt;"",NOT(OR(LEFT(TRIM($I55),1)="A",LEFT(TRIM($I55),1)="B",LEFT(TRIM($I55),1)="C",LEFT(TRIM($I55),1)="D",LEFT(TRIM($I55),1)="E"))),IF(COUNTIF($Q55:$AG55,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8458,7 +8459,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L56" s="347" t="str">
-        <x:f>IF(TRIM($A56)="","",IF(COUNTIF($Q56:$AJ56,"?*")=0,"OK","Falta revisar: "&amp;$Q56&amp;$R56&amp;$S56&amp;$T56&amp;$U56&amp;$V56&amp;$W56&amp;$X56&amp;$Y56&amp;$Z56&amp;$AA56&amp;$AB56&amp;$AC56&amp;$AD56&amp;$AE56&amp;$AF56&amp;$AG56&amp;$AH56&amp;$AI56&amp;$AJ56))</x:f>
+        <x:f>IF(TRIM($A56)="","",IF(OR($A56="Selección de la mejor respuesta",$A56="SELECCION_MEJOR_RESPUESTA",$A56="Subítem de caso o problema",$A56="SUBITEM_CASO"),IF(TRIM($C56)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D56:$H56&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I56)&lt;&gt;"",OR(LEFT(TRIM($I56),1)="A",LEFT(TRIM($I56),1)="B",LEFT(TRIM($I56),1)="C",LEFT(TRIM($I56),1)="D",LEFT(TRIM($I56),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A56)="","",IF(COUNTIF($Q56:$AJ56,"?*")=0,"OK","Falta revisar: "&amp;$Q56&amp;$R56&amp;$S56&amp;$T56&amp;$U56&amp;$V56&amp;$W56&amp;$X56&amp;$Y56&amp;$Z56&amp;$AA56&amp;$AB56&amp;$AC56&amp;$AD56&amp;$AE56&amp;$AF56&amp;$AG56&amp;$AH56&amp;$AI56&amp;$AJ56))))</x:f>
       </x:c>
       <x:c r="M56" s="341"/>
       <x:c r="N56"/>
@@ -8514,7 +8515,7 @@
         <x:f>IF(AND($A56="Verdadero o Falso Complejas",TRIM($I56)&lt;&gt;"",NOT(OR(LEFT(TRIM($I56),1)="A",LEFT(TRIM($I56),1)="B",LEFT(TRIM($I56),1)="C",LEFT(TRIM($I56),1)="D",LEFT(TRIM($I56),1)="E"))),IF(COUNTIF($Q56:$AE56,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG56" t="str">
-        <x:f>IF(AND(OR($A56="Selección de la mejor respuesta",$A56="Subítem de caso o problema"),COUNTIF($D56:$H56,"?*")&lt;5),IF(COUNTIF($Q56:$AF56,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A56="Selección de la mejor respuesta",$A56="Subítem de caso o problema"),COUNTA($D56:$H56)&lt;5),IF(COUNTIF($Q56:$AF56,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH56" t="str">
         <x:f>IF(AND(OR($A56="Selección de la mejor respuesta",$A56="Subítem de caso o problema"),TRIM($I56)&lt;&gt;"",NOT(OR(LEFT(TRIM($I56),1)="A",LEFT(TRIM($I56),1)="B",LEFT(TRIM($I56),1)="C",LEFT(TRIM($I56),1)="D",LEFT(TRIM($I56),1)="E"))),IF(COUNTIF($Q56:$AG56,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8565,7 +8566,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L57" s="347" t="str">
-        <x:f>IF(TRIM($A57)="","",IF(COUNTIF($Q57:$AJ57,"?*")=0,"OK","Falta revisar: "&amp;$Q57&amp;$R57&amp;$S57&amp;$T57&amp;$U57&amp;$V57&amp;$W57&amp;$X57&amp;$Y57&amp;$Z57&amp;$AA57&amp;$AB57&amp;$AC57&amp;$AD57&amp;$AE57&amp;$AF57&amp;$AG57&amp;$AH57&amp;$AI57&amp;$AJ57))</x:f>
+        <x:f>IF(TRIM($A57)="","",IF(OR($A57="Selección de la mejor respuesta",$A57="SELECCION_MEJOR_RESPUESTA",$A57="Subítem de caso o problema",$A57="SUBITEM_CASO"),IF(TRIM($C57)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D57:$H57&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I57)&lt;&gt;"",OR(LEFT(TRIM($I57),1)="A",LEFT(TRIM($I57),1)="B",LEFT(TRIM($I57),1)="C",LEFT(TRIM($I57),1)="D",LEFT(TRIM($I57),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A57)="","",IF(COUNTIF($Q57:$AJ57,"?*")=0,"OK","Falta revisar: "&amp;$Q57&amp;$R57&amp;$S57&amp;$T57&amp;$U57&amp;$V57&amp;$W57&amp;$X57&amp;$Y57&amp;$Z57&amp;$AA57&amp;$AB57&amp;$AC57&amp;$AD57&amp;$AE57&amp;$AF57&amp;$AG57&amp;$AH57&amp;$AI57&amp;$AJ57))))</x:f>
       </x:c>
       <x:c r="M57" s="341"/>
       <x:c r="N57"/>
@@ -8621,7 +8622,7 @@
         <x:f>IF(AND($A57="Verdadero o Falso Complejas",TRIM($I57)&lt;&gt;"",NOT(OR(LEFT(TRIM($I57),1)="A",LEFT(TRIM($I57),1)="B",LEFT(TRIM($I57),1)="C",LEFT(TRIM($I57),1)="D",LEFT(TRIM($I57),1)="E"))),IF(COUNTIF($Q57:$AE57,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG57" t="str">
-        <x:f>IF(AND(OR($A57="Selección de la mejor respuesta",$A57="Subítem de caso o problema"),COUNTIF($D57:$H57,"?*")&lt;5),IF(COUNTIF($Q57:$AF57,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A57="Selección de la mejor respuesta",$A57="Subítem de caso o problema"),COUNTA($D57:$H57)&lt;5),IF(COUNTIF($Q57:$AF57,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH57" t="str">
         <x:f>IF(AND(OR($A57="Selección de la mejor respuesta",$A57="Subítem de caso o problema"),TRIM($I57)&lt;&gt;"",NOT(OR(LEFT(TRIM($I57),1)="A",LEFT(TRIM($I57),1)="B",LEFT(TRIM($I57),1)="C",LEFT(TRIM($I57),1)="D",LEFT(TRIM($I57),1)="E"))),IF(COUNTIF($Q57:$AG57,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8672,7 +8673,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L58" s="347" t="str">
-        <x:f>IF(TRIM($A58)="","",IF(COUNTIF($Q58:$AJ58,"?*")=0,"OK","Falta revisar: "&amp;$Q58&amp;$R58&amp;$S58&amp;$T58&amp;$U58&amp;$V58&amp;$W58&amp;$X58&amp;$Y58&amp;$Z58&amp;$AA58&amp;$AB58&amp;$AC58&amp;$AD58&amp;$AE58&amp;$AF58&amp;$AG58&amp;$AH58&amp;$AI58&amp;$AJ58))</x:f>
+        <x:f>IF(TRIM($A58)="","",IF(OR($A58="Selección de la mejor respuesta",$A58="SELECCION_MEJOR_RESPUESTA",$A58="Subítem de caso o problema",$A58="SUBITEM_CASO"),IF(TRIM($C58)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D58:$H58&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I58)&lt;&gt;"",OR(LEFT(TRIM($I58),1)="A",LEFT(TRIM($I58),1)="B",LEFT(TRIM($I58),1)="C",LEFT(TRIM($I58),1)="D",LEFT(TRIM($I58),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A58)="","",IF(COUNTIF($Q58:$AJ58,"?*")=0,"OK","Falta revisar: "&amp;$Q58&amp;$R58&amp;$S58&amp;$T58&amp;$U58&amp;$V58&amp;$W58&amp;$X58&amp;$Y58&amp;$Z58&amp;$AA58&amp;$AB58&amp;$AC58&amp;$AD58&amp;$AE58&amp;$AF58&amp;$AG58&amp;$AH58&amp;$AI58&amp;$AJ58))))</x:f>
       </x:c>
       <x:c r="M58" s="341"/>
       <x:c r="N58"/>
@@ -8728,7 +8729,7 @@
         <x:f>IF(AND($A58="Verdadero o Falso Complejas",TRIM($I58)&lt;&gt;"",NOT(OR(LEFT(TRIM($I58),1)="A",LEFT(TRIM($I58),1)="B",LEFT(TRIM($I58),1)="C",LEFT(TRIM($I58),1)="D",LEFT(TRIM($I58),1)="E"))),IF(COUNTIF($Q58:$AE58,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG58" t="str">
-        <x:f>IF(AND(OR($A58="Selección de la mejor respuesta",$A58="Subítem de caso o problema"),COUNTIF($D58:$H58,"?*")&lt;5),IF(COUNTIF($Q58:$AF58,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A58="Selección de la mejor respuesta",$A58="Subítem de caso o problema"),COUNTA($D58:$H58)&lt;5),IF(COUNTIF($Q58:$AF58,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH58" t="str">
         <x:f>IF(AND(OR($A58="Selección de la mejor respuesta",$A58="Subítem de caso o problema"),TRIM($I58)&lt;&gt;"",NOT(OR(LEFT(TRIM($I58),1)="A",LEFT(TRIM($I58),1)="B",LEFT(TRIM($I58),1)="C",LEFT(TRIM($I58),1)="D",LEFT(TRIM($I58),1)="E"))),IF(COUNTIF($Q58:$AG58,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8779,7 +8780,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L59" s="347" t="str">
-        <x:f>IF(TRIM($A59)="","",IF(COUNTIF($Q59:$AJ59,"?*")=0,"OK","Falta revisar: "&amp;$Q59&amp;$R59&amp;$S59&amp;$T59&amp;$U59&amp;$V59&amp;$W59&amp;$X59&amp;$Y59&amp;$Z59&amp;$AA59&amp;$AB59&amp;$AC59&amp;$AD59&amp;$AE59&amp;$AF59&amp;$AG59&amp;$AH59&amp;$AI59&amp;$AJ59))</x:f>
+        <x:f>IF(TRIM($A59)="","",IF(OR($A59="Selección de la mejor respuesta",$A59="SELECCION_MEJOR_RESPUESTA",$A59="Subítem de caso o problema",$A59="SUBITEM_CASO"),IF(TRIM($C59)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D59:$H59&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I59)&lt;&gt;"",OR(LEFT(TRIM($I59),1)="A",LEFT(TRIM($I59),1)="B",LEFT(TRIM($I59),1)="C",LEFT(TRIM($I59),1)="D",LEFT(TRIM($I59),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A59)="","",IF(COUNTIF($Q59:$AJ59,"?*")=0,"OK","Falta revisar: "&amp;$Q59&amp;$R59&amp;$S59&amp;$T59&amp;$U59&amp;$V59&amp;$W59&amp;$X59&amp;$Y59&amp;$Z59&amp;$AA59&amp;$AB59&amp;$AC59&amp;$AD59&amp;$AE59&amp;$AF59&amp;$AG59&amp;$AH59&amp;$AI59&amp;$AJ59))))</x:f>
       </x:c>
       <x:c r="M59" s="341"/>
       <x:c r="N59"/>
@@ -8835,7 +8836,7 @@
         <x:f>IF(AND($A59="Verdadero o Falso Complejas",TRIM($I59)&lt;&gt;"",NOT(OR(LEFT(TRIM($I59),1)="A",LEFT(TRIM($I59),1)="B",LEFT(TRIM($I59),1)="C",LEFT(TRIM($I59),1)="D",LEFT(TRIM($I59),1)="E"))),IF(COUNTIF($Q59:$AE59,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG59" t="str">
-        <x:f>IF(AND(OR($A59="Selección de la mejor respuesta",$A59="Subítem de caso o problema"),COUNTIF($D59:$H59,"?*")&lt;5),IF(COUNTIF($Q59:$AF59,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A59="Selección de la mejor respuesta",$A59="Subítem de caso o problema"),COUNTA($D59:$H59)&lt;5),IF(COUNTIF($Q59:$AF59,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH59" t="str">
         <x:f>IF(AND(OR($A59="Selección de la mejor respuesta",$A59="Subítem de caso o problema"),TRIM($I59)&lt;&gt;"",NOT(OR(LEFT(TRIM($I59),1)="A",LEFT(TRIM($I59),1)="B",LEFT(TRIM($I59),1)="C",LEFT(TRIM($I59),1)="D",LEFT(TRIM($I59),1)="E"))),IF(COUNTIF($Q59:$AG59,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8886,7 +8887,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L60" s="347" t="str">
-        <x:f>IF(TRIM($A60)="","",IF(COUNTIF($Q60:$AJ60,"?*")=0,"OK","Falta revisar: "&amp;$Q60&amp;$R60&amp;$S60&amp;$T60&amp;$U60&amp;$V60&amp;$W60&amp;$X60&amp;$Y60&amp;$Z60&amp;$AA60&amp;$AB60&amp;$AC60&amp;$AD60&amp;$AE60&amp;$AF60&amp;$AG60&amp;$AH60&amp;$AI60&amp;$AJ60))</x:f>
+        <x:f>IF(TRIM($A60)="","",IF(OR($A60="Selección de la mejor respuesta",$A60="SELECCION_MEJOR_RESPUESTA",$A60="Subítem de caso o problema",$A60="SUBITEM_CASO"),IF(TRIM($C60)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D60:$H60&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I60)&lt;&gt;"",OR(LEFT(TRIM($I60),1)="A",LEFT(TRIM($I60),1)="B",LEFT(TRIM($I60),1)="C",LEFT(TRIM($I60),1)="D",LEFT(TRIM($I60),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A60)="","",IF(COUNTIF($Q60:$AJ60,"?*")=0,"OK","Falta revisar: "&amp;$Q60&amp;$R60&amp;$S60&amp;$T60&amp;$U60&amp;$V60&amp;$W60&amp;$X60&amp;$Y60&amp;$Z60&amp;$AA60&amp;$AB60&amp;$AC60&amp;$AD60&amp;$AE60&amp;$AF60&amp;$AG60&amp;$AH60&amp;$AI60&amp;$AJ60))))</x:f>
       </x:c>
       <x:c r="M60" s="341"/>
       <x:c r="N60"/>
@@ -8942,7 +8943,7 @@
         <x:f>IF(AND($A60="Verdadero o Falso Complejas",TRIM($I60)&lt;&gt;"",NOT(OR(LEFT(TRIM($I60),1)="A",LEFT(TRIM($I60),1)="B",LEFT(TRIM($I60),1)="C",LEFT(TRIM($I60),1)="D",LEFT(TRIM($I60),1)="E"))),IF(COUNTIF($Q60:$AE60,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG60" t="str">
-        <x:f>IF(AND(OR($A60="Selección de la mejor respuesta",$A60="Subítem de caso o problema"),COUNTIF($D60:$H60,"?*")&lt;5),IF(COUNTIF($Q60:$AF60,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A60="Selección de la mejor respuesta",$A60="Subítem de caso o problema"),COUNTA($D60:$H60)&lt;5),IF(COUNTIF($Q60:$AF60,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH60" t="str">
         <x:f>IF(AND(OR($A60="Selección de la mejor respuesta",$A60="Subítem de caso o problema"),TRIM($I60)&lt;&gt;"",NOT(OR(LEFT(TRIM($I60),1)="A",LEFT(TRIM($I60),1)="B",LEFT(TRIM($I60),1)="C",LEFT(TRIM($I60),1)="D",LEFT(TRIM($I60),1)="E"))),IF(COUNTIF($Q60:$AG60,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -8993,7 +8994,7 @@
         <x:v>1P</x:v>
       </x:c>
       <x:c r="L61" s="347" t="str">
-        <x:f>IF(TRIM($A61)="","",IF(COUNTIF($Q61:$AJ61,"?*")=0,"OK","Falta revisar: "&amp;$Q61&amp;$R61&amp;$S61&amp;$T61&amp;$U61&amp;$V61&amp;$W61&amp;$X61&amp;$Y61&amp;$Z61&amp;$AA61&amp;$AB61&amp;$AC61&amp;$AD61&amp;$AE61&amp;$AF61&amp;$AG61&amp;$AH61&amp;$AI61&amp;$AJ61))</x:f>
+        <x:f>IF(TRIM($A61)="","",IF(OR($A61="Selección de la mejor respuesta",$A61="SELECCION_MEJOR_RESPUESTA",$A61="Subítem de caso o problema",$A61="SUBITEM_CASO"),IF(TRIM($C61)="","Completar enunciado",IF(SUMPRODUCT(--(LEN(TRIM($D61:$H61&amp;""))&gt;0))&lt;5,"Completar opciones A-E",IF(AND(TRIM($I61)&lt;&gt;"",OR(LEFT(TRIM($I61),1)="A",LEFT(TRIM($I61),1)="B",LEFT(TRIM($I61),1)="C",LEFT(TRIM($I61),1)="D",LEFT(TRIM($I61),1)="E")),"OK","Completar respuesta correcta A-E"))),IF(TRIM($A61)="","",IF(COUNTIF($Q61:$AJ61,"?*")=0,"OK","Falta revisar: "&amp;$Q61&amp;$R61&amp;$S61&amp;$T61&amp;$U61&amp;$V61&amp;$W61&amp;$X61&amp;$Y61&amp;$Z61&amp;$AA61&amp;$AB61&amp;$AC61&amp;$AD61&amp;$AE61&amp;$AF61&amp;$AG61&amp;$AH61&amp;$AI61&amp;$AJ61))))</x:f>
       </x:c>
       <x:c r="M61" s="341"/>
       <x:c r="N61"/>
@@ -9049,7 +9050,7 @@
         <x:f>IF(AND($A61="Verdadero o Falso Complejas",TRIM($I61)&lt;&gt;"",NOT(OR(LEFT(TRIM($I61),1)="A",LEFT(TRIM($I61),1)="B",LEFT(TRIM($I61),1)="C",LEFT(TRIM($I61),1)="D",LEFT(TRIM($I61),1)="E"))),IF(COUNTIF($Q61:$AE61,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
       </x:c>
       <x:c r="AG61" t="str">
-        <x:f>IF(AND(OR($A61="Selección de la mejor respuesta",$A61="Subítem de caso o problema"),COUNTIF($D61:$H61,"?*")&lt;5),IF(COUNTIF($Q61:$AF61,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
+        <x:f>IF(AND(OR($A61="Selección de la mejor respuesta",$A61="Subítem de caso o problema"),COUNTA($D61:$H61)&lt;5),IF(COUNTIF($Q61:$AF61,"?*")&gt;0,", ","")&amp;"incisos A-E","")</x:f>
       </x:c>
       <x:c r="AH61" t="str">
         <x:f>IF(AND(OR($A61="Selección de la mejor respuesta",$A61="Subítem de caso o problema"),TRIM($I61)&lt;&gt;"",NOT(OR(LEFT(TRIM($I61),1)="A",LEFT(TRIM($I61),1)="B",LEFT(TRIM($I61),1)="C",LEFT(TRIM($I61),1)="D",LEFT(TRIM($I61),1)="E"))),IF(COUNTIF($Q61:$AG61,"?*")&gt;0,", ","")&amp;"respuesta A-E","")</x:f>
@@ -12190,1264 +12191,1264 @@
   </x:conditionalFormatting>
   <x:dataValidations count="481">
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B10">
-      <x:formula1>IF(ISNUMBER(MATCH($A10,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B10))&gt;0,LEN(TRIM($B10))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A10,TIPOS_REQUIEREN_GRUPO,0)),OR($A10="CASO_CLINICO_TRONCO",$A10="CASO_CLINICO",$A10="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A10="PROBLEMA",$A10="SUBPROBLEMA",$A10="SUBITEM_CASO",$A10="SUBITEM_DE_CASO_O_PROBLEMA",$A10="EMPAREJAMIENTO_TRONCO",$A10="EMPAREJAMIENTO_AMPLIADO",$A10="EMPAREJAMIENTO_DE_CONCEPTOS",$A10="OPCION_EMPAREJAMIENTO",$A10="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B10))&gt;0,LEN(TRIM($B10))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B11">
-      <x:formula1>IF(ISNUMBER(MATCH($A11,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B11))&gt;0,LEN(TRIM($B11))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A11,TIPOS_REQUIEREN_GRUPO,0)),OR($A11="CASO_CLINICO_TRONCO",$A11="CASO_CLINICO",$A11="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A11="PROBLEMA",$A11="SUBPROBLEMA",$A11="SUBITEM_CASO",$A11="SUBITEM_DE_CASO_O_PROBLEMA",$A11="EMPAREJAMIENTO_TRONCO",$A11="EMPAREJAMIENTO_AMPLIADO",$A11="EMPAREJAMIENTO_DE_CONCEPTOS",$A11="OPCION_EMPAREJAMIENTO",$A11="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B11))&gt;0,LEN(TRIM($B11))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B12">
-      <x:formula1>IF(ISNUMBER(MATCH($A12,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B12))&gt;0,LEN(TRIM($B12))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A12,TIPOS_REQUIEREN_GRUPO,0)),OR($A12="CASO_CLINICO_TRONCO",$A12="CASO_CLINICO",$A12="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A12="PROBLEMA",$A12="SUBPROBLEMA",$A12="SUBITEM_CASO",$A12="SUBITEM_DE_CASO_O_PROBLEMA",$A12="EMPAREJAMIENTO_TRONCO",$A12="EMPAREJAMIENTO_AMPLIADO",$A12="EMPAREJAMIENTO_DE_CONCEPTOS",$A12="OPCION_EMPAREJAMIENTO",$A12="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B12))&gt;0,LEN(TRIM($B12))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B13">
-      <x:formula1>IF(ISNUMBER(MATCH($A13,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B13))&gt;0,LEN(TRIM($B13))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A13,TIPOS_REQUIEREN_GRUPO,0)),OR($A13="CASO_CLINICO_TRONCO",$A13="CASO_CLINICO",$A13="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A13="PROBLEMA",$A13="SUBPROBLEMA",$A13="SUBITEM_CASO",$A13="SUBITEM_DE_CASO_O_PROBLEMA",$A13="EMPAREJAMIENTO_TRONCO",$A13="EMPAREJAMIENTO_AMPLIADO",$A13="EMPAREJAMIENTO_DE_CONCEPTOS",$A13="OPCION_EMPAREJAMIENTO",$A13="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B13))&gt;0,LEN(TRIM($B13))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B14">
-      <x:formula1>IF(ISNUMBER(MATCH($A14,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B14))&gt;0,LEN(TRIM($B14))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A14,TIPOS_REQUIEREN_GRUPO,0)),OR($A14="CASO_CLINICO_TRONCO",$A14="CASO_CLINICO",$A14="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A14="PROBLEMA",$A14="SUBPROBLEMA",$A14="SUBITEM_CASO",$A14="SUBITEM_DE_CASO_O_PROBLEMA",$A14="EMPAREJAMIENTO_TRONCO",$A14="EMPAREJAMIENTO_AMPLIADO",$A14="EMPAREJAMIENTO_DE_CONCEPTOS",$A14="OPCION_EMPAREJAMIENTO",$A14="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B14))&gt;0,LEN(TRIM($B14))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B15">
-      <x:formula1>IF(ISNUMBER(MATCH($A15,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B15))&gt;0,LEN(TRIM($B15))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A15,TIPOS_REQUIEREN_GRUPO,0)),OR($A15="CASO_CLINICO_TRONCO",$A15="CASO_CLINICO",$A15="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A15="PROBLEMA",$A15="SUBPROBLEMA",$A15="SUBITEM_CASO",$A15="SUBITEM_DE_CASO_O_PROBLEMA",$A15="EMPAREJAMIENTO_TRONCO",$A15="EMPAREJAMIENTO_AMPLIADO",$A15="EMPAREJAMIENTO_DE_CONCEPTOS",$A15="OPCION_EMPAREJAMIENTO",$A15="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B15))&gt;0,LEN(TRIM($B15))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B16">
-      <x:formula1>IF(ISNUMBER(MATCH($A16,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B16))&gt;0,LEN(TRIM($B16))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A16,TIPOS_REQUIEREN_GRUPO,0)),OR($A16="CASO_CLINICO_TRONCO",$A16="CASO_CLINICO",$A16="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A16="PROBLEMA",$A16="SUBPROBLEMA",$A16="SUBITEM_CASO",$A16="SUBITEM_DE_CASO_O_PROBLEMA",$A16="EMPAREJAMIENTO_TRONCO",$A16="EMPAREJAMIENTO_AMPLIADO",$A16="EMPAREJAMIENTO_DE_CONCEPTOS",$A16="OPCION_EMPAREJAMIENTO",$A16="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B16))&gt;0,LEN(TRIM($B16))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B17">
-      <x:formula1>IF(ISNUMBER(MATCH($A17,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B17))&gt;0,LEN(TRIM($B17))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A17,TIPOS_REQUIEREN_GRUPO,0)),OR($A17="CASO_CLINICO_TRONCO",$A17="CASO_CLINICO",$A17="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A17="PROBLEMA",$A17="SUBPROBLEMA",$A17="SUBITEM_CASO",$A17="SUBITEM_DE_CASO_O_PROBLEMA",$A17="EMPAREJAMIENTO_TRONCO",$A17="EMPAREJAMIENTO_AMPLIADO",$A17="EMPAREJAMIENTO_DE_CONCEPTOS",$A17="OPCION_EMPAREJAMIENTO",$A17="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B17))&gt;0,LEN(TRIM($B17))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B18">
-      <x:formula1>IF(ISNUMBER(MATCH($A18,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B18))&gt;0,LEN(TRIM($B18))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A18,TIPOS_REQUIEREN_GRUPO,0)),OR($A18="CASO_CLINICO_TRONCO",$A18="CASO_CLINICO",$A18="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A18="PROBLEMA",$A18="SUBPROBLEMA",$A18="SUBITEM_CASO",$A18="SUBITEM_DE_CASO_O_PROBLEMA",$A18="EMPAREJAMIENTO_TRONCO",$A18="EMPAREJAMIENTO_AMPLIADO",$A18="EMPAREJAMIENTO_DE_CONCEPTOS",$A18="OPCION_EMPAREJAMIENTO",$A18="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B18))&gt;0,LEN(TRIM($B18))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B19">
-      <x:formula1>IF(ISNUMBER(MATCH($A19,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B19))&gt;0,LEN(TRIM($B19))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A19,TIPOS_REQUIEREN_GRUPO,0)),OR($A19="CASO_CLINICO_TRONCO",$A19="CASO_CLINICO",$A19="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A19="PROBLEMA",$A19="SUBPROBLEMA",$A19="SUBITEM_CASO",$A19="SUBITEM_DE_CASO_O_PROBLEMA",$A19="EMPAREJAMIENTO_TRONCO",$A19="EMPAREJAMIENTO_AMPLIADO",$A19="EMPAREJAMIENTO_DE_CONCEPTOS",$A19="OPCION_EMPAREJAMIENTO",$A19="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B19))&gt;0,LEN(TRIM($B19))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B2">
-      <x:formula1>IF(ISNUMBER(MATCH($A2,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B2))&gt;0,LEN(TRIM($B2))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A2,TIPOS_REQUIEREN_GRUPO,0)),OR($A2="CASO_CLINICO_TRONCO",$A2="CASO_CLINICO",$A2="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A2="PROBLEMA",$A2="SUBPROBLEMA",$A2="SUBITEM_CASO",$A2="SUBITEM_DE_CASO_O_PROBLEMA",$A2="EMPAREJAMIENTO_TRONCO",$A2="EMPAREJAMIENTO_AMPLIADO",$A2="EMPAREJAMIENTO_DE_CONCEPTOS",$A2="OPCION_EMPAREJAMIENTO",$A2="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B2))&gt;0,LEN(TRIM($B2))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B20">
-      <x:formula1>IF(ISNUMBER(MATCH($A20,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B20))&gt;0,LEN(TRIM($B20))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A20,TIPOS_REQUIEREN_GRUPO,0)),OR($A20="CASO_CLINICO_TRONCO",$A20="CASO_CLINICO",$A20="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A20="PROBLEMA",$A20="SUBPROBLEMA",$A20="SUBITEM_CASO",$A20="SUBITEM_DE_CASO_O_PROBLEMA",$A20="EMPAREJAMIENTO_TRONCO",$A20="EMPAREJAMIENTO_AMPLIADO",$A20="EMPAREJAMIENTO_DE_CONCEPTOS",$A20="OPCION_EMPAREJAMIENTO",$A20="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B20))&gt;0,LEN(TRIM($B20))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B21">
-      <x:formula1>IF(ISNUMBER(MATCH($A21,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B21))&gt;0,LEN(TRIM($B21))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A21,TIPOS_REQUIEREN_GRUPO,0)),OR($A21="CASO_CLINICO_TRONCO",$A21="CASO_CLINICO",$A21="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A21="PROBLEMA",$A21="SUBPROBLEMA",$A21="SUBITEM_CASO",$A21="SUBITEM_DE_CASO_O_PROBLEMA",$A21="EMPAREJAMIENTO_TRONCO",$A21="EMPAREJAMIENTO_AMPLIADO",$A21="EMPAREJAMIENTO_DE_CONCEPTOS",$A21="OPCION_EMPAREJAMIENTO",$A21="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B21))&gt;0,LEN(TRIM($B21))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B22">
-      <x:formula1>IF(ISNUMBER(MATCH($A22,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B22))&gt;0,LEN(TRIM($B22))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A22,TIPOS_REQUIEREN_GRUPO,0)),OR($A22="CASO_CLINICO_TRONCO",$A22="CASO_CLINICO",$A22="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A22="PROBLEMA",$A22="SUBPROBLEMA",$A22="SUBITEM_CASO",$A22="SUBITEM_DE_CASO_O_PROBLEMA",$A22="EMPAREJAMIENTO_TRONCO",$A22="EMPAREJAMIENTO_AMPLIADO",$A22="EMPAREJAMIENTO_DE_CONCEPTOS",$A22="OPCION_EMPAREJAMIENTO",$A22="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B22))&gt;0,LEN(TRIM($B22))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B23">
-      <x:formula1>IF(ISNUMBER(MATCH($A23,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B23))&gt;0,LEN(TRIM($B23))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A23,TIPOS_REQUIEREN_GRUPO,0)),OR($A23="CASO_CLINICO_TRONCO",$A23="CASO_CLINICO",$A23="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A23="PROBLEMA",$A23="SUBPROBLEMA",$A23="SUBITEM_CASO",$A23="SUBITEM_DE_CASO_O_PROBLEMA",$A23="EMPAREJAMIENTO_TRONCO",$A23="EMPAREJAMIENTO_AMPLIADO",$A23="EMPAREJAMIENTO_DE_CONCEPTOS",$A23="OPCION_EMPAREJAMIENTO",$A23="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B23))&gt;0,LEN(TRIM($B23))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B24">
-      <x:formula1>IF(ISNUMBER(MATCH($A24,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B24))&gt;0,LEN(TRIM($B24))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A24,TIPOS_REQUIEREN_GRUPO,0)),OR($A24="CASO_CLINICO_TRONCO",$A24="CASO_CLINICO",$A24="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A24="PROBLEMA",$A24="SUBPROBLEMA",$A24="SUBITEM_CASO",$A24="SUBITEM_DE_CASO_O_PROBLEMA",$A24="EMPAREJAMIENTO_TRONCO",$A24="EMPAREJAMIENTO_AMPLIADO",$A24="EMPAREJAMIENTO_DE_CONCEPTOS",$A24="OPCION_EMPAREJAMIENTO",$A24="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B24))&gt;0,LEN(TRIM($B24))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B25">
-      <x:formula1>IF(ISNUMBER(MATCH($A25,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B25))&gt;0,LEN(TRIM($B25))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A25,TIPOS_REQUIEREN_GRUPO,0)),OR($A25="CASO_CLINICO_TRONCO",$A25="CASO_CLINICO",$A25="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A25="PROBLEMA",$A25="SUBPROBLEMA",$A25="SUBITEM_CASO",$A25="SUBITEM_DE_CASO_O_PROBLEMA",$A25="EMPAREJAMIENTO_TRONCO",$A25="EMPAREJAMIENTO_AMPLIADO",$A25="EMPAREJAMIENTO_DE_CONCEPTOS",$A25="OPCION_EMPAREJAMIENTO",$A25="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B25))&gt;0,LEN(TRIM($B25))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B26">
-      <x:formula1>IF(ISNUMBER(MATCH($A26,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B26))&gt;0,LEN(TRIM($B26))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A26,TIPOS_REQUIEREN_GRUPO,0)),OR($A26="CASO_CLINICO_TRONCO",$A26="CASO_CLINICO",$A26="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A26="PROBLEMA",$A26="SUBPROBLEMA",$A26="SUBITEM_CASO",$A26="SUBITEM_DE_CASO_O_PROBLEMA",$A26="EMPAREJAMIENTO_TRONCO",$A26="EMPAREJAMIENTO_AMPLIADO",$A26="EMPAREJAMIENTO_DE_CONCEPTOS",$A26="OPCION_EMPAREJAMIENTO",$A26="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B26))&gt;0,LEN(TRIM($B26))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B27">
-      <x:formula1>IF(ISNUMBER(MATCH($A27,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B27))&gt;0,LEN(TRIM($B27))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A27,TIPOS_REQUIEREN_GRUPO,0)),OR($A27="CASO_CLINICO_TRONCO",$A27="CASO_CLINICO",$A27="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A27="PROBLEMA",$A27="SUBPROBLEMA",$A27="SUBITEM_CASO",$A27="SUBITEM_DE_CASO_O_PROBLEMA",$A27="EMPAREJAMIENTO_TRONCO",$A27="EMPAREJAMIENTO_AMPLIADO",$A27="EMPAREJAMIENTO_DE_CONCEPTOS",$A27="OPCION_EMPAREJAMIENTO",$A27="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B27))&gt;0,LEN(TRIM($B27))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B28">
-      <x:formula1>IF(ISNUMBER(MATCH($A28,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B28))&gt;0,LEN(TRIM($B28))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A28,TIPOS_REQUIEREN_GRUPO,0)),OR($A28="CASO_CLINICO_TRONCO",$A28="CASO_CLINICO",$A28="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A28="PROBLEMA",$A28="SUBPROBLEMA",$A28="SUBITEM_CASO",$A28="SUBITEM_DE_CASO_O_PROBLEMA",$A28="EMPAREJAMIENTO_TRONCO",$A28="EMPAREJAMIENTO_AMPLIADO",$A28="EMPAREJAMIENTO_DE_CONCEPTOS",$A28="OPCION_EMPAREJAMIENTO",$A28="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B28))&gt;0,LEN(TRIM($B28))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B29">
-      <x:formula1>IF(ISNUMBER(MATCH($A29,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B29))&gt;0,LEN(TRIM($B29))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A29,TIPOS_REQUIEREN_GRUPO,0)),OR($A29="CASO_CLINICO_TRONCO",$A29="CASO_CLINICO",$A29="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A29="PROBLEMA",$A29="SUBPROBLEMA",$A29="SUBITEM_CASO",$A29="SUBITEM_DE_CASO_O_PROBLEMA",$A29="EMPAREJAMIENTO_TRONCO",$A29="EMPAREJAMIENTO_AMPLIADO",$A29="EMPAREJAMIENTO_DE_CONCEPTOS",$A29="OPCION_EMPAREJAMIENTO",$A29="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B29))&gt;0,LEN(TRIM($B29))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B3">
-      <x:formula1>IF(ISNUMBER(MATCH($A3,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B3))&gt;0,LEN(TRIM($B3))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A3,TIPOS_REQUIEREN_GRUPO,0)),OR($A3="CASO_CLINICO_TRONCO",$A3="CASO_CLINICO",$A3="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A3="PROBLEMA",$A3="SUBPROBLEMA",$A3="SUBITEM_CASO",$A3="SUBITEM_DE_CASO_O_PROBLEMA",$A3="EMPAREJAMIENTO_TRONCO",$A3="EMPAREJAMIENTO_AMPLIADO",$A3="EMPAREJAMIENTO_DE_CONCEPTOS",$A3="OPCION_EMPAREJAMIENTO",$A3="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B3))&gt;0,LEN(TRIM($B3))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B30">
-      <x:formula1>IF(ISNUMBER(MATCH($A30,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B30))&gt;0,LEN(TRIM($B30))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A30,TIPOS_REQUIEREN_GRUPO,0)),OR($A30="CASO_CLINICO_TRONCO",$A30="CASO_CLINICO",$A30="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A30="PROBLEMA",$A30="SUBPROBLEMA",$A30="SUBITEM_CASO",$A30="SUBITEM_DE_CASO_O_PROBLEMA",$A30="EMPAREJAMIENTO_TRONCO",$A30="EMPAREJAMIENTO_AMPLIADO",$A30="EMPAREJAMIENTO_DE_CONCEPTOS",$A30="OPCION_EMPAREJAMIENTO",$A30="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B30))&gt;0,LEN(TRIM($B30))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B31">
-      <x:formula1>IF(ISNUMBER(MATCH($A31,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B31))&gt;0,LEN(TRIM($B31))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A31,TIPOS_REQUIEREN_GRUPO,0)),OR($A31="CASO_CLINICO_TRONCO",$A31="CASO_CLINICO",$A31="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A31="PROBLEMA",$A31="SUBPROBLEMA",$A31="SUBITEM_CASO",$A31="SUBITEM_DE_CASO_O_PROBLEMA",$A31="EMPAREJAMIENTO_TRONCO",$A31="EMPAREJAMIENTO_AMPLIADO",$A31="EMPAREJAMIENTO_DE_CONCEPTOS",$A31="OPCION_EMPAREJAMIENTO",$A31="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B31))&gt;0,LEN(TRIM($B31))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B32">
-      <x:formula1>IF(ISNUMBER(MATCH($A32,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B32))&gt;0,LEN(TRIM($B32))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A32,TIPOS_REQUIEREN_GRUPO,0)),OR($A32="CASO_CLINICO_TRONCO",$A32="CASO_CLINICO",$A32="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A32="PROBLEMA",$A32="SUBPROBLEMA",$A32="SUBITEM_CASO",$A32="SUBITEM_DE_CASO_O_PROBLEMA",$A32="EMPAREJAMIENTO_TRONCO",$A32="EMPAREJAMIENTO_AMPLIADO",$A32="EMPAREJAMIENTO_DE_CONCEPTOS",$A32="OPCION_EMPAREJAMIENTO",$A32="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B32))&gt;0,LEN(TRIM($B32))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B33">
-      <x:formula1>IF(ISNUMBER(MATCH($A33,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B33))&gt;0,LEN(TRIM($B33))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A33,TIPOS_REQUIEREN_GRUPO,0)),OR($A33="CASO_CLINICO_TRONCO",$A33="CASO_CLINICO",$A33="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A33="PROBLEMA",$A33="SUBPROBLEMA",$A33="SUBITEM_CASO",$A33="SUBITEM_DE_CASO_O_PROBLEMA",$A33="EMPAREJAMIENTO_TRONCO",$A33="EMPAREJAMIENTO_AMPLIADO",$A33="EMPAREJAMIENTO_DE_CONCEPTOS",$A33="OPCION_EMPAREJAMIENTO",$A33="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B33))&gt;0,LEN(TRIM($B33))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B34">
-      <x:formula1>IF(ISNUMBER(MATCH($A34,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B34))&gt;0,LEN(TRIM($B34))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A34,TIPOS_REQUIEREN_GRUPO,0)),OR($A34="CASO_CLINICO_TRONCO",$A34="CASO_CLINICO",$A34="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A34="PROBLEMA",$A34="SUBPROBLEMA",$A34="SUBITEM_CASO",$A34="SUBITEM_DE_CASO_O_PROBLEMA",$A34="EMPAREJAMIENTO_TRONCO",$A34="EMPAREJAMIENTO_AMPLIADO",$A34="EMPAREJAMIENTO_DE_CONCEPTOS",$A34="OPCION_EMPAREJAMIENTO",$A34="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B34))&gt;0,LEN(TRIM($B34))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B35">
-      <x:formula1>IF(ISNUMBER(MATCH($A35,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B35))&gt;0,LEN(TRIM($B35))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A35,TIPOS_REQUIEREN_GRUPO,0)),OR($A35="CASO_CLINICO_TRONCO",$A35="CASO_CLINICO",$A35="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A35="PROBLEMA",$A35="SUBPROBLEMA",$A35="SUBITEM_CASO",$A35="SUBITEM_DE_CASO_O_PROBLEMA",$A35="EMPAREJAMIENTO_TRONCO",$A35="EMPAREJAMIENTO_AMPLIADO",$A35="EMPAREJAMIENTO_DE_CONCEPTOS",$A35="OPCION_EMPAREJAMIENTO",$A35="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B35))&gt;0,LEN(TRIM($B35))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B36">
-      <x:formula1>IF(ISNUMBER(MATCH($A36,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B36))&gt;0,LEN(TRIM($B36))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A36,TIPOS_REQUIEREN_GRUPO,0)),OR($A36="CASO_CLINICO_TRONCO",$A36="CASO_CLINICO",$A36="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A36="PROBLEMA",$A36="SUBPROBLEMA",$A36="SUBITEM_CASO",$A36="SUBITEM_DE_CASO_O_PROBLEMA",$A36="EMPAREJAMIENTO_TRONCO",$A36="EMPAREJAMIENTO_AMPLIADO",$A36="EMPAREJAMIENTO_DE_CONCEPTOS",$A36="OPCION_EMPAREJAMIENTO",$A36="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B36))&gt;0,LEN(TRIM($B36))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B37">
-      <x:formula1>IF(ISNUMBER(MATCH($A37,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B37))&gt;0,LEN(TRIM($B37))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A37,TIPOS_REQUIEREN_GRUPO,0)),OR($A37="CASO_CLINICO_TRONCO",$A37="CASO_CLINICO",$A37="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A37="PROBLEMA",$A37="SUBPROBLEMA",$A37="SUBITEM_CASO",$A37="SUBITEM_DE_CASO_O_PROBLEMA",$A37="EMPAREJAMIENTO_TRONCO",$A37="EMPAREJAMIENTO_AMPLIADO",$A37="EMPAREJAMIENTO_DE_CONCEPTOS",$A37="OPCION_EMPAREJAMIENTO",$A37="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B37))&gt;0,LEN(TRIM($B37))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B38">
-      <x:formula1>IF(ISNUMBER(MATCH($A38,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B38))&gt;0,LEN(TRIM($B38))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A38,TIPOS_REQUIEREN_GRUPO,0)),OR($A38="CASO_CLINICO_TRONCO",$A38="CASO_CLINICO",$A38="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A38="PROBLEMA",$A38="SUBPROBLEMA",$A38="SUBITEM_CASO",$A38="SUBITEM_DE_CASO_O_PROBLEMA",$A38="EMPAREJAMIENTO_TRONCO",$A38="EMPAREJAMIENTO_AMPLIADO",$A38="EMPAREJAMIENTO_DE_CONCEPTOS",$A38="OPCION_EMPAREJAMIENTO",$A38="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B38))&gt;0,LEN(TRIM($B38))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B39">
-      <x:formula1>IF(ISNUMBER(MATCH($A39,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B39))&gt;0,LEN(TRIM($B39))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A39,TIPOS_REQUIEREN_GRUPO,0)),OR($A39="CASO_CLINICO_TRONCO",$A39="CASO_CLINICO",$A39="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A39="PROBLEMA",$A39="SUBPROBLEMA",$A39="SUBITEM_CASO",$A39="SUBITEM_DE_CASO_O_PROBLEMA",$A39="EMPAREJAMIENTO_TRONCO",$A39="EMPAREJAMIENTO_AMPLIADO",$A39="EMPAREJAMIENTO_DE_CONCEPTOS",$A39="OPCION_EMPAREJAMIENTO",$A39="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B39))&gt;0,LEN(TRIM($B39))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B4">
-      <x:formula1>IF(ISNUMBER(MATCH($A4,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B4))&gt;0,LEN(TRIM($B4))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A4,TIPOS_REQUIEREN_GRUPO,0)),OR($A4="CASO_CLINICO_TRONCO",$A4="CASO_CLINICO",$A4="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A4="PROBLEMA",$A4="SUBPROBLEMA",$A4="SUBITEM_CASO",$A4="SUBITEM_DE_CASO_O_PROBLEMA",$A4="EMPAREJAMIENTO_TRONCO",$A4="EMPAREJAMIENTO_AMPLIADO",$A4="EMPAREJAMIENTO_DE_CONCEPTOS",$A4="OPCION_EMPAREJAMIENTO",$A4="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B4))&gt;0,LEN(TRIM($B4))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B40">
-      <x:formula1>IF(ISNUMBER(MATCH($A40,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B40))&gt;0,LEN(TRIM($B40))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A40,TIPOS_REQUIEREN_GRUPO,0)),OR($A40="CASO_CLINICO_TRONCO",$A40="CASO_CLINICO",$A40="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A40="PROBLEMA",$A40="SUBPROBLEMA",$A40="SUBITEM_CASO",$A40="SUBITEM_DE_CASO_O_PROBLEMA",$A40="EMPAREJAMIENTO_TRONCO",$A40="EMPAREJAMIENTO_AMPLIADO",$A40="EMPAREJAMIENTO_DE_CONCEPTOS",$A40="OPCION_EMPAREJAMIENTO",$A40="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B40))&gt;0,LEN(TRIM($B40))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B41">
-      <x:formula1>IF(ISNUMBER(MATCH($A41,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B41))&gt;0,LEN(TRIM($B41))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A41,TIPOS_REQUIEREN_GRUPO,0)),OR($A41="CASO_CLINICO_TRONCO",$A41="CASO_CLINICO",$A41="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A41="PROBLEMA",$A41="SUBPROBLEMA",$A41="SUBITEM_CASO",$A41="SUBITEM_DE_CASO_O_PROBLEMA",$A41="EMPAREJAMIENTO_TRONCO",$A41="EMPAREJAMIENTO_AMPLIADO",$A41="EMPAREJAMIENTO_DE_CONCEPTOS",$A41="OPCION_EMPAREJAMIENTO",$A41="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B41))&gt;0,LEN(TRIM($B41))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B42">
-      <x:formula1>IF(ISNUMBER(MATCH($A42,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B42))&gt;0,LEN(TRIM($B42))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A42,TIPOS_REQUIEREN_GRUPO,0)),OR($A42="CASO_CLINICO_TRONCO",$A42="CASO_CLINICO",$A42="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A42="PROBLEMA",$A42="SUBPROBLEMA",$A42="SUBITEM_CASO",$A42="SUBITEM_DE_CASO_O_PROBLEMA",$A42="EMPAREJAMIENTO_TRONCO",$A42="EMPAREJAMIENTO_AMPLIADO",$A42="EMPAREJAMIENTO_DE_CONCEPTOS",$A42="OPCION_EMPAREJAMIENTO",$A42="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B42))&gt;0,LEN(TRIM($B42))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B43">
-      <x:formula1>IF(ISNUMBER(MATCH($A43,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B43))&gt;0,LEN(TRIM($B43))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A43,TIPOS_REQUIEREN_GRUPO,0)),OR($A43="CASO_CLINICO_TRONCO",$A43="CASO_CLINICO",$A43="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A43="PROBLEMA",$A43="SUBPROBLEMA",$A43="SUBITEM_CASO",$A43="SUBITEM_DE_CASO_O_PROBLEMA",$A43="EMPAREJAMIENTO_TRONCO",$A43="EMPAREJAMIENTO_AMPLIADO",$A43="EMPAREJAMIENTO_DE_CONCEPTOS",$A43="OPCION_EMPAREJAMIENTO",$A43="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B43))&gt;0,LEN(TRIM($B43))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B44">
-      <x:formula1>IF(ISNUMBER(MATCH($A44,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B44))&gt;0,LEN(TRIM($B44))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A44,TIPOS_REQUIEREN_GRUPO,0)),OR($A44="CASO_CLINICO_TRONCO",$A44="CASO_CLINICO",$A44="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A44="PROBLEMA",$A44="SUBPROBLEMA",$A44="SUBITEM_CASO",$A44="SUBITEM_DE_CASO_O_PROBLEMA",$A44="EMPAREJAMIENTO_TRONCO",$A44="EMPAREJAMIENTO_AMPLIADO",$A44="EMPAREJAMIENTO_DE_CONCEPTOS",$A44="OPCION_EMPAREJAMIENTO",$A44="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B44))&gt;0,LEN(TRIM($B44))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B45">
-      <x:formula1>IF(ISNUMBER(MATCH($A45,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B45))&gt;0,LEN(TRIM($B45))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A45,TIPOS_REQUIEREN_GRUPO,0)),OR($A45="CASO_CLINICO_TRONCO",$A45="CASO_CLINICO",$A45="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A45="PROBLEMA",$A45="SUBPROBLEMA",$A45="SUBITEM_CASO",$A45="SUBITEM_DE_CASO_O_PROBLEMA",$A45="EMPAREJAMIENTO_TRONCO",$A45="EMPAREJAMIENTO_AMPLIADO",$A45="EMPAREJAMIENTO_DE_CONCEPTOS",$A45="OPCION_EMPAREJAMIENTO",$A45="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B45))&gt;0,LEN(TRIM($B45))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B46">
-      <x:formula1>IF(ISNUMBER(MATCH($A46,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B46))&gt;0,LEN(TRIM($B46))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A46,TIPOS_REQUIEREN_GRUPO,0)),OR($A46="CASO_CLINICO_TRONCO",$A46="CASO_CLINICO",$A46="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A46="PROBLEMA",$A46="SUBPROBLEMA",$A46="SUBITEM_CASO",$A46="SUBITEM_DE_CASO_O_PROBLEMA",$A46="EMPAREJAMIENTO_TRONCO",$A46="EMPAREJAMIENTO_AMPLIADO",$A46="EMPAREJAMIENTO_DE_CONCEPTOS",$A46="OPCION_EMPAREJAMIENTO",$A46="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B46))&gt;0,LEN(TRIM($B46))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B47">
-      <x:formula1>IF(ISNUMBER(MATCH($A47,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B47))&gt;0,LEN(TRIM($B47))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A47,TIPOS_REQUIEREN_GRUPO,0)),OR($A47="CASO_CLINICO_TRONCO",$A47="CASO_CLINICO",$A47="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A47="PROBLEMA",$A47="SUBPROBLEMA",$A47="SUBITEM_CASO",$A47="SUBITEM_DE_CASO_O_PROBLEMA",$A47="EMPAREJAMIENTO_TRONCO",$A47="EMPAREJAMIENTO_AMPLIADO",$A47="EMPAREJAMIENTO_DE_CONCEPTOS",$A47="OPCION_EMPAREJAMIENTO",$A47="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B47))&gt;0,LEN(TRIM($B47))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B48">
-      <x:formula1>IF(ISNUMBER(MATCH($A48,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B48))&gt;0,LEN(TRIM($B48))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A48,TIPOS_REQUIEREN_GRUPO,0)),OR($A48="CASO_CLINICO_TRONCO",$A48="CASO_CLINICO",$A48="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A48="PROBLEMA",$A48="SUBPROBLEMA",$A48="SUBITEM_CASO",$A48="SUBITEM_DE_CASO_O_PROBLEMA",$A48="EMPAREJAMIENTO_TRONCO",$A48="EMPAREJAMIENTO_AMPLIADO",$A48="EMPAREJAMIENTO_DE_CONCEPTOS",$A48="OPCION_EMPAREJAMIENTO",$A48="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B48))&gt;0,LEN(TRIM($B48))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B49">
-      <x:formula1>IF(ISNUMBER(MATCH($A49,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B49))&gt;0,LEN(TRIM($B49))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A49,TIPOS_REQUIEREN_GRUPO,0)),OR($A49="CASO_CLINICO_TRONCO",$A49="CASO_CLINICO",$A49="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A49="PROBLEMA",$A49="SUBPROBLEMA",$A49="SUBITEM_CASO",$A49="SUBITEM_DE_CASO_O_PROBLEMA",$A49="EMPAREJAMIENTO_TRONCO",$A49="EMPAREJAMIENTO_AMPLIADO",$A49="EMPAREJAMIENTO_DE_CONCEPTOS",$A49="OPCION_EMPAREJAMIENTO",$A49="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B49))&gt;0,LEN(TRIM($B49))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B5">
-      <x:formula1>IF(ISNUMBER(MATCH($A5,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B5))&gt;0,LEN(TRIM($B5))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A5,TIPOS_REQUIEREN_GRUPO,0)),OR($A5="CASO_CLINICO_TRONCO",$A5="CASO_CLINICO",$A5="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A5="PROBLEMA",$A5="SUBPROBLEMA",$A5="SUBITEM_CASO",$A5="SUBITEM_DE_CASO_O_PROBLEMA",$A5="EMPAREJAMIENTO_TRONCO",$A5="EMPAREJAMIENTO_AMPLIADO",$A5="EMPAREJAMIENTO_DE_CONCEPTOS",$A5="OPCION_EMPAREJAMIENTO",$A5="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B5))&gt;0,LEN(TRIM($B5))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B50">
-      <x:formula1>IF(ISNUMBER(MATCH($A50,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B50))&gt;0,LEN(TRIM($B50))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A50,TIPOS_REQUIEREN_GRUPO,0)),OR($A50="CASO_CLINICO_TRONCO",$A50="CASO_CLINICO",$A50="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A50="PROBLEMA",$A50="SUBPROBLEMA",$A50="SUBITEM_CASO",$A50="SUBITEM_DE_CASO_O_PROBLEMA",$A50="EMPAREJAMIENTO_TRONCO",$A50="EMPAREJAMIENTO_AMPLIADO",$A50="EMPAREJAMIENTO_DE_CONCEPTOS",$A50="OPCION_EMPAREJAMIENTO",$A50="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B50))&gt;0,LEN(TRIM($B50))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B51">
-      <x:formula1>IF(ISNUMBER(MATCH($A51,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B51))&gt;0,LEN(TRIM($B51))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A51,TIPOS_REQUIEREN_GRUPO,0)),OR($A51="CASO_CLINICO_TRONCO",$A51="CASO_CLINICO",$A51="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A51="PROBLEMA",$A51="SUBPROBLEMA",$A51="SUBITEM_CASO",$A51="SUBITEM_DE_CASO_O_PROBLEMA",$A51="EMPAREJAMIENTO_TRONCO",$A51="EMPAREJAMIENTO_AMPLIADO",$A51="EMPAREJAMIENTO_DE_CONCEPTOS",$A51="OPCION_EMPAREJAMIENTO",$A51="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B51))&gt;0,LEN(TRIM($B51))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B52">
-      <x:formula1>IF(ISNUMBER(MATCH($A52,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B52))&gt;0,LEN(TRIM($B52))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A52,TIPOS_REQUIEREN_GRUPO,0)),OR($A52="CASO_CLINICO_TRONCO",$A52="CASO_CLINICO",$A52="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A52="PROBLEMA",$A52="SUBPROBLEMA",$A52="SUBITEM_CASO",$A52="SUBITEM_DE_CASO_O_PROBLEMA",$A52="EMPAREJAMIENTO_TRONCO",$A52="EMPAREJAMIENTO_AMPLIADO",$A52="EMPAREJAMIENTO_DE_CONCEPTOS",$A52="OPCION_EMPAREJAMIENTO",$A52="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B52))&gt;0,LEN(TRIM($B52))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B53">
-      <x:formula1>IF(ISNUMBER(MATCH($A53,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B53))&gt;0,LEN(TRIM($B53))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A53,TIPOS_REQUIEREN_GRUPO,0)),OR($A53="CASO_CLINICO_TRONCO",$A53="CASO_CLINICO",$A53="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A53="PROBLEMA",$A53="SUBPROBLEMA",$A53="SUBITEM_CASO",$A53="SUBITEM_DE_CASO_O_PROBLEMA",$A53="EMPAREJAMIENTO_TRONCO",$A53="EMPAREJAMIENTO_AMPLIADO",$A53="EMPAREJAMIENTO_DE_CONCEPTOS",$A53="OPCION_EMPAREJAMIENTO",$A53="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B53))&gt;0,LEN(TRIM($B53))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B54">
-      <x:formula1>IF(ISNUMBER(MATCH($A54,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B54))&gt;0,LEN(TRIM($B54))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A54,TIPOS_REQUIEREN_GRUPO,0)),OR($A54="CASO_CLINICO_TRONCO",$A54="CASO_CLINICO",$A54="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A54="PROBLEMA",$A54="SUBPROBLEMA",$A54="SUBITEM_CASO",$A54="SUBITEM_DE_CASO_O_PROBLEMA",$A54="EMPAREJAMIENTO_TRONCO",$A54="EMPAREJAMIENTO_AMPLIADO",$A54="EMPAREJAMIENTO_DE_CONCEPTOS",$A54="OPCION_EMPAREJAMIENTO",$A54="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B54))&gt;0,LEN(TRIM($B54))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B55">
-      <x:formula1>IF(ISNUMBER(MATCH($A55,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B55))&gt;0,LEN(TRIM($B55))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A55,TIPOS_REQUIEREN_GRUPO,0)),OR($A55="CASO_CLINICO_TRONCO",$A55="CASO_CLINICO",$A55="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A55="PROBLEMA",$A55="SUBPROBLEMA",$A55="SUBITEM_CASO",$A55="SUBITEM_DE_CASO_O_PROBLEMA",$A55="EMPAREJAMIENTO_TRONCO",$A55="EMPAREJAMIENTO_AMPLIADO",$A55="EMPAREJAMIENTO_DE_CONCEPTOS",$A55="OPCION_EMPAREJAMIENTO",$A55="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B55))&gt;0,LEN(TRIM($B55))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B56">
-      <x:formula1>IF(ISNUMBER(MATCH($A56,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B56))&gt;0,LEN(TRIM($B56))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A56,TIPOS_REQUIEREN_GRUPO,0)),OR($A56="CASO_CLINICO_TRONCO",$A56="CASO_CLINICO",$A56="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A56="PROBLEMA",$A56="SUBPROBLEMA",$A56="SUBITEM_CASO",$A56="SUBITEM_DE_CASO_O_PROBLEMA",$A56="EMPAREJAMIENTO_TRONCO",$A56="EMPAREJAMIENTO_AMPLIADO",$A56="EMPAREJAMIENTO_DE_CONCEPTOS",$A56="OPCION_EMPAREJAMIENTO",$A56="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B56))&gt;0,LEN(TRIM($B56))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B57">
-      <x:formula1>IF(ISNUMBER(MATCH($A57,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B57))&gt;0,LEN(TRIM($B57))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A57,TIPOS_REQUIEREN_GRUPO,0)),OR($A57="CASO_CLINICO_TRONCO",$A57="CASO_CLINICO",$A57="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A57="PROBLEMA",$A57="SUBPROBLEMA",$A57="SUBITEM_CASO",$A57="SUBITEM_DE_CASO_O_PROBLEMA",$A57="EMPAREJAMIENTO_TRONCO",$A57="EMPAREJAMIENTO_AMPLIADO",$A57="EMPAREJAMIENTO_DE_CONCEPTOS",$A57="OPCION_EMPAREJAMIENTO",$A57="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B57))&gt;0,LEN(TRIM($B57))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B58">
-      <x:formula1>IF(ISNUMBER(MATCH($A58,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B58))&gt;0,LEN(TRIM($B58))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A58,TIPOS_REQUIEREN_GRUPO,0)),OR($A58="CASO_CLINICO_TRONCO",$A58="CASO_CLINICO",$A58="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A58="PROBLEMA",$A58="SUBPROBLEMA",$A58="SUBITEM_CASO",$A58="SUBITEM_DE_CASO_O_PROBLEMA",$A58="EMPAREJAMIENTO_TRONCO",$A58="EMPAREJAMIENTO_AMPLIADO",$A58="EMPAREJAMIENTO_DE_CONCEPTOS",$A58="OPCION_EMPAREJAMIENTO",$A58="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B58))&gt;0,LEN(TRIM($B58))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B59">
-      <x:formula1>IF(ISNUMBER(MATCH($A59,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B59))&gt;0,LEN(TRIM($B59))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A59,TIPOS_REQUIEREN_GRUPO,0)),OR($A59="CASO_CLINICO_TRONCO",$A59="CASO_CLINICO",$A59="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A59="PROBLEMA",$A59="SUBPROBLEMA",$A59="SUBITEM_CASO",$A59="SUBITEM_DE_CASO_O_PROBLEMA",$A59="EMPAREJAMIENTO_TRONCO",$A59="EMPAREJAMIENTO_AMPLIADO",$A59="EMPAREJAMIENTO_DE_CONCEPTOS",$A59="OPCION_EMPAREJAMIENTO",$A59="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B59))&gt;0,LEN(TRIM($B59))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B6">
-      <x:formula1>IF(ISNUMBER(MATCH($A6,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B6))&gt;0,LEN(TRIM($B6))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A6,TIPOS_REQUIEREN_GRUPO,0)),OR($A6="CASO_CLINICO_TRONCO",$A6="CASO_CLINICO",$A6="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A6="PROBLEMA",$A6="SUBPROBLEMA",$A6="SUBITEM_CASO",$A6="SUBITEM_DE_CASO_O_PROBLEMA",$A6="EMPAREJAMIENTO_TRONCO",$A6="EMPAREJAMIENTO_AMPLIADO",$A6="EMPAREJAMIENTO_DE_CONCEPTOS",$A6="OPCION_EMPAREJAMIENTO",$A6="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B6))&gt;0,LEN(TRIM($B6))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B60">
-      <x:formula1>IF(ISNUMBER(MATCH($A60,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B60))&gt;0,LEN(TRIM($B60))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A60,TIPOS_REQUIEREN_GRUPO,0)),OR($A60="CASO_CLINICO_TRONCO",$A60="CASO_CLINICO",$A60="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A60="PROBLEMA",$A60="SUBPROBLEMA",$A60="SUBITEM_CASO",$A60="SUBITEM_DE_CASO_O_PROBLEMA",$A60="EMPAREJAMIENTO_TRONCO",$A60="EMPAREJAMIENTO_AMPLIADO",$A60="EMPAREJAMIENTO_DE_CONCEPTOS",$A60="OPCION_EMPAREJAMIENTO",$A60="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B60))&gt;0,LEN(TRIM($B60))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B61">
-      <x:formula1>IF(ISNUMBER(MATCH($A61,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B61))&gt;0,LEN(TRIM($B61))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A61,TIPOS_REQUIEREN_GRUPO,0)),OR($A61="CASO_CLINICO_TRONCO",$A61="CASO_CLINICO",$A61="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A61="PROBLEMA",$A61="SUBPROBLEMA",$A61="SUBITEM_CASO",$A61="SUBITEM_DE_CASO_O_PROBLEMA",$A61="EMPAREJAMIENTO_TRONCO",$A61="EMPAREJAMIENTO_AMPLIADO",$A61="EMPAREJAMIENTO_DE_CONCEPTOS",$A61="OPCION_EMPAREJAMIENTO",$A61="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B61))&gt;0,LEN(TRIM($B61))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B7">
-      <x:formula1>IF(ISNUMBER(MATCH($A7,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B7))&gt;0,LEN(TRIM($B7))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A7,TIPOS_REQUIEREN_GRUPO,0)),OR($A7="CASO_CLINICO_TRONCO",$A7="CASO_CLINICO",$A7="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A7="PROBLEMA",$A7="SUBPROBLEMA",$A7="SUBITEM_CASO",$A7="SUBITEM_DE_CASO_O_PROBLEMA",$A7="EMPAREJAMIENTO_TRONCO",$A7="EMPAREJAMIENTO_AMPLIADO",$A7="EMPAREJAMIENTO_DE_CONCEPTOS",$A7="OPCION_EMPAREJAMIENTO",$A7="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B7))&gt;0,LEN(TRIM($B7))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B8">
-      <x:formula1>IF(ISNUMBER(MATCH($A8,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B8))&gt;0,LEN(TRIM($B8))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A8,TIPOS_REQUIEREN_GRUPO,0)),OR($A8="CASO_CLINICO_TRONCO",$A8="CASO_CLINICO",$A8="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A8="PROBLEMA",$A8="SUBPROBLEMA",$A8="SUBITEM_CASO",$A8="SUBITEM_DE_CASO_O_PROBLEMA",$A8="EMPAREJAMIENTO_TRONCO",$A8="EMPAREJAMIENTO_AMPLIADO",$A8="EMPAREJAMIENTO_DE_CONCEPTOS",$A8="OPCION_EMPAREJAMIENTO",$A8="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B8))&gt;0,LEN(TRIM($B8))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Grupo invalido" error="El grupo solo se llena en casos/problemas, subitems, emparejamiento ampliado y opciones de emparejamiento." sqref="B9">
-      <x:formula1>IF(ISNUMBER(MATCH($A9,TIPOS_REQUIEREN_GRUPO,0)),LEN(TRIM($B9))&gt;0,LEN(TRIM($B9))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A9,TIPOS_REQUIEREN_GRUPO,0)),OR($A9="CASO_CLINICO_TRONCO",$A9="CASO_CLINICO",$A9="ITEMS_AGRUPADOS_POR_CASO_CLINICO_O_PROBLEMA",$A9="PROBLEMA",$A9="SUBPROBLEMA",$A9="SUBITEM_CASO",$A9="SUBITEM_DE_CASO_O_PROBLEMA",$A9="EMPAREJAMIENTO_TRONCO",$A9="EMPAREJAMIENTO_AMPLIADO",$A9="EMPAREJAMIENTO_DE_CONCEPTOS",$A9="OPCION_EMPAREJAMIENTO",$A9="OPCION_DE_EMPAREJAMIENTO_AMPLIADO")),LEN(TRIM($B9))&gt;0,LEN(TRIM($B9))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D10">
-      <x:formula1>IF(ISNUMBER(MATCH($A10,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D10))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A10,TIPOS_OPCION_D,0)),OR($A10="SELECCION_MEJOR_RESPUESTA",$A10="SELECCION_SIMPLE",$A10="SELECCION_UNICA",$A10="SELECCION_DE_LA_MEJOR_RESPUESTA",$A10="SUBITEM_CASO",$A10="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D10))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D11">
-      <x:formula1>IF(ISNUMBER(MATCH($A11,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D11))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A11,TIPOS_OPCION_D,0)),OR($A11="SELECCION_MEJOR_RESPUESTA",$A11="SELECCION_SIMPLE",$A11="SELECCION_UNICA",$A11="SELECCION_DE_LA_MEJOR_RESPUESTA",$A11="SUBITEM_CASO",$A11="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D11))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D12">
-      <x:formula1>IF(ISNUMBER(MATCH($A12,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D12))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A12,TIPOS_OPCION_D,0)),OR($A12="SELECCION_MEJOR_RESPUESTA",$A12="SELECCION_SIMPLE",$A12="SELECCION_UNICA",$A12="SELECCION_DE_LA_MEJOR_RESPUESTA",$A12="SUBITEM_CASO",$A12="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D12))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D13">
-      <x:formula1>IF(ISNUMBER(MATCH($A13,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D13))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A13,TIPOS_OPCION_D,0)),OR($A13="SELECCION_MEJOR_RESPUESTA",$A13="SELECCION_SIMPLE",$A13="SELECCION_UNICA",$A13="SELECCION_DE_LA_MEJOR_RESPUESTA",$A13="SUBITEM_CASO",$A13="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D13))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D14">
-      <x:formula1>IF(ISNUMBER(MATCH($A14,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D14))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A14,TIPOS_OPCION_D,0)),OR($A14="SELECCION_MEJOR_RESPUESTA",$A14="SELECCION_SIMPLE",$A14="SELECCION_UNICA",$A14="SELECCION_DE_LA_MEJOR_RESPUESTA",$A14="SUBITEM_CASO",$A14="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D14))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D15">
-      <x:formula1>IF(ISNUMBER(MATCH($A15,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D15))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A15,TIPOS_OPCION_D,0)),OR($A15="SELECCION_MEJOR_RESPUESTA",$A15="SELECCION_SIMPLE",$A15="SELECCION_UNICA",$A15="SELECCION_DE_LA_MEJOR_RESPUESTA",$A15="SUBITEM_CASO",$A15="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D15))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D16">
-      <x:formula1>IF(ISNUMBER(MATCH($A16,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D16))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A16,TIPOS_OPCION_D,0)),OR($A16="SELECCION_MEJOR_RESPUESTA",$A16="SELECCION_SIMPLE",$A16="SELECCION_UNICA",$A16="SELECCION_DE_LA_MEJOR_RESPUESTA",$A16="SUBITEM_CASO",$A16="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D16))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D17">
-      <x:formula1>IF(ISNUMBER(MATCH($A17,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D17))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A17,TIPOS_OPCION_D,0)),OR($A17="SELECCION_MEJOR_RESPUESTA",$A17="SELECCION_SIMPLE",$A17="SELECCION_UNICA",$A17="SELECCION_DE_LA_MEJOR_RESPUESTA",$A17="SUBITEM_CASO",$A17="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D17))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D18">
-      <x:formula1>IF(ISNUMBER(MATCH($A18,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D18))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A18,TIPOS_OPCION_D,0)),OR($A18="SELECCION_MEJOR_RESPUESTA",$A18="SELECCION_SIMPLE",$A18="SELECCION_UNICA",$A18="SELECCION_DE_LA_MEJOR_RESPUESTA",$A18="SUBITEM_CASO",$A18="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D18))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D19">
-      <x:formula1>IF(ISNUMBER(MATCH($A19,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D19))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A19,TIPOS_OPCION_D,0)),OR($A19="SELECCION_MEJOR_RESPUESTA",$A19="SELECCION_SIMPLE",$A19="SELECCION_UNICA",$A19="SELECCION_DE_LA_MEJOR_RESPUESTA",$A19="SUBITEM_CASO",$A19="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D19))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D2">
-      <x:formula1>IF(ISNUMBER(MATCH($A2,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D2))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A2,TIPOS_OPCION_D,0)),OR($A2="SELECCION_MEJOR_RESPUESTA",$A2="SELECCION_SIMPLE",$A2="SELECCION_UNICA",$A2="SELECCION_DE_LA_MEJOR_RESPUESTA",$A2="SUBITEM_CASO",$A2="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D2))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D20">
-      <x:formula1>IF(ISNUMBER(MATCH($A20,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D20))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A20,TIPOS_OPCION_D,0)),OR($A20="SELECCION_MEJOR_RESPUESTA",$A20="SELECCION_SIMPLE",$A20="SELECCION_UNICA",$A20="SELECCION_DE_LA_MEJOR_RESPUESTA",$A20="SUBITEM_CASO",$A20="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D20))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D21">
-      <x:formula1>IF(ISNUMBER(MATCH($A21,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D21))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A21,TIPOS_OPCION_D,0)),OR($A21="SELECCION_MEJOR_RESPUESTA",$A21="SELECCION_SIMPLE",$A21="SELECCION_UNICA",$A21="SELECCION_DE_LA_MEJOR_RESPUESTA",$A21="SUBITEM_CASO",$A21="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D21))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D22">
-      <x:formula1>IF(ISNUMBER(MATCH($A22,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D22))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A22,TIPOS_OPCION_D,0)),OR($A22="SELECCION_MEJOR_RESPUESTA",$A22="SELECCION_SIMPLE",$A22="SELECCION_UNICA",$A22="SELECCION_DE_LA_MEJOR_RESPUESTA",$A22="SUBITEM_CASO",$A22="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D22))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D23">
-      <x:formula1>IF(ISNUMBER(MATCH($A23,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D23))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A23,TIPOS_OPCION_D,0)),OR($A23="SELECCION_MEJOR_RESPUESTA",$A23="SELECCION_SIMPLE",$A23="SELECCION_UNICA",$A23="SELECCION_DE_LA_MEJOR_RESPUESTA",$A23="SUBITEM_CASO",$A23="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D23))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D24">
-      <x:formula1>IF(ISNUMBER(MATCH($A24,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D24))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A24,TIPOS_OPCION_D,0)),OR($A24="SELECCION_MEJOR_RESPUESTA",$A24="SELECCION_SIMPLE",$A24="SELECCION_UNICA",$A24="SELECCION_DE_LA_MEJOR_RESPUESTA",$A24="SUBITEM_CASO",$A24="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D24))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D25">
-      <x:formula1>IF(ISNUMBER(MATCH($A25,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D25))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A25,TIPOS_OPCION_D,0)),OR($A25="SELECCION_MEJOR_RESPUESTA",$A25="SELECCION_SIMPLE",$A25="SELECCION_UNICA",$A25="SELECCION_DE_LA_MEJOR_RESPUESTA",$A25="SUBITEM_CASO",$A25="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D25))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D26">
-      <x:formula1>IF(ISNUMBER(MATCH($A26,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D26))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A26,TIPOS_OPCION_D,0)),OR($A26="SELECCION_MEJOR_RESPUESTA",$A26="SELECCION_SIMPLE",$A26="SELECCION_UNICA",$A26="SELECCION_DE_LA_MEJOR_RESPUESTA",$A26="SUBITEM_CASO",$A26="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D26))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D27">
-      <x:formula1>IF(ISNUMBER(MATCH($A27,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D27))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A27,TIPOS_OPCION_D,0)),OR($A27="SELECCION_MEJOR_RESPUESTA",$A27="SELECCION_SIMPLE",$A27="SELECCION_UNICA",$A27="SELECCION_DE_LA_MEJOR_RESPUESTA",$A27="SUBITEM_CASO",$A27="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D27))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D28">
-      <x:formula1>IF(ISNUMBER(MATCH($A28,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D28))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A28,TIPOS_OPCION_D,0)),OR($A28="SELECCION_MEJOR_RESPUESTA",$A28="SELECCION_SIMPLE",$A28="SELECCION_UNICA",$A28="SELECCION_DE_LA_MEJOR_RESPUESTA",$A28="SUBITEM_CASO",$A28="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D28))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D29">
-      <x:formula1>IF(ISNUMBER(MATCH($A29,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D29))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A29,TIPOS_OPCION_D,0)),OR($A29="SELECCION_MEJOR_RESPUESTA",$A29="SELECCION_SIMPLE",$A29="SELECCION_UNICA",$A29="SELECCION_DE_LA_MEJOR_RESPUESTA",$A29="SUBITEM_CASO",$A29="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D29))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D3">
-      <x:formula1>IF(ISNUMBER(MATCH($A3,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D3))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A3,TIPOS_OPCION_D,0)),OR($A3="SELECCION_MEJOR_RESPUESTA",$A3="SELECCION_SIMPLE",$A3="SELECCION_UNICA",$A3="SELECCION_DE_LA_MEJOR_RESPUESTA",$A3="SUBITEM_CASO",$A3="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D3))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D30">
-      <x:formula1>IF(ISNUMBER(MATCH($A30,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D30))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A30,TIPOS_OPCION_D,0)),OR($A30="SELECCION_MEJOR_RESPUESTA",$A30="SELECCION_SIMPLE",$A30="SELECCION_UNICA",$A30="SELECCION_DE_LA_MEJOR_RESPUESTA",$A30="SUBITEM_CASO",$A30="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D30))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D31">
-      <x:formula1>IF(ISNUMBER(MATCH($A31,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D31))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A31,TIPOS_OPCION_D,0)),OR($A31="SELECCION_MEJOR_RESPUESTA",$A31="SELECCION_SIMPLE",$A31="SELECCION_UNICA",$A31="SELECCION_DE_LA_MEJOR_RESPUESTA",$A31="SUBITEM_CASO",$A31="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D31))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D32">
-      <x:formula1>IF(ISNUMBER(MATCH($A32,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D32))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A32,TIPOS_OPCION_D,0)),OR($A32="SELECCION_MEJOR_RESPUESTA",$A32="SELECCION_SIMPLE",$A32="SELECCION_UNICA",$A32="SELECCION_DE_LA_MEJOR_RESPUESTA",$A32="SUBITEM_CASO",$A32="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D32))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D33">
-      <x:formula1>IF(ISNUMBER(MATCH($A33,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D33))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A33,TIPOS_OPCION_D,0)),OR($A33="SELECCION_MEJOR_RESPUESTA",$A33="SELECCION_SIMPLE",$A33="SELECCION_UNICA",$A33="SELECCION_DE_LA_MEJOR_RESPUESTA",$A33="SUBITEM_CASO",$A33="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D33))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D34">
-      <x:formula1>IF(ISNUMBER(MATCH($A34,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D34))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A34,TIPOS_OPCION_D,0)),OR($A34="SELECCION_MEJOR_RESPUESTA",$A34="SELECCION_SIMPLE",$A34="SELECCION_UNICA",$A34="SELECCION_DE_LA_MEJOR_RESPUESTA",$A34="SUBITEM_CASO",$A34="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D34))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D35">
-      <x:formula1>IF(ISNUMBER(MATCH($A35,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D35))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A35,TIPOS_OPCION_D,0)),OR($A35="SELECCION_MEJOR_RESPUESTA",$A35="SELECCION_SIMPLE",$A35="SELECCION_UNICA",$A35="SELECCION_DE_LA_MEJOR_RESPUESTA",$A35="SUBITEM_CASO",$A35="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D35))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D36">
-      <x:formula1>IF(ISNUMBER(MATCH($A36,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D36))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A36,TIPOS_OPCION_D,0)),OR($A36="SELECCION_MEJOR_RESPUESTA",$A36="SELECCION_SIMPLE",$A36="SELECCION_UNICA",$A36="SELECCION_DE_LA_MEJOR_RESPUESTA",$A36="SUBITEM_CASO",$A36="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D36))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D37">
-      <x:formula1>IF(ISNUMBER(MATCH($A37,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D37))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A37,TIPOS_OPCION_D,0)),OR($A37="SELECCION_MEJOR_RESPUESTA",$A37="SELECCION_SIMPLE",$A37="SELECCION_UNICA",$A37="SELECCION_DE_LA_MEJOR_RESPUESTA",$A37="SUBITEM_CASO",$A37="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D37))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D38">
-      <x:formula1>IF(ISNUMBER(MATCH($A38,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D38))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A38,TIPOS_OPCION_D,0)),OR($A38="SELECCION_MEJOR_RESPUESTA",$A38="SELECCION_SIMPLE",$A38="SELECCION_UNICA",$A38="SELECCION_DE_LA_MEJOR_RESPUESTA",$A38="SUBITEM_CASO",$A38="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D38))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D39">
-      <x:formula1>IF(ISNUMBER(MATCH($A39,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D39))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A39,TIPOS_OPCION_D,0)),OR($A39="SELECCION_MEJOR_RESPUESTA",$A39="SELECCION_SIMPLE",$A39="SELECCION_UNICA",$A39="SELECCION_DE_LA_MEJOR_RESPUESTA",$A39="SUBITEM_CASO",$A39="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D39))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D4">
-      <x:formula1>IF(ISNUMBER(MATCH($A4,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D4))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A4,TIPOS_OPCION_D,0)),OR($A4="SELECCION_MEJOR_RESPUESTA",$A4="SELECCION_SIMPLE",$A4="SELECCION_UNICA",$A4="SELECCION_DE_LA_MEJOR_RESPUESTA",$A4="SUBITEM_CASO",$A4="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D4))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D40">
-      <x:formula1>IF(ISNUMBER(MATCH($A40,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D40))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A40,TIPOS_OPCION_D,0)),OR($A40="SELECCION_MEJOR_RESPUESTA",$A40="SELECCION_SIMPLE",$A40="SELECCION_UNICA",$A40="SELECCION_DE_LA_MEJOR_RESPUESTA",$A40="SUBITEM_CASO",$A40="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D40))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D41">
-      <x:formula1>IF(ISNUMBER(MATCH($A41,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D41))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A41,TIPOS_OPCION_D,0)),OR($A41="SELECCION_MEJOR_RESPUESTA",$A41="SELECCION_SIMPLE",$A41="SELECCION_UNICA",$A41="SELECCION_DE_LA_MEJOR_RESPUESTA",$A41="SUBITEM_CASO",$A41="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D41))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D42">
-      <x:formula1>IF(ISNUMBER(MATCH($A42,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D42))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A42,TIPOS_OPCION_D,0)),OR($A42="SELECCION_MEJOR_RESPUESTA",$A42="SELECCION_SIMPLE",$A42="SELECCION_UNICA",$A42="SELECCION_DE_LA_MEJOR_RESPUESTA",$A42="SUBITEM_CASO",$A42="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D42))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D43">
-      <x:formula1>IF(ISNUMBER(MATCH($A43,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D43))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A43,TIPOS_OPCION_D,0)),OR($A43="SELECCION_MEJOR_RESPUESTA",$A43="SELECCION_SIMPLE",$A43="SELECCION_UNICA",$A43="SELECCION_DE_LA_MEJOR_RESPUESTA",$A43="SUBITEM_CASO",$A43="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D43))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D44">
-      <x:formula1>IF(ISNUMBER(MATCH($A44,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D44))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A44,TIPOS_OPCION_D,0)),OR($A44="SELECCION_MEJOR_RESPUESTA",$A44="SELECCION_SIMPLE",$A44="SELECCION_UNICA",$A44="SELECCION_DE_LA_MEJOR_RESPUESTA",$A44="SUBITEM_CASO",$A44="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D44))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D45">
-      <x:formula1>IF(ISNUMBER(MATCH($A45,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D45))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A45,TIPOS_OPCION_D,0)),OR($A45="SELECCION_MEJOR_RESPUESTA",$A45="SELECCION_SIMPLE",$A45="SELECCION_UNICA",$A45="SELECCION_DE_LA_MEJOR_RESPUESTA",$A45="SUBITEM_CASO",$A45="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D45))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D46">
-      <x:formula1>IF(ISNUMBER(MATCH($A46,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D46))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A46,TIPOS_OPCION_D,0)),OR($A46="SELECCION_MEJOR_RESPUESTA",$A46="SELECCION_SIMPLE",$A46="SELECCION_UNICA",$A46="SELECCION_DE_LA_MEJOR_RESPUESTA",$A46="SUBITEM_CASO",$A46="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D46))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D47">
-      <x:formula1>IF(ISNUMBER(MATCH($A47,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D47))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A47,TIPOS_OPCION_D,0)),OR($A47="SELECCION_MEJOR_RESPUESTA",$A47="SELECCION_SIMPLE",$A47="SELECCION_UNICA",$A47="SELECCION_DE_LA_MEJOR_RESPUESTA",$A47="SUBITEM_CASO",$A47="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D47))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D48">
-      <x:formula1>IF(ISNUMBER(MATCH($A48,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D48))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A48,TIPOS_OPCION_D,0)),OR($A48="SELECCION_MEJOR_RESPUESTA",$A48="SELECCION_SIMPLE",$A48="SELECCION_UNICA",$A48="SELECCION_DE_LA_MEJOR_RESPUESTA",$A48="SUBITEM_CASO",$A48="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D48))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D49">
-      <x:formula1>IF(ISNUMBER(MATCH($A49,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D49))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A49,TIPOS_OPCION_D,0)),OR($A49="SELECCION_MEJOR_RESPUESTA",$A49="SELECCION_SIMPLE",$A49="SELECCION_UNICA",$A49="SELECCION_DE_LA_MEJOR_RESPUESTA",$A49="SUBITEM_CASO",$A49="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D49))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D5">
-      <x:formula1>IF(ISNUMBER(MATCH($A5,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D5))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A5,TIPOS_OPCION_D,0)),OR($A5="SELECCION_MEJOR_RESPUESTA",$A5="SELECCION_SIMPLE",$A5="SELECCION_UNICA",$A5="SELECCION_DE_LA_MEJOR_RESPUESTA",$A5="SUBITEM_CASO",$A5="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D5))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D50">
-      <x:formula1>IF(ISNUMBER(MATCH($A50,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D50))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A50,TIPOS_OPCION_D,0)),OR($A50="SELECCION_MEJOR_RESPUESTA",$A50="SELECCION_SIMPLE",$A50="SELECCION_UNICA",$A50="SELECCION_DE_LA_MEJOR_RESPUESTA",$A50="SUBITEM_CASO",$A50="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D50))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D51">
-      <x:formula1>IF(ISNUMBER(MATCH($A51,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D51))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A51,TIPOS_OPCION_D,0)),OR($A51="SELECCION_MEJOR_RESPUESTA",$A51="SELECCION_SIMPLE",$A51="SELECCION_UNICA",$A51="SELECCION_DE_LA_MEJOR_RESPUESTA",$A51="SUBITEM_CASO",$A51="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D51))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D52">
-      <x:formula1>IF(ISNUMBER(MATCH($A52,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D52))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A52,TIPOS_OPCION_D,0)),OR($A52="SELECCION_MEJOR_RESPUESTA",$A52="SELECCION_SIMPLE",$A52="SELECCION_UNICA",$A52="SELECCION_DE_LA_MEJOR_RESPUESTA",$A52="SUBITEM_CASO",$A52="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D52))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D53">
-      <x:formula1>IF(ISNUMBER(MATCH($A53,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D53))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A53,TIPOS_OPCION_D,0)),OR($A53="SELECCION_MEJOR_RESPUESTA",$A53="SELECCION_SIMPLE",$A53="SELECCION_UNICA",$A53="SELECCION_DE_LA_MEJOR_RESPUESTA",$A53="SUBITEM_CASO",$A53="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D53))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D54">
-      <x:formula1>IF(ISNUMBER(MATCH($A54,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D54))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A54,TIPOS_OPCION_D,0)),OR($A54="SELECCION_MEJOR_RESPUESTA",$A54="SELECCION_SIMPLE",$A54="SELECCION_UNICA",$A54="SELECCION_DE_LA_MEJOR_RESPUESTA",$A54="SUBITEM_CASO",$A54="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D54))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D55">
-      <x:formula1>IF(ISNUMBER(MATCH($A55,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D55))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A55,TIPOS_OPCION_D,0)),OR($A55="SELECCION_MEJOR_RESPUESTA",$A55="SELECCION_SIMPLE",$A55="SELECCION_UNICA",$A55="SELECCION_DE_LA_MEJOR_RESPUESTA",$A55="SUBITEM_CASO",$A55="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D55))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D56">
-      <x:formula1>IF(ISNUMBER(MATCH($A56,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D56))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A56,TIPOS_OPCION_D,0)),OR($A56="SELECCION_MEJOR_RESPUESTA",$A56="SELECCION_SIMPLE",$A56="SELECCION_UNICA",$A56="SELECCION_DE_LA_MEJOR_RESPUESTA",$A56="SUBITEM_CASO",$A56="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D56))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D57">
-      <x:formula1>IF(ISNUMBER(MATCH($A57,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D57))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A57,TIPOS_OPCION_D,0)),OR($A57="SELECCION_MEJOR_RESPUESTA",$A57="SELECCION_SIMPLE",$A57="SELECCION_UNICA",$A57="SELECCION_DE_LA_MEJOR_RESPUESTA",$A57="SUBITEM_CASO",$A57="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D57))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D58">
-      <x:formula1>IF(ISNUMBER(MATCH($A58,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D58))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A58,TIPOS_OPCION_D,0)),OR($A58="SELECCION_MEJOR_RESPUESTA",$A58="SELECCION_SIMPLE",$A58="SELECCION_UNICA",$A58="SELECCION_DE_LA_MEJOR_RESPUESTA",$A58="SUBITEM_CASO",$A58="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D58))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D59">
-      <x:formula1>IF(ISNUMBER(MATCH($A59,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D59))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A59,TIPOS_OPCION_D,0)),OR($A59="SELECCION_MEJOR_RESPUESTA",$A59="SELECCION_SIMPLE",$A59="SELECCION_UNICA",$A59="SELECCION_DE_LA_MEJOR_RESPUESTA",$A59="SUBITEM_CASO",$A59="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D59))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D6">
-      <x:formula1>IF(ISNUMBER(MATCH($A6,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D6))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A6,TIPOS_OPCION_D,0)),OR($A6="SELECCION_MEJOR_RESPUESTA",$A6="SELECCION_SIMPLE",$A6="SELECCION_UNICA",$A6="SELECCION_DE_LA_MEJOR_RESPUESTA",$A6="SUBITEM_CASO",$A6="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D6))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D60">
-      <x:formula1>IF(ISNUMBER(MATCH($A60,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D60))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A60,TIPOS_OPCION_D,0)),OR($A60="SELECCION_MEJOR_RESPUESTA",$A60="SELECCION_SIMPLE",$A60="SELECCION_UNICA",$A60="SELECCION_DE_LA_MEJOR_RESPUESTA",$A60="SUBITEM_CASO",$A60="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D60))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D61">
-      <x:formula1>IF(ISNUMBER(MATCH($A61,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D61))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A61,TIPOS_OPCION_D,0)),OR($A61="SELECCION_MEJOR_RESPUESTA",$A61="SELECCION_SIMPLE",$A61="SELECCION_UNICA",$A61="SELECCION_DE_LA_MEJOR_RESPUESTA",$A61="SUBITEM_CASO",$A61="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D61))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D7">
-      <x:formula1>IF(ISNUMBER(MATCH($A7,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D7))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A7,TIPOS_OPCION_D,0)),OR($A7="SELECCION_MEJOR_RESPUESTA",$A7="SELECCION_SIMPLE",$A7="SELECCION_UNICA",$A7="SELECCION_DE_LA_MEJOR_RESPUESTA",$A7="SUBITEM_CASO",$A7="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D7))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D8">
-      <x:formula1>IF(ISNUMBER(MATCH($A8,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D8))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A8,TIPOS_OPCION_D,0)),OR($A8="SELECCION_MEJOR_RESPUESTA",$A8="SELECCION_SIMPLE",$A8="SELECCION_UNICA",$A8="SELECCION_DE_LA_MEJOR_RESPUESTA",$A8="SUBITEM_CASO",$A8="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D8))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="D9">
-      <x:formula1>IF(ISNUMBER(MATCH($A9,TIPOS_OPCION_D,0)),TRUE,LEN(TRIM($D9))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A9,TIPOS_OPCION_D,0)),OR($A9="SELECCION_MEJOR_RESPUESTA",$A9="SELECCION_SIMPLE",$A9="SELECCION_UNICA",$A9="SELECCION_DE_LA_MEJOR_RESPUESTA",$A9="SUBITEM_CASO",$A9="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($D9))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E10">
-      <x:formula1>IF(ISNUMBER(MATCH($A10,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E10))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A10,TIPOS_OPCION_E,0)),OR($A10="SELECCION_MEJOR_RESPUESTA",$A10="SELECCION_SIMPLE",$A10="SELECCION_UNICA",$A10="SELECCION_DE_LA_MEJOR_RESPUESTA",$A10="SUBITEM_CASO",$A10="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E10))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E11">
-      <x:formula1>IF(ISNUMBER(MATCH($A11,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E11))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A11,TIPOS_OPCION_E,0)),OR($A11="SELECCION_MEJOR_RESPUESTA",$A11="SELECCION_SIMPLE",$A11="SELECCION_UNICA",$A11="SELECCION_DE_LA_MEJOR_RESPUESTA",$A11="SUBITEM_CASO",$A11="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E11))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E12">
-      <x:formula1>IF(ISNUMBER(MATCH($A12,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E12))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A12,TIPOS_OPCION_E,0)),OR($A12="SELECCION_MEJOR_RESPUESTA",$A12="SELECCION_SIMPLE",$A12="SELECCION_UNICA",$A12="SELECCION_DE_LA_MEJOR_RESPUESTA",$A12="SUBITEM_CASO",$A12="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E12))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E13">
-      <x:formula1>IF(ISNUMBER(MATCH($A13,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E13))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A13,TIPOS_OPCION_E,0)),OR($A13="SELECCION_MEJOR_RESPUESTA",$A13="SELECCION_SIMPLE",$A13="SELECCION_UNICA",$A13="SELECCION_DE_LA_MEJOR_RESPUESTA",$A13="SUBITEM_CASO",$A13="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E13))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E14">
-      <x:formula1>IF(ISNUMBER(MATCH($A14,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E14))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A14,TIPOS_OPCION_E,0)),OR($A14="SELECCION_MEJOR_RESPUESTA",$A14="SELECCION_SIMPLE",$A14="SELECCION_UNICA",$A14="SELECCION_DE_LA_MEJOR_RESPUESTA",$A14="SUBITEM_CASO",$A14="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E14))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E15">
-      <x:formula1>IF(ISNUMBER(MATCH($A15,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E15))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A15,TIPOS_OPCION_E,0)),OR($A15="SELECCION_MEJOR_RESPUESTA",$A15="SELECCION_SIMPLE",$A15="SELECCION_UNICA",$A15="SELECCION_DE_LA_MEJOR_RESPUESTA",$A15="SUBITEM_CASO",$A15="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E15))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E16">
-      <x:formula1>IF(ISNUMBER(MATCH($A16,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E16))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A16,TIPOS_OPCION_E,0)),OR($A16="SELECCION_MEJOR_RESPUESTA",$A16="SELECCION_SIMPLE",$A16="SELECCION_UNICA",$A16="SELECCION_DE_LA_MEJOR_RESPUESTA",$A16="SUBITEM_CASO",$A16="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E16))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E17">
-      <x:formula1>IF(ISNUMBER(MATCH($A17,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E17))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A17,TIPOS_OPCION_E,0)),OR($A17="SELECCION_MEJOR_RESPUESTA",$A17="SELECCION_SIMPLE",$A17="SELECCION_UNICA",$A17="SELECCION_DE_LA_MEJOR_RESPUESTA",$A17="SUBITEM_CASO",$A17="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E17))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E18">
-      <x:formula1>IF(ISNUMBER(MATCH($A18,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E18))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A18,TIPOS_OPCION_E,0)),OR($A18="SELECCION_MEJOR_RESPUESTA",$A18="SELECCION_SIMPLE",$A18="SELECCION_UNICA",$A18="SELECCION_DE_LA_MEJOR_RESPUESTA",$A18="SUBITEM_CASO",$A18="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E18))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E19">
-      <x:formula1>IF(ISNUMBER(MATCH($A19,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E19))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A19,TIPOS_OPCION_E,0)),OR($A19="SELECCION_MEJOR_RESPUESTA",$A19="SELECCION_SIMPLE",$A19="SELECCION_UNICA",$A19="SELECCION_DE_LA_MEJOR_RESPUESTA",$A19="SUBITEM_CASO",$A19="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E19))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E2">
-      <x:formula1>IF(ISNUMBER(MATCH($A2,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E2))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A2,TIPOS_OPCION_E,0)),OR($A2="SELECCION_MEJOR_RESPUESTA",$A2="SELECCION_SIMPLE",$A2="SELECCION_UNICA",$A2="SELECCION_DE_LA_MEJOR_RESPUESTA",$A2="SUBITEM_CASO",$A2="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E2))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E20">
-      <x:formula1>IF(ISNUMBER(MATCH($A20,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E20))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A20,TIPOS_OPCION_E,0)),OR($A20="SELECCION_MEJOR_RESPUESTA",$A20="SELECCION_SIMPLE",$A20="SELECCION_UNICA",$A20="SELECCION_DE_LA_MEJOR_RESPUESTA",$A20="SUBITEM_CASO",$A20="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E20))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E21">
-      <x:formula1>IF(ISNUMBER(MATCH($A21,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E21))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A21,TIPOS_OPCION_E,0)),OR($A21="SELECCION_MEJOR_RESPUESTA",$A21="SELECCION_SIMPLE",$A21="SELECCION_UNICA",$A21="SELECCION_DE_LA_MEJOR_RESPUESTA",$A21="SUBITEM_CASO",$A21="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E21))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E22">
-      <x:formula1>IF(ISNUMBER(MATCH($A22,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E22))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A22,TIPOS_OPCION_E,0)),OR($A22="SELECCION_MEJOR_RESPUESTA",$A22="SELECCION_SIMPLE",$A22="SELECCION_UNICA",$A22="SELECCION_DE_LA_MEJOR_RESPUESTA",$A22="SUBITEM_CASO",$A22="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E22))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E23">
-      <x:formula1>IF(ISNUMBER(MATCH($A23,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E23))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A23,TIPOS_OPCION_E,0)),OR($A23="SELECCION_MEJOR_RESPUESTA",$A23="SELECCION_SIMPLE",$A23="SELECCION_UNICA",$A23="SELECCION_DE_LA_MEJOR_RESPUESTA",$A23="SUBITEM_CASO",$A23="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E23))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E24">
-      <x:formula1>IF(ISNUMBER(MATCH($A24,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E24))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A24,TIPOS_OPCION_E,0)),OR($A24="SELECCION_MEJOR_RESPUESTA",$A24="SELECCION_SIMPLE",$A24="SELECCION_UNICA",$A24="SELECCION_DE_LA_MEJOR_RESPUESTA",$A24="SUBITEM_CASO",$A24="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E24))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E25">
-      <x:formula1>IF(ISNUMBER(MATCH($A25,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E25))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A25,TIPOS_OPCION_E,0)),OR($A25="SELECCION_MEJOR_RESPUESTA",$A25="SELECCION_SIMPLE",$A25="SELECCION_UNICA",$A25="SELECCION_DE_LA_MEJOR_RESPUESTA",$A25="SUBITEM_CASO",$A25="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E25))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E26">
-      <x:formula1>IF(ISNUMBER(MATCH($A26,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E26))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A26,TIPOS_OPCION_E,0)),OR($A26="SELECCION_MEJOR_RESPUESTA",$A26="SELECCION_SIMPLE",$A26="SELECCION_UNICA",$A26="SELECCION_DE_LA_MEJOR_RESPUESTA",$A26="SUBITEM_CASO",$A26="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E26))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E27">
-      <x:formula1>IF(ISNUMBER(MATCH($A27,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E27))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A27,TIPOS_OPCION_E,0)),OR($A27="SELECCION_MEJOR_RESPUESTA",$A27="SELECCION_SIMPLE",$A27="SELECCION_UNICA",$A27="SELECCION_DE_LA_MEJOR_RESPUESTA",$A27="SUBITEM_CASO",$A27="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E27))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E28">
-      <x:formula1>IF(ISNUMBER(MATCH($A28,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E28))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A28,TIPOS_OPCION_E,0)),OR($A28="SELECCION_MEJOR_RESPUESTA",$A28="SELECCION_SIMPLE",$A28="SELECCION_UNICA",$A28="SELECCION_DE_LA_MEJOR_RESPUESTA",$A28="SUBITEM_CASO",$A28="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E28))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E29">
-      <x:formula1>IF(ISNUMBER(MATCH($A29,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E29))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A29,TIPOS_OPCION_E,0)),OR($A29="SELECCION_MEJOR_RESPUESTA",$A29="SELECCION_SIMPLE",$A29="SELECCION_UNICA",$A29="SELECCION_DE_LA_MEJOR_RESPUESTA",$A29="SUBITEM_CASO",$A29="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E29))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E3">
-      <x:formula1>IF(ISNUMBER(MATCH($A3,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E3))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A3,TIPOS_OPCION_E,0)),OR($A3="SELECCION_MEJOR_RESPUESTA",$A3="SELECCION_SIMPLE",$A3="SELECCION_UNICA",$A3="SELECCION_DE_LA_MEJOR_RESPUESTA",$A3="SUBITEM_CASO",$A3="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E3))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E30">
-      <x:formula1>IF(ISNUMBER(MATCH($A30,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E30))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A30,TIPOS_OPCION_E,0)),OR($A30="SELECCION_MEJOR_RESPUESTA",$A30="SELECCION_SIMPLE",$A30="SELECCION_UNICA",$A30="SELECCION_DE_LA_MEJOR_RESPUESTA",$A30="SUBITEM_CASO",$A30="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E30))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E31">
-      <x:formula1>IF(ISNUMBER(MATCH($A31,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E31))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A31,TIPOS_OPCION_E,0)),OR($A31="SELECCION_MEJOR_RESPUESTA",$A31="SELECCION_SIMPLE",$A31="SELECCION_UNICA",$A31="SELECCION_DE_LA_MEJOR_RESPUESTA",$A31="SUBITEM_CASO",$A31="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E31))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E32">
-      <x:formula1>IF(ISNUMBER(MATCH($A32,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E32))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A32,TIPOS_OPCION_E,0)),OR($A32="SELECCION_MEJOR_RESPUESTA",$A32="SELECCION_SIMPLE",$A32="SELECCION_UNICA",$A32="SELECCION_DE_LA_MEJOR_RESPUESTA",$A32="SUBITEM_CASO",$A32="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E32))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E33">
-      <x:formula1>IF(ISNUMBER(MATCH($A33,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E33))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A33,TIPOS_OPCION_E,0)),OR($A33="SELECCION_MEJOR_RESPUESTA",$A33="SELECCION_SIMPLE",$A33="SELECCION_UNICA",$A33="SELECCION_DE_LA_MEJOR_RESPUESTA",$A33="SUBITEM_CASO",$A33="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E33))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E34">
-      <x:formula1>IF(ISNUMBER(MATCH($A34,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E34))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A34,TIPOS_OPCION_E,0)),OR($A34="SELECCION_MEJOR_RESPUESTA",$A34="SELECCION_SIMPLE",$A34="SELECCION_UNICA",$A34="SELECCION_DE_LA_MEJOR_RESPUESTA",$A34="SUBITEM_CASO",$A34="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E34))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E35">
-      <x:formula1>IF(ISNUMBER(MATCH($A35,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E35))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A35,TIPOS_OPCION_E,0)),OR($A35="SELECCION_MEJOR_RESPUESTA",$A35="SELECCION_SIMPLE",$A35="SELECCION_UNICA",$A35="SELECCION_DE_LA_MEJOR_RESPUESTA",$A35="SUBITEM_CASO",$A35="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E35))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E36">
-      <x:formula1>IF(ISNUMBER(MATCH($A36,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E36))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A36,TIPOS_OPCION_E,0)),OR($A36="SELECCION_MEJOR_RESPUESTA",$A36="SELECCION_SIMPLE",$A36="SELECCION_UNICA",$A36="SELECCION_DE_LA_MEJOR_RESPUESTA",$A36="SUBITEM_CASO",$A36="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E36))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E37">
-      <x:formula1>IF(ISNUMBER(MATCH($A37,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E37))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A37,TIPOS_OPCION_E,0)),OR($A37="SELECCION_MEJOR_RESPUESTA",$A37="SELECCION_SIMPLE",$A37="SELECCION_UNICA",$A37="SELECCION_DE_LA_MEJOR_RESPUESTA",$A37="SUBITEM_CASO",$A37="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E37))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E38">
-      <x:formula1>IF(ISNUMBER(MATCH($A38,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E38))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A38,TIPOS_OPCION_E,0)),OR($A38="SELECCION_MEJOR_RESPUESTA",$A38="SELECCION_SIMPLE",$A38="SELECCION_UNICA",$A38="SELECCION_DE_LA_MEJOR_RESPUESTA",$A38="SUBITEM_CASO",$A38="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E38))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E39">
-      <x:formula1>IF(ISNUMBER(MATCH($A39,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E39))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A39,TIPOS_OPCION_E,0)),OR($A39="SELECCION_MEJOR_RESPUESTA",$A39="SELECCION_SIMPLE",$A39="SELECCION_UNICA",$A39="SELECCION_DE_LA_MEJOR_RESPUESTA",$A39="SUBITEM_CASO",$A39="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E39))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E4">
-      <x:formula1>IF(ISNUMBER(MATCH($A4,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E4))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A4,TIPOS_OPCION_E,0)),OR($A4="SELECCION_MEJOR_RESPUESTA",$A4="SELECCION_SIMPLE",$A4="SELECCION_UNICA",$A4="SELECCION_DE_LA_MEJOR_RESPUESTA",$A4="SUBITEM_CASO",$A4="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E4))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E40">
-      <x:formula1>IF(ISNUMBER(MATCH($A40,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E40))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A40,TIPOS_OPCION_E,0)),OR($A40="SELECCION_MEJOR_RESPUESTA",$A40="SELECCION_SIMPLE",$A40="SELECCION_UNICA",$A40="SELECCION_DE_LA_MEJOR_RESPUESTA",$A40="SUBITEM_CASO",$A40="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E40))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E41">
-      <x:formula1>IF(ISNUMBER(MATCH($A41,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E41))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A41,TIPOS_OPCION_E,0)),OR($A41="SELECCION_MEJOR_RESPUESTA",$A41="SELECCION_SIMPLE",$A41="SELECCION_UNICA",$A41="SELECCION_DE_LA_MEJOR_RESPUESTA",$A41="SUBITEM_CASO",$A41="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E41))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E42">
-      <x:formula1>IF(ISNUMBER(MATCH($A42,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E42))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A42,TIPOS_OPCION_E,0)),OR($A42="SELECCION_MEJOR_RESPUESTA",$A42="SELECCION_SIMPLE",$A42="SELECCION_UNICA",$A42="SELECCION_DE_LA_MEJOR_RESPUESTA",$A42="SUBITEM_CASO",$A42="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E42))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E43">
-      <x:formula1>IF(ISNUMBER(MATCH($A43,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E43))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A43,TIPOS_OPCION_E,0)),OR($A43="SELECCION_MEJOR_RESPUESTA",$A43="SELECCION_SIMPLE",$A43="SELECCION_UNICA",$A43="SELECCION_DE_LA_MEJOR_RESPUESTA",$A43="SUBITEM_CASO",$A43="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E43))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E44">
-      <x:formula1>IF(ISNUMBER(MATCH($A44,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E44))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A44,TIPOS_OPCION_E,0)),OR($A44="SELECCION_MEJOR_RESPUESTA",$A44="SELECCION_SIMPLE",$A44="SELECCION_UNICA",$A44="SELECCION_DE_LA_MEJOR_RESPUESTA",$A44="SUBITEM_CASO",$A44="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E44))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E45">
-      <x:formula1>IF(ISNUMBER(MATCH($A45,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E45))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A45,TIPOS_OPCION_E,0)),OR($A45="SELECCION_MEJOR_RESPUESTA",$A45="SELECCION_SIMPLE",$A45="SELECCION_UNICA",$A45="SELECCION_DE_LA_MEJOR_RESPUESTA",$A45="SUBITEM_CASO",$A45="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E45))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E46">
-      <x:formula1>IF(ISNUMBER(MATCH($A46,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E46))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A46,TIPOS_OPCION_E,0)),OR($A46="SELECCION_MEJOR_RESPUESTA",$A46="SELECCION_SIMPLE",$A46="SELECCION_UNICA",$A46="SELECCION_DE_LA_MEJOR_RESPUESTA",$A46="SUBITEM_CASO",$A46="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E46))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E47">
-      <x:formula1>IF(ISNUMBER(MATCH($A47,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E47))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A47,TIPOS_OPCION_E,0)),OR($A47="SELECCION_MEJOR_RESPUESTA",$A47="SELECCION_SIMPLE",$A47="SELECCION_UNICA",$A47="SELECCION_DE_LA_MEJOR_RESPUESTA",$A47="SUBITEM_CASO",$A47="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E47))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E48">
-      <x:formula1>IF(ISNUMBER(MATCH($A48,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E48))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A48,TIPOS_OPCION_E,0)),OR($A48="SELECCION_MEJOR_RESPUESTA",$A48="SELECCION_SIMPLE",$A48="SELECCION_UNICA",$A48="SELECCION_DE_LA_MEJOR_RESPUESTA",$A48="SUBITEM_CASO",$A48="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E48))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E49">
-      <x:formula1>IF(ISNUMBER(MATCH($A49,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E49))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A49,TIPOS_OPCION_E,0)),OR($A49="SELECCION_MEJOR_RESPUESTA",$A49="SELECCION_SIMPLE",$A49="SELECCION_UNICA",$A49="SELECCION_DE_LA_MEJOR_RESPUESTA",$A49="SUBITEM_CASO",$A49="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E49))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E5">
-      <x:formula1>IF(ISNUMBER(MATCH($A5,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E5))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A5,TIPOS_OPCION_E,0)),OR($A5="SELECCION_MEJOR_RESPUESTA",$A5="SELECCION_SIMPLE",$A5="SELECCION_UNICA",$A5="SELECCION_DE_LA_MEJOR_RESPUESTA",$A5="SUBITEM_CASO",$A5="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E5))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E50">
-      <x:formula1>IF(ISNUMBER(MATCH($A50,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E50))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A50,TIPOS_OPCION_E,0)),OR($A50="SELECCION_MEJOR_RESPUESTA",$A50="SELECCION_SIMPLE",$A50="SELECCION_UNICA",$A50="SELECCION_DE_LA_MEJOR_RESPUESTA",$A50="SUBITEM_CASO",$A50="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E50))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E51">
-      <x:formula1>IF(ISNUMBER(MATCH($A51,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E51))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A51,TIPOS_OPCION_E,0)),OR($A51="SELECCION_MEJOR_RESPUESTA",$A51="SELECCION_SIMPLE",$A51="SELECCION_UNICA",$A51="SELECCION_DE_LA_MEJOR_RESPUESTA",$A51="SUBITEM_CASO",$A51="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E51))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E52">
-      <x:formula1>IF(ISNUMBER(MATCH($A52,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E52))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A52,TIPOS_OPCION_E,0)),OR($A52="SELECCION_MEJOR_RESPUESTA",$A52="SELECCION_SIMPLE",$A52="SELECCION_UNICA",$A52="SELECCION_DE_LA_MEJOR_RESPUESTA",$A52="SUBITEM_CASO",$A52="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E52))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E53">
-      <x:formula1>IF(ISNUMBER(MATCH($A53,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E53))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A53,TIPOS_OPCION_E,0)),OR($A53="SELECCION_MEJOR_RESPUESTA",$A53="SELECCION_SIMPLE",$A53="SELECCION_UNICA",$A53="SELECCION_DE_LA_MEJOR_RESPUESTA",$A53="SUBITEM_CASO",$A53="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E53))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E54">
-      <x:formula1>IF(ISNUMBER(MATCH($A54,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E54))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A54,TIPOS_OPCION_E,0)),OR($A54="SELECCION_MEJOR_RESPUESTA",$A54="SELECCION_SIMPLE",$A54="SELECCION_UNICA",$A54="SELECCION_DE_LA_MEJOR_RESPUESTA",$A54="SUBITEM_CASO",$A54="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E54))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E55">
-      <x:formula1>IF(ISNUMBER(MATCH($A55,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E55))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A55,TIPOS_OPCION_E,0)),OR($A55="SELECCION_MEJOR_RESPUESTA",$A55="SELECCION_SIMPLE",$A55="SELECCION_UNICA",$A55="SELECCION_DE_LA_MEJOR_RESPUESTA",$A55="SUBITEM_CASO",$A55="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E55))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E56">
-      <x:formula1>IF(ISNUMBER(MATCH($A56,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E56))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A56,TIPOS_OPCION_E,0)),OR($A56="SELECCION_MEJOR_RESPUESTA",$A56="SELECCION_SIMPLE",$A56="SELECCION_UNICA",$A56="SELECCION_DE_LA_MEJOR_RESPUESTA",$A56="SUBITEM_CASO",$A56="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E56))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E57">
-      <x:formula1>IF(ISNUMBER(MATCH($A57,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E57))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A57,TIPOS_OPCION_E,0)),OR($A57="SELECCION_MEJOR_RESPUESTA",$A57="SELECCION_SIMPLE",$A57="SELECCION_UNICA",$A57="SELECCION_DE_LA_MEJOR_RESPUESTA",$A57="SUBITEM_CASO",$A57="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E57))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E58">
-      <x:formula1>IF(ISNUMBER(MATCH($A58,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E58))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A58,TIPOS_OPCION_E,0)),OR($A58="SELECCION_MEJOR_RESPUESTA",$A58="SELECCION_SIMPLE",$A58="SELECCION_UNICA",$A58="SELECCION_DE_LA_MEJOR_RESPUESTA",$A58="SUBITEM_CASO",$A58="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E58))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E59">
-      <x:formula1>IF(ISNUMBER(MATCH($A59,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E59))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A59,TIPOS_OPCION_E,0)),OR($A59="SELECCION_MEJOR_RESPUESTA",$A59="SELECCION_SIMPLE",$A59="SELECCION_UNICA",$A59="SELECCION_DE_LA_MEJOR_RESPUESTA",$A59="SUBITEM_CASO",$A59="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E59))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E6">
-      <x:formula1>IF(ISNUMBER(MATCH($A6,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E6))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A6,TIPOS_OPCION_E,0)),OR($A6="SELECCION_MEJOR_RESPUESTA",$A6="SELECCION_SIMPLE",$A6="SELECCION_UNICA",$A6="SELECCION_DE_LA_MEJOR_RESPUESTA",$A6="SUBITEM_CASO",$A6="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E6))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E60">
-      <x:formula1>IF(ISNUMBER(MATCH($A60,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E60))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A60,TIPOS_OPCION_E,0)),OR($A60="SELECCION_MEJOR_RESPUESTA",$A60="SELECCION_SIMPLE",$A60="SELECCION_UNICA",$A60="SELECCION_DE_LA_MEJOR_RESPUESTA",$A60="SUBITEM_CASO",$A60="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E60))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E61">
-      <x:formula1>IF(ISNUMBER(MATCH($A61,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E61))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A61,TIPOS_OPCION_E,0)),OR($A61="SELECCION_MEJOR_RESPUESTA",$A61="SELECCION_SIMPLE",$A61="SELECCION_UNICA",$A61="SELECCION_DE_LA_MEJOR_RESPUESTA",$A61="SUBITEM_CASO",$A61="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E61))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E7">
-      <x:formula1>IF(ISNUMBER(MATCH($A7,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E7))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A7,TIPOS_OPCION_E,0)),OR($A7="SELECCION_MEJOR_RESPUESTA",$A7="SELECCION_SIMPLE",$A7="SELECCION_UNICA",$A7="SELECCION_DE_LA_MEJOR_RESPUESTA",$A7="SUBITEM_CASO",$A7="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E7))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E8">
-      <x:formula1>IF(ISNUMBER(MATCH($A8,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E8))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A8,TIPOS_OPCION_E,0)),OR($A8="SELECCION_MEJOR_RESPUESTA",$A8="SELECCION_SIMPLE",$A8="SELECCION_UNICA",$A8="SELECCION_DE_LA_MEJOR_RESPUESTA",$A8="SUBITEM_CASO",$A8="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E8))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="E9">
-      <x:formula1>IF(ISNUMBER(MATCH($A9,TIPOS_OPCION_E,0)),TRUE,LEN(TRIM($E9))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A9,TIPOS_OPCION_E,0)),OR($A9="SELECCION_MEJOR_RESPUESTA",$A9="SELECCION_SIMPLE",$A9="SELECCION_UNICA",$A9="SELECCION_DE_LA_MEJOR_RESPUESTA",$A9="SUBITEM_CASO",$A9="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($E9))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F10">
-      <x:formula1>IF(ISNUMBER(MATCH($A10,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F10))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A10,TIPOS_OPCION_F,0)),OR($A10="SELECCION_MEJOR_RESPUESTA",$A10="SELECCION_SIMPLE",$A10="SELECCION_UNICA",$A10="SELECCION_DE_LA_MEJOR_RESPUESTA",$A10="SUBITEM_CASO",$A10="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F10))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F11">
-      <x:formula1>IF(ISNUMBER(MATCH($A11,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F11))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A11,TIPOS_OPCION_F,0)),OR($A11="SELECCION_MEJOR_RESPUESTA",$A11="SELECCION_SIMPLE",$A11="SELECCION_UNICA",$A11="SELECCION_DE_LA_MEJOR_RESPUESTA",$A11="SUBITEM_CASO",$A11="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F11))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F12">
-      <x:formula1>IF(ISNUMBER(MATCH($A12,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F12))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A12,TIPOS_OPCION_F,0)),OR($A12="SELECCION_MEJOR_RESPUESTA",$A12="SELECCION_SIMPLE",$A12="SELECCION_UNICA",$A12="SELECCION_DE_LA_MEJOR_RESPUESTA",$A12="SUBITEM_CASO",$A12="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F12))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F13">
-      <x:formula1>IF(ISNUMBER(MATCH($A13,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F13))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A13,TIPOS_OPCION_F,0)),OR($A13="SELECCION_MEJOR_RESPUESTA",$A13="SELECCION_SIMPLE",$A13="SELECCION_UNICA",$A13="SELECCION_DE_LA_MEJOR_RESPUESTA",$A13="SUBITEM_CASO",$A13="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F13))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F14">
-      <x:formula1>IF(ISNUMBER(MATCH($A14,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F14))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A14,TIPOS_OPCION_F,0)),OR($A14="SELECCION_MEJOR_RESPUESTA",$A14="SELECCION_SIMPLE",$A14="SELECCION_UNICA",$A14="SELECCION_DE_LA_MEJOR_RESPUESTA",$A14="SUBITEM_CASO",$A14="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F14))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F15">
-      <x:formula1>IF(ISNUMBER(MATCH($A15,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F15))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A15,TIPOS_OPCION_F,0)),OR($A15="SELECCION_MEJOR_RESPUESTA",$A15="SELECCION_SIMPLE",$A15="SELECCION_UNICA",$A15="SELECCION_DE_LA_MEJOR_RESPUESTA",$A15="SUBITEM_CASO",$A15="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F15))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F16">
-      <x:formula1>IF(ISNUMBER(MATCH($A16,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F16))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A16,TIPOS_OPCION_F,0)),OR($A16="SELECCION_MEJOR_RESPUESTA",$A16="SELECCION_SIMPLE",$A16="SELECCION_UNICA",$A16="SELECCION_DE_LA_MEJOR_RESPUESTA",$A16="SUBITEM_CASO",$A16="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F16))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F17">
-      <x:formula1>IF(ISNUMBER(MATCH($A17,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F17))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A17,TIPOS_OPCION_F,0)),OR($A17="SELECCION_MEJOR_RESPUESTA",$A17="SELECCION_SIMPLE",$A17="SELECCION_UNICA",$A17="SELECCION_DE_LA_MEJOR_RESPUESTA",$A17="SUBITEM_CASO",$A17="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F17))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F18">
-      <x:formula1>IF(ISNUMBER(MATCH($A18,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F18))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A18,TIPOS_OPCION_F,0)),OR($A18="SELECCION_MEJOR_RESPUESTA",$A18="SELECCION_SIMPLE",$A18="SELECCION_UNICA",$A18="SELECCION_DE_LA_MEJOR_RESPUESTA",$A18="SUBITEM_CASO",$A18="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F18))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F19">
-      <x:formula1>IF(ISNUMBER(MATCH($A19,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F19))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A19,TIPOS_OPCION_F,0)),OR($A19="SELECCION_MEJOR_RESPUESTA",$A19="SELECCION_SIMPLE",$A19="SELECCION_UNICA",$A19="SELECCION_DE_LA_MEJOR_RESPUESTA",$A19="SUBITEM_CASO",$A19="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F19))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F2">
-      <x:formula1>IF(ISNUMBER(MATCH($A2,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F2))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A2,TIPOS_OPCION_F,0)),OR($A2="SELECCION_MEJOR_RESPUESTA",$A2="SELECCION_SIMPLE",$A2="SELECCION_UNICA",$A2="SELECCION_DE_LA_MEJOR_RESPUESTA",$A2="SUBITEM_CASO",$A2="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F2))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F20">
-      <x:formula1>IF(ISNUMBER(MATCH($A20,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F20))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A20,TIPOS_OPCION_F,0)),OR($A20="SELECCION_MEJOR_RESPUESTA",$A20="SELECCION_SIMPLE",$A20="SELECCION_UNICA",$A20="SELECCION_DE_LA_MEJOR_RESPUESTA",$A20="SUBITEM_CASO",$A20="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F20))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F21">
-      <x:formula1>IF(ISNUMBER(MATCH($A21,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F21))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A21,TIPOS_OPCION_F,0)),OR($A21="SELECCION_MEJOR_RESPUESTA",$A21="SELECCION_SIMPLE",$A21="SELECCION_UNICA",$A21="SELECCION_DE_LA_MEJOR_RESPUESTA",$A21="SUBITEM_CASO",$A21="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F21))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F22">
-      <x:formula1>IF(ISNUMBER(MATCH($A22,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F22))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A22,TIPOS_OPCION_F,0)),OR($A22="SELECCION_MEJOR_RESPUESTA",$A22="SELECCION_SIMPLE",$A22="SELECCION_UNICA",$A22="SELECCION_DE_LA_MEJOR_RESPUESTA",$A22="SUBITEM_CASO",$A22="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F22))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F23">
-      <x:formula1>IF(ISNUMBER(MATCH($A23,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F23))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A23,TIPOS_OPCION_F,0)),OR($A23="SELECCION_MEJOR_RESPUESTA",$A23="SELECCION_SIMPLE",$A23="SELECCION_UNICA",$A23="SELECCION_DE_LA_MEJOR_RESPUESTA",$A23="SUBITEM_CASO",$A23="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F23))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F24">
-      <x:formula1>IF(ISNUMBER(MATCH($A24,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F24))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A24,TIPOS_OPCION_F,0)),OR($A24="SELECCION_MEJOR_RESPUESTA",$A24="SELECCION_SIMPLE",$A24="SELECCION_UNICA",$A24="SELECCION_DE_LA_MEJOR_RESPUESTA",$A24="SUBITEM_CASO",$A24="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F24))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F25">
-      <x:formula1>IF(ISNUMBER(MATCH($A25,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F25))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A25,TIPOS_OPCION_F,0)),OR($A25="SELECCION_MEJOR_RESPUESTA",$A25="SELECCION_SIMPLE",$A25="SELECCION_UNICA",$A25="SELECCION_DE_LA_MEJOR_RESPUESTA",$A25="SUBITEM_CASO",$A25="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F25))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F26">
-      <x:formula1>IF(ISNUMBER(MATCH($A26,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F26))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A26,TIPOS_OPCION_F,0)),OR($A26="SELECCION_MEJOR_RESPUESTA",$A26="SELECCION_SIMPLE",$A26="SELECCION_UNICA",$A26="SELECCION_DE_LA_MEJOR_RESPUESTA",$A26="SUBITEM_CASO",$A26="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F26))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F27">
-      <x:formula1>IF(ISNUMBER(MATCH($A27,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F27))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A27,TIPOS_OPCION_F,0)),OR($A27="SELECCION_MEJOR_RESPUESTA",$A27="SELECCION_SIMPLE",$A27="SELECCION_UNICA",$A27="SELECCION_DE_LA_MEJOR_RESPUESTA",$A27="SUBITEM_CASO",$A27="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F27))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F28">
-      <x:formula1>IF(ISNUMBER(MATCH($A28,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F28))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A28,TIPOS_OPCION_F,0)),OR($A28="SELECCION_MEJOR_RESPUESTA",$A28="SELECCION_SIMPLE",$A28="SELECCION_UNICA",$A28="SELECCION_DE_LA_MEJOR_RESPUESTA",$A28="SUBITEM_CASO",$A28="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F28))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F29">
-      <x:formula1>IF(ISNUMBER(MATCH($A29,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F29))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A29,TIPOS_OPCION_F,0)),OR($A29="SELECCION_MEJOR_RESPUESTA",$A29="SELECCION_SIMPLE",$A29="SELECCION_UNICA",$A29="SELECCION_DE_LA_MEJOR_RESPUESTA",$A29="SUBITEM_CASO",$A29="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F29))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F3">
-      <x:formula1>IF(ISNUMBER(MATCH($A3,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F3))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A3,TIPOS_OPCION_F,0)),OR($A3="SELECCION_MEJOR_RESPUESTA",$A3="SELECCION_SIMPLE",$A3="SELECCION_UNICA",$A3="SELECCION_DE_LA_MEJOR_RESPUESTA",$A3="SUBITEM_CASO",$A3="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F3))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F30">
-      <x:formula1>IF(ISNUMBER(MATCH($A30,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F30))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A30,TIPOS_OPCION_F,0)),OR($A30="SELECCION_MEJOR_RESPUESTA",$A30="SELECCION_SIMPLE",$A30="SELECCION_UNICA",$A30="SELECCION_DE_LA_MEJOR_RESPUESTA",$A30="SUBITEM_CASO",$A30="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F30))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F31">
-      <x:formula1>IF(ISNUMBER(MATCH($A31,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F31))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A31,TIPOS_OPCION_F,0)),OR($A31="SELECCION_MEJOR_RESPUESTA",$A31="SELECCION_SIMPLE",$A31="SELECCION_UNICA",$A31="SELECCION_DE_LA_MEJOR_RESPUESTA",$A31="SUBITEM_CASO",$A31="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F31))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F32">
-      <x:formula1>IF(ISNUMBER(MATCH($A32,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F32))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A32,TIPOS_OPCION_F,0)),OR($A32="SELECCION_MEJOR_RESPUESTA",$A32="SELECCION_SIMPLE",$A32="SELECCION_UNICA",$A32="SELECCION_DE_LA_MEJOR_RESPUESTA",$A32="SUBITEM_CASO",$A32="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F32))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F33">
-      <x:formula1>IF(ISNUMBER(MATCH($A33,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F33))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A33,TIPOS_OPCION_F,0)),OR($A33="SELECCION_MEJOR_RESPUESTA",$A33="SELECCION_SIMPLE",$A33="SELECCION_UNICA",$A33="SELECCION_DE_LA_MEJOR_RESPUESTA",$A33="SUBITEM_CASO",$A33="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F33))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F34">
-      <x:formula1>IF(ISNUMBER(MATCH($A34,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F34))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A34,TIPOS_OPCION_F,0)),OR($A34="SELECCION_MEJOR_RESPUESTA",$A34="SELECCION_SIMPLE",$A34="SELECCION_UNICA",$A34="SELECCION_DE_LA_MEJOR_RESPUESTA",$A34="SUBITEM_CASO",$A34="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F34))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F35">
-      <x:formula1>IF(ISNUMBER(MATCH($A35,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F35))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A35,TIPOS_OPCION_F,0)),OR($A35="SELECCION_MEJOR_RESPUESTA",$A35="SELECCION_SIMPLE",$A35="SELECCION_UNICA",$A35="SELECCION_DE_LA_MEJOR_RESPUESTA",$A35="SUBITEM_CASO",$A35="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F35))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F36">
-      <x:formula1>IF(ISNUMBER(MATCH($A36,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F36))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A36,TIPOS_OPCION_F,0)),OR($A36="SELECCION_MEJOR_RESPUESTA",$A36="SELECCION_SIMPLE",$A36="SELECCION_UNICA",$A36="SELECCION_DE_LA_MEJOR_RESPUESTA",$A36="SUBITEM_CASO",$A36="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F36))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F37">
-      <x:formula1>IF(ISNUMBER(MATCH($A37,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F37))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A37,TIPOS_OPCION_F,0)),OR($A37="SELECCION_MEJOR_RESPUESTA",$A37="SELECCION_SIMPLE",$A37="SELECCION_UNICA",$A37="SELECCION_DE_LA_MEJOR_RESPUESTA",$A37="SUBITEM_CASO",$A37="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F37))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F38">
-      <x:formula1>IF(ISNUMBER(MATCH($A38,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F38))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A38,TIPOS_OPCION_F,0)),OR($A38="SELECCION_MEJOR_RESPUESTA",$A38="SELECCION_SIMPLE",$A38="SELECCION_UNICA",$A38="SELECCION_DE_LA_MEJOR_RESPUESTA",$A38="SUBITEM_CASO",$A38="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F38))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F39">
-      <x:formula1>IF(ISNUMBER(MATCH($A39,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F39))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A39,TIPOS_OPCION_F,0)),OR($A39="SELECCION_MEJOR_RESPUESTA",$A39="SELECCION_SIMPLE",$A39="SELECCION_UNICA",$A39="SELECCION_DE_LA_MEJOR_RESPUESTA",$A39="SUBITEM_CASO",$A39="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F39))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F4">
-      <x:formula1>IF(ISNUMBER(MATCH($A4,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F4))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A4,TIPOS_OPCION_F,0)),OR($A4="SELECCION_MEJOR_RESPUESTA",$A4="SELECCION_SIMPLE",$A4="SELECCION_UNICA",$A4="SELECCION_DE_LA_MEJOR_RESPUESTA",$A4="SUBITEM_CASO",$A4="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F4))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F40">
-      <x:formula1>IF(ISNUMBER(MATCH($A40,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F40))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A40,TIPOS_OPCION_F,0)),OR($A40="SELECCION_MEJOR_RESPUESTA",$A40="SELECCION_SIMPLE",$A40="SELECCION_UNICA",$A40="SELECCION_DE_LA_MEJOR_RESPUESTA",$A40="SUBITEM_CASO",$A40="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F40))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F41">
-      <x:formula1>IF(ISNUMBER(MATCH($A41,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F41))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A41,TIPOS_OPCION_F,0)),OR($A41="SELECCION_MEJOR_RESPUESTA",$A41="SELECCION_SIMPLE",$A41="SELECCION_UNICA",$A41="SELECCION_DE_LA_MEJOR_RESPUESTA",$A41="SUBITEM_CASO",$A41="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F41))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F42">
-      <x:formula1>IF(ISNUMBER(MATCH($A42,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F42))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A42,TIPOS_OPCION_F,0)),OR($A42="SELECCION_MEJOR_RESPUESTA",$A42="SELECCION_SIMPLE",$A42="SELECCION_UNICA",$A42="SELECCION_DE_LA_MEJOR_RESPUESTA",$A42="SUBITEM_CASO",$A42="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F42))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F43">
-      <x:formula1>IF(ISNUMBER(MATCH($A43,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F43))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A43,TIPOS_OPCION_F,0)),OR($A43="SELECCION_MEJOR_RESPUESTA",$A43="SELECCION_SIMPLE",$A43="SELECCION_UNICA",$A43="SELECCION_DE_LA_MEJOR_RESPUESTA",$A43="SUBITEM_CASO",$A43="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F43))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F44">
-      <x:formula1>IF(ISNUMBER(MATCH($A44,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F44))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A44,TIPOS_OPCION_F,0)),OR($A44="SELECCION_MEJOR_RESPUESTA",$A44="SELECCION_SIMPLE",$A44="SELECCION_UNICA",$A44="SELECCION_DE_LA_MEJOR_RESPUESTA",$A44="SUBITEM_CASO",$A44="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F44))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F45">
-      <x:formula1>IF(ISNUMBER(MATCH($A45,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F45))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A45,TIPOS_OPCION_F,0)),OR($A45="SELECCION_MEJOR_RESPUESTA",$A45="SELECCION_SIMPLE",$A45="SELECCION_UNICA",$A45="SELECCION_DE_LA_MEJOR_RESPUESTA",$A45="SUBITEM_CASO",$A45="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F45))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F46">
-      <x:formula1>IF(ISNUMBER(MATCH($A46,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F46))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A46,TIPOS_OPCION_F,0)),OR($A46="SELECCION_MEJOR_RESPUESTA",$A46="SELECCION_SIMPLE",$A46="SELECCION_UNICA",$A46="SELECCION_DE_LA_MEJOR_RESPUESTA",$A46="SUBITEM_CASO",$A46="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F46))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F47">
-      <x:formula1>IF(ISNUMBER(MATCH($A47,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F47))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A47,TIPOS_OPCION_F,0)),OR($A47="SELECCION_MEJOR_RESPUESTA",$A47="SELECCION_SIMPLE",$A47="SELECCION_UNICA",$A47="SELECCION_DE_LA_MEJOR_RESPUESTA",$A47="SUBITEM_CASO",$A47="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F47))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F48">
-      <x:formula1>IF(ISNUMBER(MATCH($A48,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F48))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A48,TIPOS_OPCION_F,0)),OR($A48="SELECCION_MEJOR_RESPUESTA",$A48="SELECCION_SIMPLE",$A48="SELECCION_UNICA",$A48="SELECCION_DE_LA_MEJOR_RESPUESTA",$A48="SUBITEM_CASO",$A48="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F48))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F49">
-      <x:formula1>IF(ISNUMBER(MATCH($A49,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F49))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A49,TIPOS_OPCION_F,0)),OR($A49="SELECCION_MEJOR_RESPUESTA",$A49="SELECCION_SIMPLE",$A49="SELECCION_UNICA",$A49="SELECCION_DE_LA_MEJOR_RESPUESTA",$A49="SUBITEM_CASO",$A49="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F49))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F5">
-      <x:formula1>IF(ISNUMBER(MATCH($A5,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F5))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A5,TIPOS_OPCION_F,0)),OR($A5="SELECCION_MEJOR_RESPUESTA",$A5="SELECCION_SIMPLE",$A5="SELECCION_UNICA",$A5="SELECCION_DE_LA_MEJOR_RESPUESTA",$A5="SUBITEM_CASO",$A5="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F5))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F50">
-      <x:formula1>IF(ISNUMBER(MATCH($A50,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F50))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A50,TIPOS_OPCION_F,0)),OR($A50="SELECCION_MEJOR_RESPUESTA",$A50="SELECCION_SIMPLE",$A50="SELECCION_UNICA",$A50="SELECCION_DE_LA_MEJOR_RESPUESTA",$A50="SUBITEM_CASO",$A50="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F50))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F51">
-      <x:formula1>IF(ISNUMBER(MATCH($A51,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F51))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A51,TIPOS_OPCION_F,0)),OR($A51="SELECCION_MEJOR_RESPUESTA",$A51="SELECCION_SIMPLE",$A51="SELECCION_UNICA",$A51="SELECCION_DE_LA_MEJOR_RESPUESTA",$A51="SUBITEM_CASO",$A51="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F51))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F52">
-      <x:formula1>IF(ISNUMBER(MATCH($A52,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F52))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A52,TIPOS_OPCION_F,0)),OR($A52="SELECCION_MEJOR_RESPUESTA",$A52="SELECCION_SIMPLE",$A52="SELECCION_UNICA",$A52="SELECCION_DE_LA_MEJOR_RESPUESTA",$A52="SUBITEM_CASO",$A52="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F52))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F53">
-      <x:formula1>IF(ISNUMBER(MATCH($A53,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F53))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A53,TIPOS_OPCION_F,0)),OR($A53="SELECCION_MEJOR_RESPUESTA",$A53="SELECCION_SIMPLE",$A53="SELECCION_UNICA",$A53="SELECCION_DE_LA_MEJOR_RESPUESTA",$A53="SUBITEM_CASO",$A53="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F53))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F54">
-      <x:formula1>IF(ISNUMBER(MATCH($A54,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F54))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A54,TIPOS_OPCION_F,0)),OR($A54="SELECCION_MEJOR_RESPUESTA",$A54="SELECCION_SIMPLE",$A54="SELECCION_UNICA",$A54="SELECCION_DE_LA_MEJOR_RESPUESTA",$A54="SUBITEM_CASO",$A54="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F54))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F55">
-      <x:formula1>IF(ISNUMBER(MATCH($A55,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F55))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A55,TIPOS_OPCION_F,0)),OR($A55="SELECCION_MEJOR_RESPUESTA",$A55="SELECCION_SIMPLE",$A55="SELECCION_UNICA",$A55="SELECCION_DE_LA_MEJOR_RESPUESTA",$A55="SUBITEM_CASO",$A55="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F55))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F56">
-      <x:formula1>IF(ISNUMBER(MATCH($A56,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F56))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A56,TIPOS_OPCION_F,0)),OR($A56="SELECCION_MEJOR_RESPUESTA",$A56="SELECCION_SIMPLE",$A56="SELECCION_UNICA",$A56="SELECCION_DE_LA_MEJOR_RESPUESTA",$A56="SUBITEM_CASO",$A56="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F56))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F57">
-      <x:formula1>IF(ISNUMBER(MATCH($A57,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F57))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A57,TIPOS_OPCION_F,0)),OR($A57="SELECCION_MEJOR_RESPUESTA",$A57="SELECCION_SIMPLE",$A57="SELECCION_UNICA",$A57="SELECCION_DE_LA_MEJOR_RESPUESTA",$A57="SUBITEM_CASO",$A57="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F57))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F58">
-      <x:formula1>IF(ISNUMBER(MATCH($A58,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F58))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A58,TIPOS_OPCION_F,0)),OR($A58="SELECCION_MEJOR_RESPUESTA",$A58="SELECCION_SIMPLE",$A58="SELECCION_UNICA",$A58="SELECCION_DE_LA_MEJOR_RESPUESTA",$A58="SUBITEM_CASO",$A58="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F58))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F59">
-      <x:formula1>IF(ISNUMBER(MATCH($A59,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F59))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A59,TIPOS_OPCION_F,0)),OR($A59="SELECCION_MEJOR_RESPUESTA",$A59="SELECCION_SIMPLE",$A59="SELECCION_UNICA",$A59="SELECCION_DE_LA_MEJOR_RESPUESTA",$A59="SUBITEM_CASO",$A59="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F59))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F6">
-      <x:formula1>IF(ISNUMBER(MATCH($A6,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F6))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A6,TIPOS_OPCION_F,0)),OR($A6="SELECCION_MEJOR_RESPUESTA",$A6="SELECCION_SIMPLE",$A6="SELECCION_UNICA",$A6="SELECCION_DE_LA_MEJOR_RESPUESTA",$A6="SUBITEM_CASO",$A6="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F6))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F60">
-      <x:formula1>IF(ISNUMBER(MATCH($A60,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F60))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A60,TIPOS_OPCION_F,0)),OR($A60="SELECCION_MEJOR_RESPUESTA",$A60="SELECCION_SIMPLE",$A60="SELECCION_UNICA",$A60="SELECCION_DE_LA_MEJOR_RESPUESTA",$A60="SUBITEM_CASO",$A60="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F60))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F61">
-      <x:formula1>IF(ISNUMBER(MATCH($A61,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F61))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A61,TIPOS_OPCION_F,0)),OR($A61="SELECCION_MEJOR_RESPUESTA",$A61="SELECCION_SIMPLE",$A61="SELECCION_UNICA",$A61="SELECCION_DE_LA_MEJOR_RESPUESTA",$A61="SUBITEM_CASO",$A61="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F61))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F7">
-      <x:formula1>IF(ISNUMBER(MATCH($A7,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F7))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A7,TIPOS_OPCION_F,0)),OR($A7="SELECCION_MEJOR_RESPUESTA",$A7="SELECCION_SIMPLE",$A7="SELECCION_UNICA",$A7="SELECCION_DE_LA_MEJOR_RESPUESTA",$A7="SUBITEM_CASO",$A7="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F7))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F8">
-      <x:formula1>IF(ISNUMBER(MATCH($A8,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F8))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A8,TIPOS_OPCION_F,0)),OR($A8="SELECCION_MEJOR_RESPUESTA",$A8="SELECCION_SIMPLE",$A8="SELECCION_UNICA",$A8="SELECCION_DE_LA_MEJOR_RESPUESTA",$A8="SUBITEM_CASO",$A8="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F8))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="F9">
-      <x:formula1>IF(ISNUMBER(MATCH($A9,TIPOS_OPCION_F,0)),TRUE,LEN(TRIM($F9))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A9,TIPOS_OPCION_F,0)),OR($A9="SELECCION_MEJOR_RESPUESTA",$A9="SELECCION_SIMPLE",$A9="SELECCION_UNICA",$A9="SELECCION_DE_LA_MEJOR_RESPUESTA",$A9="SUBITEM_CASO",$A9="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($F9))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G10">
-      <x:formula1>IF(ISNUMBER(MATCH($A10,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G10))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A10,TIPOS_OPCION_G,0)),OR($A10="SELECCION_MEJOR_RESPUESTA",$A10="SELECCION_SIMPLE",$A10="SELECCION_UNICA",$A10="SELECCION_DE_LA_MEJOR_RESPUESTA",$A10="SUBITEM_CASO",$A10="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G10))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G11">
-      <x:formula1>IF(ISNUMBER(MATCH($A11,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G11))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A11,TIPOS_OPCION_G,0)),OR($A11="SELECCION_MEJOR_RESPUESTA",$A11="SELECCION_SIMPLE",$A11="SELECCION_UNICA",$A11="SELECCION_DE_LA_MEJOR_RESPUESTA",$A11="SUBITEM_CASO",$A11="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G11))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G12">
-      <x:formula1>IF(ISNUMBER(MATCH($A12,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G12))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A12,TIPOS_OPCION_G,0)),OR($A12="SELECCION_MEJOR_RESPUESTA",$A12="SELECCION_SIMPLE",$A12="SELECCION_UNICA",$A12="SELECCION_DE_LA_MEJOR_RESPUESTA",$A12="SUBITEM_CASO",$A12="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G12))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G13">
-      <x:formula1>IF(ISNUMBER(MATCH($A13,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G13))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A13,TIPOS_OPCION_G,0)),OR($A13="SELECCION_MEJOR_RESPUESTA",$A13="SELECCION_SIMPLE",$A13="SELECCION_UNICA",$A13="SELECCION_DE_LA_MEJOR_RESPUESTA",$A13="SUBITEM_CASO",$A13="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G13))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G14">
-      <x:formula1>IF(ISNUMBER(MATCH($A14,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G14))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A14,TIPOS_OPCION_G,0)),OR($A14="SELECCION_MEJOR_RESPUESTA",$A14="SELECCION_SIMPLE",$A14="SELECCION_UNICA",$A14="SELECCION_DE_LA_MEJOR_RESPUESTA",$A14="SUBITEM_CASO",$A14="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G14))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G15">
-      <x:formula1>IF(ISNUMBER(MATCH($A15,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G15))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A15,TIPOS_OPCION_G,0)),OR($A15="SELECCION_MEJOR_RESPUESTA",$A15="SELECCION_SIMPLE",$A15="SELECCION_UNICA",$A15="SELECCION_DE_LA_MEJOR_RESPUESTA",$A15="SUBITEM_CASO",$A15="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G15))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G16">
-      <x:formula1>IF(ISNUMBER(MATCH($A16,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G16))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A16,TIPOS_OPCION_G,0)),OR($A16="SELECCION_MEJOR_RESPUESTA",$A16="SELECCION_SIMPLE",$A16="SELECCION_UNICA",$A16="SELECCION_DE_LA_MEJOR_RESPUESTA",$A16="SUBITEM_CASO",$A16="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G16))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G17">
-      <x:formula1>IF(ISNUMBER(MATCH($A17,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G17))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A17,TIPOS_OPCION_G,0)),OR($A17="SELECCION_MEJOR_RESPUESTA",$A17="SELECCION_SIMPLE",$A17="SELECCION_UNICA",$A17="SELECCION_DE_LA_MEJOR_RESPUESTA",$A17="SUBITEM_CASO",$A17="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G17))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G18">
-      <x:formula1>IF(ISNUMBER(MATCH($A18,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G18))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A18,TIPOS_OPCION_G,0)),OR($A18="SELECCION_MEJOR_RESPUESTA",$A18="SELECCION_SIMPLE",$A18="SELECCION_UNICA",$A18="SELECCION_DE_LA_MEJOR_RESPUESTA",$A18="SUBITEM_CASO",$A18="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G18))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G19">
-      <x:formula1>IF(ISNUMBER(MATCH($A19,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G19))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A19,TIPOS_OPCION_G,0)),OR($A19="SELECCION_MEJOR_RESPUESTA",$A19="SELECCION_SIMPLE",$A19="SELECCION_UNICA",$A19="SELECCION_DE_LA_MEJOR_RESPUESTA",$A19="SUBITEM_CASO",$A19="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G19))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G2">
-      <x:formula1>IF(ISNUMBER(MATCH($A2,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G2))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A2,TIPOS_OPCION_G,0)),OR($A2="SELECCION_MEJOR_RESPUESTA",$A2="SELECCION_SIMPLE",$A2="SELECCION_UNICA",$A2="SELECCION_DE_LA_MEJOR_RESPUESTA",$A2="SUBITEM_CASO",$A2="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G2))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G20">
-      <x:formula1>IF(ISNUMBER(MATCH($A20,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G20))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A20,TIPOS_OPCION_G,0)),OR($A20="SELECCION_MEJOR_RESPUESTA",$A20="SELECCION_SIMPLE",$A20="SELECCION_UNICA",$A20="SELECCION_DE_LA_MEJOR_RESPUESTA",$A20="SUBITEM_CASO",$A20="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G20))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G21">
-      <x:formula1>IF(ISNUMBER(MATCH($A21,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G21))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A21,TIPOS_OPCION_G,0)),OR($A21="SELECCION_MEJOR_RESPUESTA",$A21="SELECCION_SIMPLE",$A21="SELECCION_UNICA",$A21="SELECCION_DE_LA_MEJOR_RESPUESTA",$A21="SUBITEM_CASO",$A21="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G21))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G22">
-      <x:formula1>IF(ISNUMBER(MATCH($A22,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G22))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A22,TIPOS_OPCION_G,0)),OR($A22="SELECCION_MEJOR_RESPUESTA",$A22="SELECCION_SIMPLE",$A22="SELECCION_UNICA",$A22="SELECCION_DE_LA_MEJOR_RESPUESTA",$A22="SUBITEM_CASO",$A22="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G22))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G23">
-      <x:formula1>IF(ISNUMBER(MATCH($A23,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G23))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A23,TIPOS_OPCION_G,0)),OR($A23="SELECCION_MEJOR_RESPUESTA",$A23="SELECCION_SIMPLE",$A23="SELECCION_UNICA",$A23="SELECCION_DE_LA_MEJOR_RESPUESTA",$A23="SUBITEM_CASO",$A23="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G23))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G24">
-      <x:formula1>IF(ISNUMBER(MATCH($A24,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G24))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A24,TIPOS_OPCION_G,0)),OR($A24="SELECCION_MEJOR_RESPUESTA",$A24="SELECCION_SIMPLE",$A24="SELECCION_UNICA",$A24="SELECCION_DE_LA_MEJOR_RESPUESTA",$A24="SUBITEM_CASO",$A24="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G24))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G25">
-      <x:formula1>IF(ISNUMBER(MATCH($A25,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G25))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A25,TIPOS_OPCION_G,0)),OR($A25="SELECCION_MEJOR_RESPUESTA",$A25="SELECCION_SIMPLE",$A25="SELECCION_UNICA",$A25="SELECCION_DE_LA_MEJOR_RESPUESTA",$A25="SUBITEM_CASO",$A25="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G25))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G26">
-      <x:formula1>IF(ISNUMBER(MATCH($A26,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G26))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A26,TIPOS_OPCION_G,0)),OR($A26="SELECCION_MEJOR_RESPUESTA",$A26="SELECCION_SIMPLE",$A26="SELECCION_UNICA",$A26="SELECCION_DE_LA_MEJOR_RESPUESTA",$A26="SUBITEM_CASO",$A26="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G26))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G27">
-      <x:formula1>IF(ISNUMBER(MATCH($A27,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G27))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A27,TIPOS_OPCION_G,0)),OR($A27="SELECCION_MEJOR_RESPUESTA",$A27="SELECCION_SIMPLE",$A27="SELECCION_UNICA",$A27="SELECCION_DE_LA_MEJOR_RESPUESTA",$A27="SUBITEM_CASO",$A27="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G27))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G28">
-      <x:formula1>IF(ISNUMBER(MATCH($A28,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G28))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A28,TIPOS_OPCION_G,0)),OR($A28="SELECCION_MEJOR_RESPUESTA",$A28="SELECCION_SIMPLE",$A28="SELECCION_UNICA",$A28="SELECCION_DE_LA_MEJOR_RESPUESTA",$A28="SUBITEM_CASO",$A28="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G28))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G29">
-      <x:formula1>IF(ISNUMBER(MATCH($A29,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G29))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A29,TIPOS_OPCION_G,0)),OR($A29="SELECCION_MEJOR_RESPUESTA",$A29="SELECCION_SIMPLE",$A29="SELECCION_UNICA",$A29="SELECCION_DE_LA_MEJOR_RESPUESTA",$A29="SUBITEM_CASO",$A29="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G29))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G3">
-      <x:formula1>IF(ISNUMBER(MATCH($A3,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G3))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A3,TIPOS_OPCION_G,0)),OR($A3="SELECCION_MEJOR_RESPUESTA",$A3="SELECCION_SIMPLE",$A3="SELECCION_UNICA",$A3="SELECCION_DE_LA_MEJOR_RESPUESTA",$A3="SUBITEM_CASO",$A3="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G3))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G30">
-      <x:formula1>IF(ISNUMBER(MATCH($A30,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G30))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A30,TIPOS_OPCION_G,0)),OR($A30="SELECCION_MEJOR_RESPUESTA",$A30="SELECCION_SIMPLE",$A30="SELECCION_UNICA",$A30="SELECCION_DE_LA_MEJOR_RESPUESTA",$A30="SUBITEM_CASO",$A30="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G30))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G31">
-      <x:formula1>IF(ISNUMBER(MATCH($A31,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G31))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A31,TIPOS_OPCION_G,0)),OR($A31="SELECCION_MEJOR_RESPUESTA",$A31="SELECCION_SIMPLE",$A31="SELECCION_UNICA",$A31="SELECCION_DE_LA_MEJOR_RESPUESTA",$A31="SUBITEM_CASO",$A31="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G31))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G32">
-      <x:formula1>IF(ISNUMBER(MATCH($A32,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G32))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A32,TIPOS_OPCION_G,0)),OR($A32="SELECCION_MEJOR_RESPUESTA",$A32="SELECCION_SIMPLE",$A32="SELECCION_UNICA",$A32="SELECCION_DE_LA_MEJOR_RESPUESTA",$A32="SUBITEM_CASO",$A32="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G32))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G33">
-      <x:formula1>IF(ISNUMBER(MATCH($A33,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G33))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A33,TIPOS_OPCION_G,0)),OR($A33="SELECCION_MEJOR_RESPUESTA",$A33="SELECCION_SIMPLE",$A33="SELECCION_UNICA",$A33="SELECCION_DE_LA_MEJOR_RESPUESTA",$A33="SUBITEM_CASO",$A33="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G33))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G34">
-      <x:formula1>IF(ISNUMBER(MATCH($A34,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G34))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A34,TIPOS_OPCION_G,0)),OR($A34="SELECCION_MEJOR_RESPUESTA",$A34="SELECCION_SIMPLE",$A34="SELECCION_UNICA",$A34="SELECCION_DE_LA_MEJOR_RESPUESTA",$A34="SUBITEM_CASO",$A34="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G34))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G35">
-      <x:formula1>IF(ISNUMBER(MATCH($A35,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G35))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A35,TIPOS_OPCION_G,0)),OR($A35="SELECCION_MEJOR_RESPUESTA",$A35="SELECCION_SIMPLE",$A35="SELECCION_UNICA",$A35="SELECCION_DE_LA_MEJOR_RESPUESTA",$A35="SUBITEM_CASO",$A35="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G35))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G36">
-      <x:formula1>IF(ISNUMBER(MATCH($A36,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G36))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A36,TIPOS_OPCION_G,0)),OR($A36="SELECCION_MEJOR_RESPUESTA",$A36="SELECCION_SIMPLE",$A36="SELECCION_UNICA",$A36="SELECCION_DE_LA_MEJOR_RESPUESTA",$A36="SUBITEM_CASO",$A36="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G36))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G37">
-      <x:formula1>IF(ISNUMBER(MATCH($A37,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G37))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A37,TIPOS_OPCION_G,0)),OR($A37="SELECCION_MEJOR_RESPUESTA",$A37="SELECCION_SIMPLE",$A37="SELECCION_UNICA",$A37="SELECCION_DE_LA_MEJOR_RESPUESTA",$A37="SUBITEM_CASO",$A37="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G37))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G38">
-      <x:formula1>IF(ISNUMBER(MATCH($A38,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G38))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A38,TIPOS_OPCION_G,0)),OR($A38="SELECCION_MEJOR_RESPUESTA",$A38="SELECCION_SIMPLE",$A38="SELECCION_UNICA",$A38="SELECCION_DE_LA_MEJOR_RESPUESTA",$A38="SUBITEM_CASO",$A38="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G38))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G39">
-      <x:formula1>IF(ISNUMBER(MATCH($A39,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G39))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A39,TIPOS_OPCION_G,0)),OR($A39="SELECCION_MEJOR_RESPUESTA",$A39="SELECCION_SIMPLE",$A39="SELECCION_UNICA",$A39="SELECCION_DE_LA_MEJOR_RESPUESTA",$A39="SUBITEM_CASO",$A39="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G39))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G4">
-      <x:formula1>IF(ISNUMBER(MATCH($A4,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G4))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A4,TIPOS_OPCION_G,0)),OR($A4="SELECCION_MEJOR_RESPUESTA",$A4="SELECCION_SIMPLE",$A4="SELECCION_UNICA",$A4="SELECCION_DE_LA_MEJOR_RESPUESTA",$A4="SUBITEM_CASO",$A4="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G4))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G40">
-      <x:formula1>IF(ISNUMBER(MATCH($A40,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G40))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A40,TIPOS_OPCION_G,0)),OR($A40="SELECCION_MEJOR_RESPUESTA",$A40="SELECCION_SIMPLE",$A40="SELECCION_UNICA",$A40="SELECCION_DE_LA_MEJOR_RESPUESTA",$A40="SUBITEM_CASO",$A40="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G40))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G41">
-      <x:formula1>IF(ISNUMBER(MATCH($A41,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G41))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A41,TIPOS_OPCION_G,0)),OR($A41="SELECCION_MEJOR_RESPUESTA",$A41="SELECCION_SIMPLE",$A41="SELECCION_UNICA",$A41="SELECCION_DE_LA_MEJOR_RESPUESTA",$A41="SUBITEM_CASO",$A41="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G41))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G42">
-      <x:formula1>IF(ISNUMBER(MATCH($A42,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G42))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A42,TIPOS_OPCION_G,0)),OR($A42="SELECCION_MEJOR_RESPUESTA",$A42="SELECCION_SIMPLE",$A42="SELECCION_UNICA",$A42="SELECCION_DE_LA_MEJOR_RESPUESTA",$A42="SUBITEM_CASO",$A42="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G42))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G43">
-      <x:formula1>IF(ISNUMBER(MATCH($A43,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G43))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A43,TIPOS_OPCION_G,0)),OR($A43="SELECCION_MEJOR_RESPUESTA",$A43="SELECCION_SIMPLE",$A43="SELECCION_UNICA",$A43="SELECCION_DE_LA_MEJOR_RESPUESTA",$A43="SUBITEM_CASO",$A43="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G43))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G44">
-      <x:formula1>IF(ISNUMBER(MATCH($A44,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G44))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A44,TIPOS_OPCION_G,0)),OR($A44="SELECCION_MEJOR_RESPUESTA",$A44="SELECCION_SIMPLE",$A44="SELECCION_UNICA",$A44="SELECCION_DE_LA_MEJOR_RESPUESTA",$A44="SUBITEM_CASO",$A44="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G44))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G45">
-      <x:formula1>IF(ISNUMBER(MATCH($A45,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G45))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A45,TIPOS_OPCION_G,0)),OR($A45="SELECCION_MEJOR_RESPUESTA",$A45="SELECCION_SIMPLE",$A45="SELECCION_UNICA",$A45="SELECCION_DE_LA_MEJOR_RESPUESTA",$A45="SUBITEM_CASO",$A45="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G45))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G46">
-      <x:formula1>IF(ISNUMBER(MATCH($A46,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G46))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A46,TIPOS_OPCION_G,0)),OR($A46="SELECCION_MEJOR_RESPUESTA",$A46="SELECCION_SIMPLE",$A46="SELECCION_UNICA",$A46="SELECCION_DE_LA_MEJOR_RESPUESTA",$A46="SUBITEM_CASO",$A46="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G46))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G47">
-      <x:formula1>IF(ISNUMBER(MATCH($A47,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G47))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A47,TIPOS_OPCION_G,0)),OR($A47="SELECCION_MEJOR_RESPUESTA",$A47="SELECCION_SIMPLE",$A47="SELECCION_UNICA",$A47="SELECCION_DE_LA_MEJOR_RESPUESTA",$A47="SUBITEM_CASO",$A47="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G47))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G48">
-      <x:formula1>IF(ISNUMBER(MATCH($A48,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G48))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A48,TIPOS_OPCION_G,0)),OR($A48="SELECCION_MEJOR_RESPUESTA",$A48="SELECCION_SIMPLE",$A48="SELECCION_UNICA",$A48="SELECCION_DE_LA_MEJOR_RESPUESTA",$A48="SUBITEM_CASO",$A48="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G48))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G49">
-      <x:formula1>IF(ISNUMBER(MATCH($A49,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G49))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A49,TIPOS_OPCION_G,0)),OR($A49="SELECCION_MEJOR_RESPUESTA",$A49="SELECCION_SIMPLE",$A49="SELECCION_UNICA",$A49="SELECCION_DE_LA_MEJOR_RESPUESTA",$A49="SUBITEM_CASO",$A49="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G49))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G5">
-      <x:formula1>IF(ISNUMBER(MATCH($A5,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G5))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A5,TIPOS_OPCION_G,0)),OR($A5="SELECCION_MEJOR_RESPUESTA",$A5="SELECCION_SIMPLE",$A5="SELECCION_UNICA",$A5="SELECCION_DE_LA_MEJOR_RESPUESTA",$A5="SUBITEM_CASO",$A5="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G5))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G50">
-      <x:formula1>IF(ISNUMBER(MATCH($A50,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G50))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A50,TIPOS_OPCION_G,0)),OR($A50="SELECCION_MEJOR_RESPUESTA",$A50="SELECCION_SIMPLE",$A50="SELECCION_UNICA",$A50="SELECCION_DE_LA_MEJOR_RESPUESTA",$A50="SUBITEM_CASO",$A50="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G50))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G51">
-      <x:formula1>IF(ISNUMBER(MATCH($A51,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G51))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A51,TIPOS_OPCION_G,0)),OR($A51="SELECCION_MEJOR_RESPUESTA",$A51="SELECCION_SIMPLE",$A51="SELECCION_UNICA",$A51="SELECCION_DE_LA_MEJOR_RESPUESTA",$A51="SUBITEM_CASO",$A51="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G51))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G52">
-      <x:formula1>IF(ISNUMBER(MATCH($A52,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G52))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A52,TIPOS_OPCION_G,0)),OR($A52="SELECCION_MEJOR_RESPUESTA",$A52="SELECCION_SIMPLE",$A52="SELECCION_UNICA",$A52="SELECCION_DE_LA_MEJOR_RESPUESTA",$A52="SUBITEM_CASO",$A52="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G52))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G53">
-      <x:formula1>IF(ISNUMBER(MATCH($A53,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G53))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A53,TIPOS_OPCION_G,0)),OR($A53="SELECCION_MEJOR_RESPUESTA",$A53="SELECCION_SIMPLE",$A53="SELECCION_UNICA",$A53="SELECCION_DE_LA_MEJOR_RESPUESTA",$A53="SUBITEM_CASO",$A53="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G53))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G54">
-      <x:formula1>IF(ISNUMBER(MATCH($A54,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G54))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A54,TIPOS_OPCION_G,0)),OR($A54="SELECCION_MEJOR_RESPUESTA",$A54="SELECCION_SIMPLE",$A54="SELECCION_UNICA",$A54="SELECCION_DE_LA_MEJOR_RESPUESTA",$A54="SUBITEM_CASO",$A54="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G54))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G55">
-      <x:formula1>IF(ISNUMBER(MATCH($A55,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G55))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A55,TIPOS_OPCION_G,0)),OR($A55="SELECCION_MEJOR_RESPUESTA",$A55="SELECCION_SIMPLE",$A55="SELECCION_UNICA",$A55="SELECCION_DE_LA_MEJOR_RESPUESTA",$A55="SUBITEM_CASO",$A55="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G55))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G56">
-      <x:formula1>IF(ISNUMBER(MATCH($A56,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G56))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A56,TIPOS_OPCION_G,0)),OR($A56="SELECCION_MEJOR_RESPUESTA",$A56="SELECCION_SIMPLE",$A56="SELECCION_UNICA",$A56="SELECCION_DE_LA_MEJOR_RESPUESTA",$A56="SUBITEM_CASO",$A56="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G56))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G57">
-      <x:formula1>IF(ISNUMBER(MATCH($A57,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G57))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A57,TIPOS_OPCION_G,0)),OR($A57="SELECCION_MEJOR_RESPUESTA",$A57="SELECCION_SIMPLE",$A57="SELECCION_UNICA",$A57="SELECCION_DE_LA_MEJOR_RESPUESTA",$A57="SUBITEM_CASO",$A57="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G57))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G58">
-      <x:formula1>IF(ISNUMBER(MATCH($A58,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G58))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A58,TIPOS_OPCION_G,0)),OR($A58="SELECCION_MEJOR_RESPUESTA",$A58="SELECCION_SIMPLE",$A58="SELECCION_UNICA",$A58="SELECCION_DE_LA_MEJOR_RESPUESTA",$A58="SUBITEM_CASO",$A58="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G58))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G59">
-      <x:formula1>IF(ISNUMBER(MATCH($A59,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G59))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A59,TIPOS_OPCION_G,0)),OR($A59="SELECCION_MEJOR_RESPUESTA",$A59="SELECCION_SIMPLE",$A59="SELECCION_UNICA",$A59="SELECCION_DE_LA_MEJOR_RESPUESTA",$A59="SUBITEM_CASO",$A59="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G59))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G6">
-      <x:formula1>IF(ISNUMBER(MATCH($A6,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G6))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A6,TIPOS_OPCION_G,0)),OR($A6="SELECCION_MEJOR_RESPUESTA",$A6="SELECCION_SIMPLE",$A6="SELECCION_UNICA",$A6="SELECCION_DE_LA_MEJOR_RESPUESTA",$A6="SUBITEM_CASO",$A6="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G6))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G60">
-      <x:formula1>IF(ISNUMBER(MATCH($A60,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G60))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A60,TIPOS_OPCION_G,0)),OR($A60="SELECCION_MEJOR_RESPUESTA",$A60="SELECCION_SIMPLE",$A60="SELECCION_UNICA",$A60="SELECCION_DE_LA_MEJOR_RESPUESTA",$A60="SUBITEM_CASO",$A60="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G60))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G61">
-      <x:formula1>IF(ISNUMBER(MATCH($A61,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G61))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A61,TIPOS_OPCION_G,0)),OR($A61="SELECCION_MEJOR_RESPUESTA",$A61="SELECCION_SIMPLE",$A61="SELECCION_UNICA",$A61="SELECCION_DE_LA_MEJOR_RESPUESTA",$A61="SUBITEM_CASO",$A61="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G61))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G7">
-      <x:formula1>IF(ISNUMBER(MATCH($A7,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G7))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A7,TIPOS_OPCION_G,0)),OR($A7="SELECCION_MEJOR_RESPUESTA",$A7="SELECCION_SIMPLE",$A7="SELECCION_UNICA",$A7="SELECCION_DE_LA_MEJOR_RESPUESTA",$A7="SUBITEM_CASO",$A7="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G7))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G8">
-      <x:formula1>IF(ISNUMBER(MATCH($A8,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G8))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A8,TIPOS_OPCION_G,0)),OR($A8="SELECCION_MEJOR_RESPUESTA",$A8="SELECCION_SIMPLE",$A8="SELECCION_UNICA",$A8="SELECCION_DE_LA_MEJOR_RESPUESTA",$A8="SUBITEM_CASO",$A8="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G8))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="G9">
-      <x:formula1>IF(ISNUMBER(MATCH($A9,TIPOS_OPCION_G,0)),TRUE,LEN(TRIM($G9))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A9,TIPOS_OPCION_G,0)),OR($A9="SELECCION_MEJOR_RESPUESTA",$A9="SELECCION_SIMPLE",$A9="SELECCION_UNICA",$A9="SELECCION_DE_LA_MEJOR_RESPUESTA",$A9="SUBITEM_CASO",$A9="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($G9))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H10">
-      <x:formula1>IF(ISNUMBER(MATCH($A10,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H10))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A10,TIPOS_OPCION_H,0)),OR($A10="SELECCION_MEJOR_RESPUESTA",$A10="SELECCION_SIMPLE",$A10="SELECCION_UNICA",$A10="SELECCION_DE_LA_MEJOR_RESPUESTA",$A10="SUBITEM_CASO",$A10="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H10))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H11">
-      <x:formula1>IF(ISNUMBER(MATCH($A11,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H11))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A11,TIPOS_OPCION_H,0)),OR($A11="SELECCION_MEJOR_RESPUESTA",$A11="SELECCION_SIMPLE",$A11="SELECCION_UNICA",$A11="SELECCION_DE_LA_MEJOR_RESPUESTA",$A11="SUBITEM_CASO",$A11="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H11))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H12">
-      <x:formula1>IF(ISNUMBER(MATCH($A12,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H12))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A12,TIPOS_OPCION_H,0)),OR($A12="SELECCION_MEJOR_RESPUESTA",$A12="SELECCION_SIMPLE",$A12="SELECCION_UNICA",$A12="SELECCION_DE_LA_MEJOR_RESPUESTA",$A12="SUBITEM_CASO",$A12="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H12))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H13">
-      <x:formula1>IF(ISNUMBER(MATCH($A13,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H13))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A13,TIPOS_OPCION_H,0)),OR($A13="SELECCION_MEJOR_RESPUESTA",$A13="SELECCION_SIMPLE",$A13="SELECCION_UNICA",$A13="SELECCION_DE_LA_MEJOR_RESPUESTA",$A13="SUBITEM_CASO",$A13="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H13))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H14">
-      <x:formula1>IF(ISNUMBER(MATCH($A14,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H14))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A14,TIPOS_OPCION_H,0)),OR($A14="SELECCION_MEJOR_RESPUESTA",$A14="SELECCION_SIMPLE",$A14="SELECCION_UNICA",$A14="SELECCION_DE_LA_MEJOR_RESPUESTA",$A14="SUBITEM_CASO",$A14="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H14))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H15">
-      <x:formula1>IF(ISNUMBER(MATCH($A15,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H15))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A15,TIPOS_OPCION_H,0)),OR($A15="SELECCION_MEJOR_RESPUESTA",$A15="SELECCION_SIMPLE",$A15="SELECCION_UNICA",$A15="SELECCION_DE_LA_MEJOR_RESPUESTA",$A15="SUBITEM_CASO",$A15="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H15))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H16">
-      <x:formula1>IF(ISNUMBER(MATCH($A16,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H16))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A16,TIPOS_OPCION_H,0)),OR($A16="SELECCION_MEJOR_RESPUESTA",$A16="SELECCION_SIMPLE",$A16="SELECCION_UNICA",$A16="SELECCION_DE_LA_MEJOR_RESPUESTA",$A16="SUBITEM_CASO",$A16="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H16))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H17">
-      <x:formula1>IF(ISNUMBER(MATCH($A17,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H17))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A17,TIPOS_OPCION_H,0)),OR($A17="SELECCION_MEJOR_RESPUESTA",$A17="SELECCION_SIMPLE",$A17="SELECCION_UNICA",$A17="SELECCION_DE_LA_MEJOR_RESPUESTA",$A17="SUBITEM_CASO",$A17="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H17))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H18">
-      <x:formula1>IF(ISNUMBER(MATCH($A18,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H18))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A18,TIPOS_OPCION_H,0)),OR($A18="SELECCION_MEJOR_RESPUESTA",$A18="SELECCION_SIMPLE",$A18="SELECCION_UNICA",$A18="SELECCION_DE_LA_MEJOR_RESPUESTA",$A18="SUBITEM_CASO",$A18="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H18))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H19">
-      <x:formula1>IF(ISNUMBER(MATCH($A19,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H19))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A19,TIPOS_OPCION_H,0)),OR($A19="SELECCION_MEJOR_RESPUESTA",$A19="SELECCION_SIMPLE",$A19="SELECCION_UNICA",$A19="SELECCION_DE_LA_MEJOR_RESPUESTA",$A19="SUBITEM_CASO",$A19="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H19))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H2">
-      <x:formula1>IF(ISNUMBER(MATCH($A2,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H2))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A2,TIPOS_OPCION_H,0)),OR($A2="SELECCION_MEJOR_RESPUESTA",$A2="SELECCION_SIMPLE",$A2="SELECCION_UNICA",$A2="SELECCION_DE_LA_MEJOR_RESPUESTA",$A2="SUBITEM_CASO",$A2="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H2))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H20">
-      <x:formula1>IF(ISNUMBER(MATCH($A20,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H20))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A20,TIPOS_OPCION_H,0)),OR($A20="SELECCION_MEJOR_RESPUESTA",$A20="SELECCION_SIMPLE",$A20="SELECCION_UNICA",$A20="SELECCION_DE_LA_MEJOR_RESPUESTA",$A20="SUBITEM_CASO",$A20="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H20))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H21">
-      <x:formula1>IF(ISNUMBER(MATCH($A21,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H21))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A21,TIPOS_OPCION_H,0)),OR($A21="SELECCION_MEJOR_RESPUESTA",$A21="SELECCION_SIMPLE",$A21="SELECCION_UNICA",$A21="SELECCION_DE_LA_MEJOR_RESPUESTA",$A21="SUBITEM_CASO",$A21="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H21))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H22">
-      <x:formula1>IF(ISNUMBER(MATCH($A22,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H22))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A22,TIPOS_OPCION_H,0)),OR($A22="SELECCION_MEJOR_RESPUESTA",$A22="SELECCION_SIMPLE",$A22="SELECCION_UNICA",$A22="SELECCION_DE_LA_MEJOR_RESPUESTA",$A22="SUBITEM_CASO",$A22="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H22))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H23">
-      <x:formula1>IF(ISNUMBER(MATCH($A23,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H23))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A23,TIPOS_OPCION_H,0)),OR($A23="SELECCION_MEJOR_RESPUESTA",$A23="SELECCION_SIMPLE",$A23="SELECCION_UNICA",$A23="SELECCION_DE_LA_MEJOR_RESPUESTA",$A23="SUBITEM_CASO",$A23="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H23))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H24">
-      <x:formula1>IF(ISNUMBER(MATCH($A24,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H24))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A24,TIPOS_OPCION_H,0)),OR($A24="SELECCION_MEJOR_RESPUESTA",$A24="SELECCION_SIMPLE",$A24="SELECCION_UNICA",$A24="SELECCION_DE_LA_MEJOR_RESPUESTA",$A24="SUBITEM_CASO",$A24="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H24))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H25">
-      <x:formula1>IF(ISNUMBER(MATCH($A25,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H25))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A25,TIPOS_OPCION_H,0)),OR($A25="SELECCION_MEJOR_RESPUESTA",$A25="SELECCION_SIMPLE",$A25="SELECCION_UNICA",$A25="SELECCION_DE_LA_MEJOR_RESPUESTA",$A25="SUBITEM_CASO",$A25="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H25))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H26">
-      <x:formula1>IF(ISNUMBER(MATCH($A26,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H26))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A26,TIPOS_OPCION_H,0)),OR($A26="SELECCION_MEJOR_RESPUESTA",$A26="SELECCION_SIMPLE",$A26="SELECCION_UNICA",$A26="SELECCION_DE_LA_MEJOR_RESPUESTA",$A26="SUBITEM_CASO",$A26="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H26))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H27">
-      <x:formula1>IF(ISNUMBER(MATCH($A27,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H27))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A27,TIPOS_OPCION_H,0)),OR($A27="SELECCION_MEJOR_RESPUESTA",$A27="SELECCION_SIMPLE",$A27="SELECCION_UNICA",$A27="SELECCION_DE_LA_MEJOR_RESPUESTA",$A27="SUBITEM_CASO",$A27="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H27))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H28">
-      <x:formula1>IF(ISNUMBER(MATCH($A28,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H28))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A28,TIPOS_OPCION_H,0)),OR($A28="SELECCION_MEJOR_RESPUESTA",$A28="SELECCION_SIMPLE",$A28="SELECCION_UNICA",$A28="SELECCION_DE_LA_MEJOR_RESPUESTA",$A28="SUBITEM_CASO",$A28="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H28))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H29">
-      <x:formula1>IF(ISNUMBER(MATCH($A29,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H29))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A29,TIPOS_OPCION_H,0)),OR($A29="SELECCION_MEJOR_RESPUESTA",$A29="SELECCION_SIMPLE",$A29="SELECCION_UNICA",$A29="SELECCION_DE_LA_MEJOR_RESPUESTA",$A29="SUBITEM_CASO",$A29="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H29))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H3">
-      <x:formula1>IF(ISNUMBER(MATCH($A3,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H3))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A3,TIPOS_OPCION_H,0)),OR($A3="SELECCION_MEJOR_RESPUESTA",$A3="SELECCION_SIMPLE",$A3="SELECCION_UNICA",$A3="SELECCION_DE_LA_MEJOR_RESPUESTA",$A3="SUBITEM_CASO",$A3="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H3))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H30">
-      <x:formula1>IF(ISNUMBER(MATCH($A30,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H30))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A30,TIPOS_OPCION_H,0)),OR($A30="SELECCION_MEJOR_RESPUESTA",$A30="SELECCION_SIMPLE",$A30="SELECCION_UNICA",$A30="SELECCION_DE_LA_MEJOR_RESPUESTA",$A30="SUBITEM_CASO",$A30="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H30))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H31">
-      <x:formula1>IF(ISNUMBER(MATCH($A31,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H31))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A31,TIPOS_OPCION_H,0)),OR($A31="SELECCION_MEJOR_RESPUESTA",$A31="SELECCION_SIMPLE",$A31="SELECCION_UNICA",$A31="SELECCION_DE_LA_MEJOR_RESPUESTA",$A31="SUBITEM_CASO",$A31="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H31))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H32">
-      <x:formula1>IF(ISNUMBER(MATCH($A32,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H32))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A32,TIPOS_OPCION_H,0)),OR($A32="SELECCION_MEJOR_RESPUESTA",$A32="SELECCION_SIMPLE",$A32="SELECCION_UNICA",$A32="SELECCION_DE_LA_MEJOR_RESPUESTA",$A32="SUBITEM_CASO",$A32="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H32))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H33">
-      <x:formula1>IF(ISNUMBER(MATCH($A33,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H33))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A33,TIPOS_OPCION_H,0)),OR($A33="SELECCION_MEJOR_RESPUESTA",$A33="SELECCION_SIMPLE",$A33="SELECCION_UNICA",$A33="SELECCION_DE_LA_MEJOR_RESPUESTA",$A33="SUBITEM_CASO",$A33="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H33))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H34">
-      <x:formula1>IF(ISNUMBER(MATCH($A34,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H34))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A34,TIPOS_OPCION_H,0)),OR($A34="SELECCION_MEJOR_RESPUESTA",$A34="SELECCION_SIMPLE",$A34="SELECCION_UNICA",$A34="SELECCION_DE_LA_MEJOR_RESPUESTA",$A34="SUBITEM_CASO",$A34="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H34))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H35">
-      <x:formula1>IF(ISNUMBER(MATCH($A35,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H35))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A35,TIPOS_OPCION_H,0)),OR($A35="SELECCION_MEJOR_RESPUESTA",$A35="SELECCION_SIMPLE",$A35="SELECCION_UNICA",$A35="SELECCION_DE_LA_MEJOR_RESPUESTA",$A35="SUBITEM_CASO",$A35="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H35))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H36">
-      <x:formula1>IF(ISNUMBER(MATCH($A36,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H36))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A36,TIPOS_OPCION_H,0)),OR($A36="SELECCION_MEJOR_RESPUESTA",$A36="SELECCION_SIMPLE",$A36="SELECCION_UNICA",$A36="SELECCION_DE_LA_MEJOR_RESPUESTA",$A36="SUBITEM_CASO",$A36="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H36))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H37">
-      <x:formula1>IF(ISNUMBER(MATCH($A37,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H37))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A37,TIPOS_OPCION_H,0)),OR($A37="SELECCION_MEJOR_RESPUESTA",$A37="SELECCION_SIMPLE",$A37="SELECCION_UNICA",$A37="SELECCION_DE_LA_MEJOR_RESPUESTA",$A37="SUBITEM_CASO",$A37="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H37))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H38">
-      <x:formula1>IF(ISNUMBER(MATCH($A38,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H38))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A38,TIPOS_OPCION_H,0)),OR($A38="SELECCION_MEJOR_RESPUESTA",$A38="SELECCION_SIMPLE",$A38="SELECCION_UNICA",$A38="SELECCION_DE_LA_MEJOR_RESPUESTA",$A38="SUBITEM_CASO",$A38="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H38))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H39">
-      <x:formula1>IF(ISNUMBER(MATCH($A39,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H39))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A39,TIPOS_OPCION_H,0)),OR($A39="SELECCION_MEJOR_RESPUESTA",$A39="SELECCION_SIMPLE",$A39="SELECCION_UNICA",$A39="SELECCION_DE_LA_MEJOR_RESPUESTA",$A39="SUBITEM_CASO",$A39="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H39))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H4">
-      <x:formula1>IF(ISNUMBER(MATCH($A4,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H4))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A4,TIPOS_OPCION_H,0)),OR($A4="SELECCION_MEJOR_RESPUESTA",$A4="SELECCION_SIMPLE",$A4="SELECCION_UNICA",$A4="SELECCION_DE_LA_MEJOR_RESPUESTA",$A4="SUBITEM_CASO",$A4="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H4))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H40">
-      <x:formula1>IF(ISNUMBER(MATCH($A40,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H40))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A40,TIPOS_OPCION_H,0)),OR($A40="SELECCION_MEJOR_RESPUESTA",$A40="SELECCION_SIMPLE",$A40="SELECCION_UNICA",$A40="SELECCION_DE_LA_MEJOR_RESPUESTA",$A40="SUBITEM_CASO",$A40="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H40))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H41">
-      <x:formula1>IF(ISNUMBER(MATCH($A41,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H41))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A41,TIPOS_OPCION_H,0)),OR($A41="SELECCION_MEJOR_RESPUESTA",$A41="SELECCION_SIMPLE",$A41="SELECCION_UNICA",$A41="SELECCION_DE_LA_MEJOR_RESPUESTA",$A41="SUBITEM_CASO",$A41="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H41))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H42">
-      <x:formula1>IF(ISNUMBER(MATCH($A42,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H42))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A42,TIPOS_OPCION_H,0)),OR($A42="SELECCION_MEJOR_RESPUESTA",$A42="SELECCION_SIMPLE",$A42="SELECCION_UNICA",$A42="SELECCION_DE_LA_MEJOR_RESPUESTA",$A42="SUBITEM_CASO",$A42="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H42))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H43">
-      <x:formula1>IF(ISNUMBER(MATCH($A43,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H43))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A43,TIPOS_OPCION_H,0)),OR($A43="SELECCION_MEJOR_RESPUESTA",$A43="SELECCION_SIMPLE",$A43="SELECCION_UNICA",$A43="SELECCION_DE_LA_MEJOR_RESPUESTA",$A43="SUBITEM_CASO",$A43="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H43))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H44">
-      <x:formula1>IF(ISNUMBER(MATCH($A44,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H44))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A44,TIPOS_OPCION_H,0)),OR($A44="SELECCION_MEJOR_RESPUESTA",$A44="SELECCION_SIMPLE",$A44="SELECCION_UNICA",$A44="SELECCION_DE_LA_MEJOR_RESPUESTA",$A44="SUBITEM_CASO",$A44="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H44))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H45">
-      <x:formula1>IF(ISNUMBER(MATCH($A45,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H45))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A45,TIPOS_OPCION_H,0)),OR($A45="SELECCION_MEJOR_RESPUESTA",$A45="SELECCION_SIMPLE",$A45="SELECCION_UNICA",$A45="SELECCION_DE_LA_MEJOR_RESPUESTA",$A45="SUBITEM_CASO",$A45="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H45))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H46">
-      <x:formula1>IF(ISNUMBER(MATCH($A46,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H46))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A46,TIPOS_OPCION_H,0)),OR($A46="SELECCION_MEJOR_RESPUESTA",$A46="SELECCION_SIMPLE",$A46="SELECCION_UNICA",$A46="SELECCION_DE_LA_MEJOR_RESPUESTA",$A46="SUBITEM_CASO",$A46="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H46))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H47">
-      <x:formula1>IF(ISNUMBER(MATCH($A47,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H47))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A47,TIPOS_OPCION_H,0)),OR($A47="SELECCION_MEJOR_RESPUESTA",$A47="SELECCION_SIMPLE",$A47="SELECCION_UNICA",$A47="SELECCION_DE_LA_MEJOR_RESPUESTA",$A47="SUBITEM_CASO",$A47="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H47))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H48">
-      <x:formula1>IF(ISNUMBER(MATCH($A48,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H48))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A48,TIPOS_OPCION_H,0)),OR($A48="SELECCION_MEJOR_RESPUESTA",$A48="SELECCION_SIMPLE",$A48="SELECCION_UNICA",$A48="SELECCION_DE_LA_MEJOR_RESPUESTA",$A48="SUBITEM_CASO",$A48="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H48))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H49">
-      <x:formula1>IF(ISNUMBER(MATCH($A49,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H49))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A49,TIPOS_OPCION_H,0)),OR($A49="SELECCION_MEJOR_RESPUESTA",$A49="SELECCION_SIMPLE",$A49="SELECCION_UNICA",$A49="SELECCION_DE_LA_MEJOR_RESPUESTA",$A49="SUBITEM_CASO",$A49="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H49))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H5">
-      <x:formula1>IF(ISNUMBER(MATCH($A5,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H5))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A5,TIPOS_OPCION_H,0)),OR($A5="SELECCION_MEJOR_RESPUESTA",$A5="SELECCION_SIMPLE",$A5="SELECCION_UNICA",$A5="SELECCION_DE_LA_MEJOR_RESPUESTA",$A5="SUBITEM_CASO",$A5="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H5))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H50">
-      <x:formula1>IF(ISNUMBER(MATCH($A50,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H50))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A50,TIPOS_OPCION_H,0)),OR($A50="SELECCION_MEJOR_RESPUESTA",$A50="SELECCION_SIMPLE",$A50="SELECCION_UNICA",$A50="SELECCION_DE_LA_MEJOR_RESPUESTA",$A50="SUBITEM_CASO",$A50="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H50))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H51">
-      <x:formula1>IF(ISNUMBER(MATCH($A51,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H51))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A51,TIPOS_OPCION_H,0)),OR($A51="SELECCION_MEJOR_RESPUESTA",$A51="SELECCION_SIMPLE",$A51="SELECCION_UNICA",$A51="SELECCION_DE_LA_MEJOR_RESPUESTA",$A51="SUBITEM_CASO",$A51="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H51))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H52">
-      <x:formula1>IF(ISNUMBER(MATCH($A52,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H52))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A52,TIPOS_OPCION_H,0)),OR($A52="SELECCION_MEJOR_RESPUESTA",$A52="SELECCION_SIMPLE",$A52="SELECCION_UNICA",$A52="SELECCION_DE_LA_MEJOR_RESPUESTA",$A52="SUBITEM_CASO",$A52="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H52))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H53">
-      <x:formula1>IF(ISNUMBER(MATCH($A53,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H53))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A53,TIPOS_OPCION_H,0)),OR($A53="SELECCION_MEJOR_RESPUESTA",$A53="SELECCION_SIMPLE",$A53="SELECCION_UNICA",$A53="SELECCION_DE_LA_MEJOR_RESPUESTA",$A53="SUBITEM_CASO",$A53="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H53))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H54">
-      <x:formula1>IF(ISNUMBER(MATCH($A54,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H54))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A54,TIPOS_OPCION_H,0)),OR($A54="SELECCION_MEJOR_RESPUESTA",$A54="SELECCION_SIMPLE",$A54="SELECCION_UNICA",$A54="SELECCION_DE_LA_MEJOR_RESPUESTA",$A54="SUBITEM_CASO",$A54="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H54))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H55">
-      <x:formula1>IF(ISNUMBER(MATCH($A55,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H55))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A55,TIPOS_OPCION_H,0)),OR($A55="SELECCION_MEJOR_RESPUESTA",$A55="SELECCION_SIMPLE",$A55="SELECCION_UNICA",$A55="SELECCION_DE_LA_MEJOR_RESPUESTA",$A55="SUBITEM_CASO",$A55="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H55))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H56">
-      <x:formula1>IF(ISNUMBER(MATCH($A56,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H56))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A56,TIPOS_OPCION_H,0)),OR($A56="SELECCION_MEJOR_RESPUESTA",$A56="SELECCION_SIMPLE",$A56="SELECCION_UNICA",$A56="SELECCION_DE_LA_MEJOR_RESPUESTA",$A56="SUBITEM_CASO",$A56="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H56))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H57">
-      <x:formula1>IF(ISNUMBER(MATCH($A57,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H57))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A57,TIPOS_OPCION_H,0)),OR($A57="SELECCION_MEJOR_RESPUESTA",$A57="SELECCION_SIMPLE",$A57="SELECCION_UNICA",$A57="SELECCION_DE_LA_MEJOR_RESPUESTA",$A57="SUBITEM_CASO",$A57="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H57))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H58">
-      <x:formula1>IF(ISNUMBER(MATCH($A58,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H58))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A58,TIPOS_OPCION_H,0)),OR($A58="SELECCION_MEJOR_RESPUESTA",$A58="SELECCION_SIMPLE",$A58="SELECCION_UNICA",$A58="SELECCION_DE_LA_MEJOR_RESPUESTA",$A58="SUBITEM_CASO",$A58="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H58))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H59">
-      <x:formula1>IF(ISNUMBER(MATCH($A59,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H59))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A59,TIPOS_OPCION_H,0)),OR($A59="SELECCION_MEJOR_RESPUESTA",$A59="SELECCION_SIMPLE",$A59="SELECCION_UNICA",$A59="SELECCION_DE_LA_MEJOR_RESPUESTA",$A59="SUBITEM_CASO",$A59="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H59))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H6">
-      <x:formula1>IF(ISNUMBER(MATCH($A6,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H6))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A6,TIPOS_OPCION_H,0)),OR($A6="SELECCION_MEJOR_RESPUESTA",$A6="SELECCION_SIMPLE",$A6="SELECCION_UNICA",$A6="SELECCION_DE_LA_MEJOR_RESPUESTA",$A6="SUBITEM_CASO",$A6="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H6))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H60">
-      <x:formula1>IF(ISNUMBER(MATCH($A60,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H60))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A60,TIPOS_OPCION_H,0)),OR($A60="SELECCION_MEJOR_RESPUESTA",$A60="SELECCION_SIMPLE",$A60="SELECCION_UNICA",$A60="SELECCION_DE_LA_MEJOR_RESPUESTA",$A60="SUBITEM_CASO",$A60="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H60))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H61">
-      <x:formula1>IF(ISNUMBER(MATCH($A61,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H61))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A61,TIPOS_OPCION_H,0)),OR($A61="SELECCION_MEJOR_RESPUESTA",$A61="SELECCION_SIMPLE",$A61="SELECCION_UNICA",$A61="SELECCION_DE_LA_MEJOR_RESPUESTA",$A61="SUBITEM_CASO",$A61="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H61))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H7">
-      <x:formula1>IF(ISNUMBER(MATCH($A7,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H7))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A7,TIPOS_OPCION_H,0)),OR($A7="SELECCION_MEJOR_RESPUESTA",$A7="SELECCION_SIMPLE",$A7="SELECCION_UNICA",$A7="SELECCION_DE_LA_MEJOR_RESPUESTA",$A7="SUBITEM_CASO",$A7="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H7))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H8">
-      <x:formula1>IF(ISNUMBER(MATCH($A8,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H8))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A8,TIPOS_OPCION_H,0)),OR($A8="SELECCION_MEJOR_RESPUESTA",$A8="SELECCION_SIMPLE",$A8="SELECCION_UNICA",$A8="SELECCION_DE_LA_MEJOR_RESPUESTA",$A8="SUBITEM_CASO",$A8="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H8))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Inciso no permitido" error="Ese inciso no corresponde al tipo seleccionado. Revise la columna L para ver que falta o sobra." promptTitle="Ayuda para incisos" prompt="Verdadero o Falso Simple: A=Verdadero y B=Falso automáticamente; deje C-E vacíos. Respuesta A/B/Ambas/Ninguna: A-D automáticamente; E vacío. Verdadero o Falso Complejas: premisas 1-4 en A-D; E vacío. Mejor respuesta/Subítem: complete A-E." sqref="H9">
-      <x:formula1>IF(ISNUMBER(MATCH($A9,TIPOS_OPCION_H,0)),TRUE,LEN(TRIM($H9))=0)</x:formula1>
+      <x:formula1>IF(OR(ISNUMBER(MATCH($A9,TIPOS_OPCION_H,0)),OR($A9="SELECCION_MEJOR_RESPUESTA",$A9="SELECCION_SIMPLE",$A9="SELECCION_UNICA",$A9="SELECCION_DE_LA_MEJOR_RESPUESTA",$A9="SUBITEM_CASO",$A9="SUBITEM_DE_CASO_O_PROBLEMA")),TRUE,LEN(TRIM($H9))=0)</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I10">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A10,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A10="SELECCION_MEJOR_RESPUESTA",$A10="SELECCION_SIMPLE",$A10="SELECCION_UNICA",$A10="SELECCION_DE_LA_MEJOR_RESPUESTA",$A10="SUBITEM_CASO",$A10="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A10,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I11">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A11,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A11="SELECCION_MEJOR_RESPUESTA",$A11="SELECCION_SIMPLE",$A11="SELECCION_UNICA",$A11="SELECCION_DE_LA_MEJOR_RESPUESTA",$A11="SUBITEM_CASO",$A11="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A11,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I12">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A12,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A12="SELECCION_MEJOR_RESPUESTA",$A12="SELECCION_SIMPLE",$A12="SELECCION_UNICA",$A12="SELECCION_DE_LA_MEJOR_RESPUESTA",$A12="SUBITEM_CASO",$A12="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A12,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I13">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A13,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A13="SELECCION_MEJOR_RESPUESTA",$A13="SELECCION_SIMPLE",$A13="SELECCION_UNICA",$A13="SELECCION_DE_LA_MEJOR_RESPUESTA",$A13="SUBITEM_CASO",$A13="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A13,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I14">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A14,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A14="SELECCION_MEJOR_RESPUESTA",$A14="SELECCION_SIMPLE",$A14="SELECCION_UNICA",$A14="SELECCION_DE_LA_MEJOR_RESPUESTA",$A14="SUBITEM_CASO",$A14="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A14,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I15">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A15,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A15="SELECCION_MEJOR_RESPUESTA",$A15="SELECCION_SIMPLE",$A15="SELECCION_UNICA",$A15="SELECCION_DE_LA_MEJOR_RESPUESTA",$A15="SUBITEM_CASO",$A15="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A15,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I16">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A16,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A16="SELECCION_MEJOR_RESPUESTA",$A16="SELECCION_SIMPLE",$A16="SELECCION_UNICA",$A16="SELECCION_DE_LA_MEJOR_RESPUESTA",$A16="SUBITEM_CASO",$A16="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A16,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I17">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A17,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A17="SELECCION_MEJOR_RESPUESTA",$A17="SELECCION_SIMPLE",$A17="SELECCION_UNICA",$A17="SELECCION_DE_LA_MEJOR_RESPUESTA",$A17="SUBITEM_CASO",$A17="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A17,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I18">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A18,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A18="SELECCION_MEJOR_RESPUESTA",$A18="SELECCION_SIMPLE",$A18="SELECCION_UNICA",$A18="SELECCION_DE_LA_MEJOR_RESPUESTA",$A18="SUBITEM_CASO",$A18="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A18,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I19">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A19,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A19="SELECCION_MEJOR_RESPUESTA",$A19="SELECCION_SIMPLE",$A19="SELECCION_UNICA",$A19="SELECCION_DE_LA_MEJOR_RESPUESTA",$A19="SUBITEM_CASO",$A19="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A19,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I2">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A2,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A2="SELECCION_MEJOR_RESPUESTA",$A2="SELECCION_SIMPLE",$A2="SELECCION_UNICA",$A2="SELECCION_DE_LA_MEJOR_RESPUESTA",$A2="SUBITEM_CASO",$A2="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A2,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I20">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A20,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A20="SELECCION_MEJOR_RESPUESTA",$A20="SELECCION_SIMPLE",$A20="SELECCION_UNICA",$A20="SELECCION_DE_LA_MEJOR_RESPUESTA",$A20="SUBITEM_CASO",$A20="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A20,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I21">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A21,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A21="SELECCION_MEJOR_RESPUESTA",$A21="SELECCION_SIMPLE",$A21="SELECCION_UNICA",$A21="SELECCION_DE_LA_MEJOR_RESPUESTA",$A21="SUBITEM_CASO",$A21="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A21,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I22">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A22,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A22="SELECCION_MEJOR_RESPUESTA",$A22="SELECCION_SIMPLE",$A22="SELECCION_UNICA",$A22="SELECCION_DE_LA_MEJOR_RESPUESTA",$A22="SUBITEM_CASO",$A22="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A22,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I23">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A23,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A23="SELECCION_MEJOR_RESPUESTA",$A23="SELECCION_SIMPLE",$A23="SELECCION_UNICA",$A23="SELECCION_DE_LA_MEJOR_RESPUESTA",$A23="SUBITEM_CASO",$A23="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A23,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I24">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A24,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A24="SELECCION_MEJOR_RESPUESTA",$A24="SELECCION_SIMPLE",$A24="SELECCION_UNICA",$A24="SELECCION_DE_LA_MEJOR_RESPUESTA",$A24="SUBITEM_CASO",$A24="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A24,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I25">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A25,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A25="SELECCION_MEJOR_RESPUESTA",$A25="SELECCION_SIMPLE",$A25="SELECCION_UNICA",$A25="SELECCION_DE_LA_MEJOR_RESPUESTA",$A25="SUBITEM_CASO",$A25="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A25,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I26">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A26,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A26="SELECCION_MEJOR_RESPUESTA",$A26="SELECCION_SIMPLE",$A26="SELECCION_UNICA",$A26="SELECCION_DE_LA_MEJOR_RESPUESTA",$A26="SUBITEM_CASO",$A26="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A26,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I27">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A27,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A27="SELECCION_MEJOR_RESPUESTA",$A27="SELECCION_SIMPLE",$A27="SELECCION_UNICA",$A27="SELECCION_DE_LA_MEJOR_RESPUESTA",$A27="SUBITEM_CASO",$A27="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A27,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I28">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A28,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A28="SELECCION_MEJOR_RESPUESTA",$A28="SELECCION_SIMPLE",$A28="SELECCION_UNICA",$A28="SELECCION_DE_LA_MEJOR_RESPUESTA",$A28="SUBITEM_CASO",$A28="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A28,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I29">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A29,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A29="SELECCION_MEJOR_RESPUESTA",$A29="SELECCION_SIMPLE",$A29="SELECCION_UNICA",$A29="SELECCION_DE_LA_MEJOR_RESPUESTA",$A29="SUBITEM_CASO",$A29="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A29,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I3">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A3,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A3="SELECCION_MEJOR_RESPUESTA",$A3="SELECCION_SIMPLE",$A3="SELECCION_UNICA",$A3="SELECCION_DE_LA_MEJOR_RESPUESTA",$A3="SUBITEM_CASO",$A3="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A3,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I30">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A30,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A30="SELECCION_MEJOR_RESPUESTA",$A30="SELECCION_SIMPLE",$A30="SELECCION_UNICA",$A30="SELECCION_DE_LA_MEJOR_RESPUESTA",$A30="SUBITEM_CASO",$A30="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A30,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I31">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A31,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A31="SELECCION_MEJOR_RESPUESTA",$A31="SELECCION_SIMPLE",$A31="SELECCION_UNICA",$A31="SELECCION_DE_LA_MEJOR_RESPUESTA",$A31="SUBITEM_CASO",$A31="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A31,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I32">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A32,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A32="SELECCION_MEJOR_RESPUESTA",$A32="SELECCION_SIMPLE",$A32="SELECCION_UNICA",$A32="SELECCION_DE_LA_MEJOR_RESPUESTA",$A32="SUBITEM_CASO",$A32="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A32,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I33">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A33,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A33="SELECCION_MEJOR_RESPUESTA",$A33="SELECCION_SIMPLE",$A33="SELECCION_UNICA",$A33="SELECCION_DE_LA_MEJOR_RESPUESTA",$A33="SUBITEM_CASO",$A33="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A33,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I34">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A34,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A34="SELECCION_MEJOR_RESPUESTA",$A34="SELECCION_SIMPLE",$A34="SELECCION_UNICA",$A34="SELECCION_DE_LA_MEJOR_RESPUESTA",$A34="SUBITEM_CASO",$A34="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A34,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I35">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A35,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A35="SELECCION_MEJOR_RESPUESTA",$A35="SELECCION_SIMPLE",$A35="SELECCION_UNICA",$A35="SELECCION_DE_LA_MEJOR_RESPUESTA",$A35="SUBITEM_CASO",$A35="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A35,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I36">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A36,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A36="SELECCION_MEJOR_RESPUESTA",$A36="SELECCION_SIMPLE",$A36="SELECCION_UNICA",$A36="SELECCION_DE_LA_MEJOR_RESPUESTA",$A36="SUBITEM_CASO",$A36="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A36,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I37">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A37,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A37="SELECCION_MEJOR_RESPUESTA",$A37="SELECCION_SIMPLE",$A37="SELECCION_UNICA",$A37="SELECCION_DE_LA_MEJOR_RESPUESTA",$A37="SUBITEM_CASO",$A37="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A37,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I38">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A38,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A38="SELECCION_MEJOR_RESPUESTA",$A38="SELECCION_SIMPLE",$A38="SELECCION_UNICA",$A38="SELECCION_DE_LA_MEJOR_RESPUESTA",$A38="SUBITEM_CASO",$A38="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A38,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I39">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A39,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A39="SELECCION_MEJOR_RESPUESTA",$A39="SELECCION_SIMPLE",$A39="SELECCION_UNICA",$A39="SELECCION_DE_LA_MEJOR_RESPUESTA",$A39="SUBITEM_CASO",$A39="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A39,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I4">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A4,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A4="SELECCION_MEJOR_RESPUESTA",$A4="SELECCION_SIMPLE",$A4="SELECCION_UNICA",$A4="SELECCION_DE_LA_MEJOR_RESPUESTA",$A4="SUBITEM_CASO",$A4="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A4,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I40">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A40,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A40="SELECCION_MEJOR_RESPUESTA",$A40="SELECCION_SIMPLE",$A40="SELECCION_UNICA",$A40="SELECCION_DE_LA_MEJOR_RESPUESTA",$A40="SUBITEM_CASO",$A40="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A40,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I41">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A41,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A41="SELECCION_MEJOR_RESPUESTA",$A41="SELECCION_SIMPLE",$A41="SELECCION_UNICA",$A41="SELECCION_DE_LA_MEJOR_RESPUESTA",$A41="SUBITEM_CASO",$A41="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A41,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I42">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A42,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A42="SELECCION_MEJOR_RESPUESTA",$A42="SELECCION_SIMPLE",$A42="SELECCION_UNICA",$A42="SELECCION_DE_LA_MEJOR_RESPUESTA",$A42="SUBITEM_CASO",$A42="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A42,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I43">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A43,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A43="SELECCION_MEJOR_RESPUESTA",$A43="SELECCION_SIMPLE",$A43="SELECCION_UNICA",$A43="SELECCION_DE_LA_MEJOR_RESPUESTA",$A43="SUBITEM_CASO",$A43="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A43,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I44">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A44,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A44="SELECCION_MEJOR_RESPUESTA",$A44="SELECCION_SIMPLE",$A44="SELECCION_UNICA",$A44="SELECCION_DE_LA_MEJOR_RESPUESTA",$A44="SUBITEM_CASO",$A44="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A44,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I45">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A45,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A45="SELECCION_MEJOR_RESPUESTA",$A45="SELECCION_SIMPLE",$A45="SELECCION_UNICA",$A45="SELECCION_DE_LA_MEJOR_RESPUESTA",$A45="SUBITEM_CASO",$A45="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A45,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I46">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A46,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A46="SELECCION_MEJOR_RESPUESTA",$A46="SELECCION_SIMPLE",$A46="SELECCION_UNICA",$A46="SELECCION_DE_LA_MEJOR_RESPUESTA",$A46="SUBITEM_CASO",$A46="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A46,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I47">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A47,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A47="SELECCION_MEJOR_RESPUESTA",$A47="SELECCION_SIMPLE",$A47="SELECCION_UNICA",$A47="SELECCION_DE_LA_MEJOR_RESPUESTA",$A47="SUBITEM_CASO",$A47="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A47,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I48">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A48,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A48="SELECCION_MEJOR_RESPUESTA",$A48="SELECCION_SIMPLE",$A48="SELECCION_UNICA",$A48="SELECCION_DE_LA_MEJOR_RESPUESTA",$A48="SUBITEM_CASO",$A48="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A48,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I49">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A49,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A49="SELECCION_MEJOR_RESPUESTA",$A49="SELECCION_SIMPLE",$A49="SELECCION_UNICA",$A49="SELECCION_DE_LA_MEJOR_RESPUESTA",$A49="SUBITEM_CASO",$A49="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A49,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I5">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A5,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A5="SELECCION_MEJOR_RESPUESTA",$A5="SELECCION_SIMPLE",$A5="SELECCION_UNICA",$A5="SELECCION_DE_LA_MEJOR_RESPUESTA",$A5="SUBITEM_CASO",$A5="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A5,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I50">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A50,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A50="SELECCION_MEJOR_RESPUESTA",$A50="SELECCION_SIMPLE",$A50="SELECCION_UNICA",$A50="SELECCION_DE_LA_MEJOR_RESPUESTA",$A50="SUBITEM_CASO",$A50="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A50,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I51">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A51,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A51="SELECCION_MEJOR_RESPUESTA",$A51="SELECCION_SIMPLE",$A51="SELECCION_UNICA",$A51="SELECCION_DE_LA_MEJOR_RESPUESTA",$A51="SUBITEM_CASO",$A51="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A51,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I52">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A52,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A52="SELECCION_MEJOR_RESPUESTA",$A52="SELECCION_SIMPLE",$A52="SELECCION_UNICA",$A52="SELECCION_DE_LA_MEJOR_RESPUESTA",$A52="SUBITEM_CASO",$A52="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A52,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I53">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A53,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A53="SELECCION_MEJOR_RESPUESTA",$A53="SELECCION_SIMPLE",$A53="SELECCION_UNICA",$A53="SELECCION_DE_LA_MEJOR_RESPUESTA",$A53="SUBITEM_CASO",$A53="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A53,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I54">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A54,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A54="SELECCION_MEJOR_RESPUESTA",$A54="SELECCION_SIMPLE",$A54="SELECCION_UNICA",$A54="SELECCION_DE_LA_MEJOR_RESPUESTA",$A54="SUBITEM_CASO",$A54="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A54,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I55">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A55,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A55="SELECCION_MEJOR_RESPUESTA",$A55="SELECCION_SIMPLE",$A55="SELECCION_UNICA",$A55="SELECCION_DE_LA_MEJOR_RESPUESTA",$A55="SUBITEM_CASO",$A55="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A55,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I56">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A56,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A56="SELECCION_MEJOR_RESPUESTA",$A56="SELECCION_SIMPLE",$A56="SELECCION_UNICA",$A56="SELECCION_DE_LA_MEJOR_RESPUESTA",$A56="SUBITEM_CASO",$A56="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A56,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I57">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A57,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A57="SELECCION_MEJOR_RESPUESTA",$A57="SELECCION_SIMPLE",$A57="SELECCION_UNICA",$A57="SELECCION_DE_LA_MEJOR_RESPUESTA",$A57="SUBITEM_CASO",$A57="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A57,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I58">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A58,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A58="SELECCION_MEJOR_RESPUESTA",$A58="SELECCION_SIMPLE",$A58="SELECCION_UNICA",$A58="SELECCION_DE_LA_MEJOR_RESPUESTA",$A58="SUBITEM_CASO",$A58="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A58,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I59">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A59,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A59="SELECCION_MEJOR_RESPUESTA",$A59="SELECCION_SIMPLE",$A59="SELECCION_UNICA",$A59="SELECCION_DE_LA_MEJOR_RESPUESTA",$A59="SUBITEM_CASO",$A59="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A59,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I6">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A6,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A6="SELECCION_MEJOR_RESPUESTA",$A6="SELECCION_SIMPLE",$A6="SELECCION_UNICA",$A6="SELECCION_DE_LA_MEJOR_RESPUESTA",$A6="SUBITEM_CASO",$A6="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A6,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I60">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A60,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A60="SELECCION_MEJOR_RESPUESTA",$A60="SELECCION_SIMPLE",$A60="SELECCION_UNICA",$A60="SELECCION_DE_LA_MEJOR_RESPUESTA",$A60="SUBITEM_CASO",$A60="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A60,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I61">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A61,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A61="SELECCION_MEJOR_RESPUESTA",$A61="SELECCION_SIMPLE",$A61="SELECCION_UNICA",$A61="SELECCION_DE_LA_MEJOR_RESPUESTA",$A61="SUBITEM_CASO",$A61="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A61,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I7">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A7,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A7="SELECCION_MEJOR_RESPUESTA",$A7="SELECCION_SIMPLE",$A7="SELECCION_UNICA",$A7="SELECCION_DE_LA_MEJOR_RESPUESTA",$A7="SUBITEM_CASO",$A7="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A7,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I8">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A8,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A8="SELECCION_MEJOR_RESPUESTA",$A8="SELECCION_SIMPLE",$A8="SELECCION_UNICA",$A8="SELECCION_DE_LA_MEJOR_RESPUESTA",$A8="SUBITEM_CASO",$A8="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A8,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Respuesta invalida" error="Seleccione una respuesta valida segun el tipo de pregunta." promptTitle="Ayuda para respuesta" prompt="Verdadero/Falso Simple inicia en A y puede cambiarse a B. Respuesta A/B/Ambas/Ninguna usa A-D. Verdadero/Falso Complejas usa combinaciones A-E." sqref="I9">
-      <x:formula1>INDIRECT(IFERROR(VLOOKUP($A9,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA"))</x:formula1>
+      <x:formula1>INDIRECT(IF(OR($A9="SELECCION_MEJOR_RESPUESTA",$A9="SELECCION_SIMPLE",$A9="SELECCION_UNICA",$A9="SELECCION_DE_LA_MEJOR_RESPUESTA",$A9="SUBITEM_CASO",$A9="SUBITEM_DE_CASO_O_PROBLEMA"),"RESP_ABCDE",IFERROR(VLOOKUP($A9,MAPA_RESPUESTA_TIPO,2,FALSE),"RESP_VACIA")))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dificultad invalida" error="Use 1, 2 o 3. Casos/problemas y Emparejamiento Ampliado no llevan dificultad." sqref="J10">
       <x:formula1>INDIRECT(IF(ISNUMBER(MATCH($A10,TIPOS_SIN_DIFICULTAD,0)),"RESP_VACIA","DIFICULTADES_123"))</x:formula1>

</xml_diff>